<commit_message>
scan: seg4 2026-09-25 18:04 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq5_2026-09-24.xlsx
+++ b/output/full_scan/batch_seq5_2026-09-24.xlsx
@@ -633,21 +633,21 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>6155</v>
+        <v>4566</v>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>鈞寶</t>
+          <t>時碩工業</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
         <v/>
       </c>
       <c r="D4" s="2" t="n">
-        <v>1058.658718814237</v>
+        <v>1064.166860120251</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>60.2</v>
+        <v>74.3</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
@@ -658,16 +658,16 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>58.14715927732101</v>
+        <v>68.81035902333016</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>7.428292181474113</v>
+        <v>12.73687841764105</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>2.984149960768015</v>
+        <v>6.479544065060112</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="L4" s="2" t="n">
         <v>0</v>
@@ -676,31 +676,31 @@
         <v>-1</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>0.419576754741398</v>
+        <v>0.9960066264025988</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, foreign_buy_3d, stronger_than_market, obv_uptrend, bb_squeeze_breakout, breakout_volume_confirm, cci_momentum, mfi_strong</t>
+          <t>ema60_gt_ema120, volume_break, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, stronger_than_market, obv_uptrend, bb_squeeze_breakout, breakout_volume_confirm, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>4566</v>
+        <v>6155</v>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>時碩工業</t>
+          <t>鈞寶</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
         <v/>
       </c>
       <c r="D5" s="2" t="n">
-        <v>1054.166860120251</v>
+        <v>1058.658718814237</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>74.3</v>
+        <v>60.2</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
@@ -711,16 +711,16 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>68.81035900292167</v>
+        <v>58.14715927732101</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>12.73687831036259</v>
+        <v>7.428292181474113</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>6.479544065060112</v>
+        <v>2.984149960768015</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="L5" s="2" t="n">
         <v>0</v>
@@ -729,11 +729,11 @@
         <v>-1</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>0.996006626288126</v>
+        <v>0.419576754741398</v>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, stronger_than_market, obv_uptrend, bb_squeeze_breakout, breakout_volume_confirm, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, volume_break, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, foreign_buy_3d, stronger_than_market, obv_uptrend, bb_squeeze_breakout, breakout_volume_confirm, cci_momentum, mfi_strong</t>
         </is>
       </c>
     </row>
@@ -803,7 +803,7 @@
         <v/>
       </c>
       <c r="D7" s="2" t="n">
-        <v>942.2605833459944</v>
+        <v>932.2605833459944</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>281.5</v>
@@ -817,10 +817,10 @@
         <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>71.77572342854027</v>
+        <v>71.77572352993795</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>32.04757408572473</v>
+        <v>32.04757420387939</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>3.826058334599439</v>
@@ -835,7 +835,7 @@
         <v>-1</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>5.013370794842064</v>
+        <v>5.013370794555861</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
@@ -1241,10 +1241,10 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>62.25575134080445</v>
+        <v>62.25575136218347</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>39.6474758653071</v>
+        <v>39.64747602894467</v>
       </c>
       <c r="J15" s="2" t="n">
         <v>0.3437488000058795</v>
@@ -1259,7 +1259,7 @@
         <v>-1</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>-0.0103754106440931</v>
+        <v>-0.0103754105487001</v>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
@@ -1492,7 +1492,7 @@
         <v/>
       </c>
       <c r="D20" s="2" t="n">
-        <v>762.9578359188234</v>
+        <v>762.9578359188235</v>
       </c>
       <c r="E20" s="2" t="n">
         <v>14.4</v>
@@ -1506,10 +1506,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>57.90946900948806</v>
+        <v>57.90946925768867</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>20.85976559794153</v>
+        <v>20.85976556234633</v>
       </c>
       <c r="J20" s="2" t="n">
         <v>2.618020138616451</v>
@@ -1524,7 +1524,7 @@
         <v>-1</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>0.0806836187779366</v>
+        <v>0.0806836185966833</v>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
@@ -1559,10 +1559,10 @@
         <v>0</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>61.02119068710096</v>
+        <v>61.02121080777088</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>29.84669893400205</v>
+        <v>29.84671089453922</v>
       </c>
       <c r="J21" s="2" t="n">
         <v>1.767059278639126</v>
@@ -1577,7 +1577,7 @@
         <v>-1</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>0.0113587208842763</v>
+        <v>0.0113587181559157</v>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
@@ -1905,21 +1905,21 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>6103</v>
+        <v>4540</v>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>合邦</t>
+          <t>全球傳動</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
         <v/>
       </c>
       <c r="D28" s="2" t="n">
-        <v>692.7834381227536</v>
+        <v>696.6508388854625</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>40.9</v>
+        <v>60</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
@@ -1930,16 +1930,16 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>57.1990037271645</v>
+        <v>54.6924297492144</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>7.55405858681615</v>
+        <v>29.11161250777786</v>
       </c>
       <c r="J28" s="2" t="n">
-        <v>1.175352918501701</v>
+        <v>0.5849274908302399</v>
       </c>
       <c r="K28" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L28" s="2" t="n">
         <v>0</v>
@@ -1948,31 +1948,31 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>0.0029533313620175</v>
+        <v>0.0568726371169409</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, ema60_gt_ema120, rsi_strong, market_above_ma60, hist_turn_positive, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>4540</v>
+        <v>6103</v>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>全球傳動</t>
+          <t>合邦</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
         <v/>
       </c>
       <c r="D29" s="2" t="n">
-        <v>686.6508388854614</v>
+        <v>692.7834381227536</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>60</v>
+        <v>40.9</v>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
@@ -1983,16 +1983,16 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>54.69242968452861</v>
+        <v>57.1990037271645</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>29.11161249563925</v>
+        <v>7.55405858681615</v>
       </c>
       <c r="J29" s="2" t="n">
-        <v>0.5849274908302399</v>
+        <v>1.175352918501701</v>
       </c>
       <c r="K29" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L29" s="2" t="n">
         <v>0</v>
@@ -2001,11 +2001,11 @@
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>0.0568726370787768</v>
+        <v>0.0029533313620175</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>macd_golden_cross, ema60_gt_ema120, rsi_strong, market_above_ma60, hist_turn_positive, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
@@ -2036,10 +2036,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>59.90121714769082</v>
+        <v>59.90121715096843</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>28.88167591183663</v>
+        <v>28.881675981026</v>
       </c>
       <c r="J30" s="2" t="n">
         <v>0.3278584951746066</v>
@@ -2054,7 +2054,7 @@
         <v>-1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>1.871470356998774</v>
+        <v>1.871470356788881</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
@@ -2128,7 +2128,7 @@
         <v/>
       </c>
       <c r="D32" s="2" t="n">
-        <v>674.8580813633281</v>
+        <v>674.858081363328</v>
       </c>
       <c r="E32" s="2" t="n">
         <v>225</v>
@@ -2142,10 +2142,10 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>48.71103066435803</v>
+        <v>48.71103069234053</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>20.00882342701923</v>
+        <v>20.00882355644496</v>
       </c>
       <c r="J32" s="2" t="n">
         <v>0.2560333412723786</v>
@@ -2160,7 +2160,7 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>-2.033759712295138</v>
+        <v>-2.033759712485915</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
@@ -2248,10 +2248,10 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>62.16432835173389</v>
+        <v>62.16432837317918</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>19.62741969606255</v>
+        <v>19.62741977985568</v>
       </c>
       <c r="J34" s="2" t="n">
         <v>1.541918131860579</v>
@@ -2266,7 +2266,7 @@
         <v>-1</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>-0.1145444813878525</v>
+        <v>-0.1145444814164639</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
@@ -2301,10 +2301,10 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>55.6040028923061</v>
+        <v>55.60400285124288</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>36.55019268287617</v>
+        <v>36.55019272855143</v>
       </c>
       <c r="J35" s="2" t="n">
         <v>0.5484099608061106</v>
@@ -2319,7 +2319,7 @@
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>-0.0782787853934082</v>
+        <v>-0.0782787853457111</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
@@ -2675,7 +2675,7 @@
         <v>49.46790685615793</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>41.51741407892816</v>
+        <v>41.51741410640639</v>
       </c>
       <c r="J42" s="2" t="n">
         <v>0.6974006104383712</v>
@@ -2690,7 +2690,7 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>-0.0777381053338731</v>
+        <v>-0.0777381052861708</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
@@ -2764,7 +2764,7 @@
         <v/>
       </c>
       <c r="D44" s="2" t="n">
-        <v>608.2299759138505</v>
+        <v>598.2299759138505</v>
       </c>
       <c r="E44" s="2" t="n">
         <v>212</v>
@@ -2778,10 +2778,10 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>53.29595624624857</v>
+        <v>53.29595625236897</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>20.28415107913301</v>
+        <v>20.28415106042165</v>
       </c>
       <c r="J44" s="2" t="n">
         <v>0.5381882763402255</v>
@@ -2796,7 +2796,7 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>0.3206892976158375</v>
+        <v>0.3206892979974283</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
@@ -3414,10 +3414,10 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>52.09329601180442</v>
+        <v>52.09329616100742</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>31.35329497743185</v>
+        <v>31.353295028226</v>
       </c>
       <c r="J56" s="2" t="n">
         <v>0.6987920384932089</v>
@@ -3432,7 +3432,7 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>-0.1160734884603043</v>
+        <v>-0.1160734882695108</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
@@ -3453,7 +3453,7 @@
         <v/>
       </c>
       <c r="D57" s="2" t="n">
-        <v>549.2786236044437</v>
+        <v>549.2786236044436</v>
       </c>
       <c r="E57" s="2" t="n">
         <v>343.5</v>
@@ -3467,10 +3467,10 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>53.31637276731875</v>
+        <v>53.31637305601383</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>10.85050408868309</v>
+        <v>10.85050409600881</v>
       </c>
       <c r="J57" s="2" t="n">
         <v>0.5676270190493309</v>
@@ -3485,7 +3485,7 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>0.0610160829795531</v>
+        <v>0.0610160808808112</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
@@ -3785,10 +3785,10 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>45.69705807396912</v>
+        <v>45.69705808265042</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>22.00689911622043</v>
+        <v>22.0068992142726</v>
       </c>
       <c r="J63" s="2" t="n">
         <v>1.611857819242779</v>
@@ -3944,10 +3944,10 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>46.26723564015835</v>
+        <v>46.26723549184492</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>17.36164442663256</v>
+        <v>17.36164429409034</v>
       </c>
       <c r="J66" s="2" t="n">
         <v>0.4550434989940676</v>
@@ -3962,7 +3962,7 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>-0.297410754677931</v>
+        <v>-0.2974107543535805</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
@@ -4103,10 +4103,10 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>64.03915314952977</v>
+        <v>64.0391531291524</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>24.56988941208595</v>
+        <v>24.56988951403187</v>
       </c>
       <c r="J69" s="2" t="n">
         <v>0.8539018775809273</v>
@@ -4121,7 +4121,7 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>0.1909805178043387</v>
+        <v>0.190980517832958</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
@@ -4262,10 +4262,10 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>51.15748831284139</v>
+        <v>51.15748839583868</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>22.47658358285572</v>
+        <v>22.47658364165237</v>
       </c>
       <c r="J72" s="2" t="n">
         <v>0.322345670775057</v>
@@ -4280,7 +4280,7 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>-0.0294860577838009</v>
+        <v>-0.0294860576120866</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
@@ -4424,7 +4424,7 @@
         <v>58.47076365709396</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>20.80775747349735</v>
+        <v>20.80775742474945</v>
       </c>
       <c r="J75" s="2" t="n">
         <v>0.5340344449746914</v>
@@ -4439,7 +4439,7 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>0.0488235968588787</v>
+        <v>0.0488235968493397</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
         <v/>
       </c>
       <c r="D76" s="2" t="n">
-        <v>484.4073872998481</v>
+        <v>484.4073872998474</v>
       </c>
       <c r="E76" s="2" t="n">
         <v>184</v>
@@ -4474,10 +4474,10 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>39.3906643099175</v>
+        <v>39.39066430309327</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>22.16140032153923</v>
+        <v>22.16140032556028</v>
       </c>
       <c r="J76" s="2" t="n">
         <v>0.9857091137268152</v>
@@ -4492,7 +4492,7 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>0.3570944327838052</v>
+        <v>0.3570944329173606</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
@@ -4527,10 +4527,10 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>33.58239304245032</v>
+        <v>33.58239287847695</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>20.69928983808294</v>
+        <v>20.69928986808966</v>
       </c>
       <c r="J77" s="2" t="n">
         <v>1.163180969647383</v>
@@ -4545,7 +4545,7 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>-1.917727767520038</v>
+        <v>-1.917727767653598</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
@@ -4725,7 +4725,7 @@
         <v/>
       </c>
       <c r="D81" s="2" t="n">
-        <v>471.5894972849058</v>
+        <v>471.5894972849057</v>
       </c>
       <c r="E81" s="2" t="n">
         <v>29.2</v>
@@ -4739,10 +4739,10 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>56.38742633999403</v>
+        <v>56.38742636564721</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>16.66945260710866</v>
+        <v>16.66945247917815</v>
       </c>
       <c r="J81" s="2" t="n">
         <v>0.5628232816407717</v>
@@ -4757,7 +4757,7 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>0.0558172350368333</v>
+        <v>0.0558172353993436</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
@@ -4792,10 +4792,10 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>55.74857810466795</v>
+        <v>55.74857831255809</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>27.2709960500854</v>
+        <v>27.27099603144418</v>
       </c>
       <c r="J82" s="2" t="n">
         <v>0.5205154316030123</v>
@@ -4810,7 +4810,7 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>0.2567259754041781</v>
+        <v>0.2567259754232558</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
@@ -4831,7 +4831,7 @@
         <v/>
       </c>
       <c r="D83" s="2" t="n">
-        <v>466.1704379378579</v>
+        <v>466.1704379378578</v>
       </c>
       <c r="E83" s="2" t="n">
         <v>165</v>
@@ -4845,10 +4845,10 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>49.10782022618816</v>
+        <v>49.10782016714725</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>19.27507842769169</v>
+        <v>19.27507845469787</v>
       </c>
       <c r="J83" s="2" t="n">
         <v>0.9312472217317814</v>
@@ -4863,7 +4863,7 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>0.3093416663630343</v>
+        <v>0.3093416667446095</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
@@ -4898,10 +4898,10 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>48.43153022983781</v>
+        <v>48.43153034516915</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>11.14616932187823</v>
+        <v>11.14616932445286</v>
       </c>
       <c r="J84" s="2" t="n">
         <v>0.1621140391137049</v>
@@ -4916,7 +4916,7 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>0.0043350087426979</v>
+        <v>0.004335008761779</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
@@ -4990,7 +4990,7 @@
         <v/>
       </c>
       <c r="D86" s="2" t="n">
-        <v>456.4896247062653</v>
+        <v>456.4896247062656</v>
       </c>
       <c r="E86" s="2" t="n">
         <v>31.75</v>
@@ -5004,10 +5004,10 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>53.49049847156886</v>
+        <v>53.49049835994364</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>17.71646480109167</v>
+        <v>17.71646470836197</v>
       </c>
       <c r="J86" s="2" t="n">
         <v>0.2831828438973704</v>
@@ -5022,7 +5022,7 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>0.1230489109030537</v>
+        <v>0.1230489110270717</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
@@ -5163,10 +5163,10 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>46.25650472737123</v>
+        <v>46.25650474090093</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>24.21747477973344</v>
+        <v>24.21747499731798</v>
       </c>
       <c r="J89" s="2" t="n">
         <v>0.3851726453046433</v>
@@ -5181,7 +5181,7 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>0.3293088506749222</v>
+        <v>0.3293088506272185</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
@@ -5520,7 +5520,7 @@
         <v/>
       </c>
       <c r="D96" s="2" t="n">
-        <v>434.9205764127132</v>
+        <v>434.9205764127134</v>
       </c>
       <c r="E96" s="2" t="n">
         <v>32</v>
@@ -5537,7 +5537,7 @@
         <v>50.13890692747822</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>13.72758223785097</v>
+        <v>13.72758210319665</v>
       </c>
       <c r="J96" s="2" t="n">
         <v>0.9215231654956528</v>
@@ -5552,7 +5552,7 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>0.1341400419917552</v>
+        <v>0.1341400420394524</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
@@ -5587,10 +5587,10 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>36.96293587133512</v>
+        <v>36.96293594032589</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>12.69260822785411</v>
+        <v>12.69260824695648</v>
       </c>
       <c r="J97" s="2" t="n">
         <v>0.688833328680561</v>
@@ -5605,7 +5605,7 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>-0.5553395641912624</v>
+        <v>-0.5553395643820627</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
@@ -5905,10 +5905,10 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>49.94527219749282</v>
+        <v>49.94527225999974</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>10.94208471651164</v>
+        <v>10.94208471153626</v>
       </c>
       <c r="J103" s="2" t="n">
         <v>0.941309601978234</v>
@@ -6382,10 +6382,10 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>52.32291636862959</v>
+        <v>52.32291639244881</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>24.27558900119032</v>
+        <v>24.27558905999737</v>
       </c>
       <c r="J112" s="2" t="n">
         <v>0.343876719416974</v>
@@ -6516,21 +6516,21 @@
     </row>
     <row r="115">
       <c r="A115" s="2" t="n">
-        <v>4736</v>
+        <v>4977</v>
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>泰博</t>
+          <t>眾達-KY</t>
         </is>
       </c>
       <c r="C115" s="2" t="n">
         <v/>
       </c>
       <c r="D115" s="2" t="n">
-        <v>379.6217727484305</v>
+        <v>377.4037210051063</v>
       </c>
       <c r="E115" s="2" t="n">
-        <v>129.5</v>
+        <v>168.5</v>
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
@@ -6541,13 +6541,13 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>47.23850738202734</v>
+        <v>51.07901750427845</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>18.72845511702576</v>
+        <v>20.27325832830773</v>
       </c>
       <c r="J115" s="2" t="n">
-        <v>0.6903758132354407</v>
+        <v>0.2509217443451846</v>
       </c>
       <c r="K115" s="2" t="n">
         <v>0</v>
@@ -6559,31 +6559,31 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>0.4435926936248615</v>
+        <v>-1.551407385573853</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="n">
-        <v>4977</v>
+        <v>5471</v>
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>眾達-KY</t>
+          <t>松翰</t>
         </is>
       </c>
       <c r="C116" s="2" t="n">
         <v/>
       </c>
       <c r="D116" s="2" t="n">
-        <v>377.4037210051063</v>
+        <v>377.2937479712092</v>
       </c>
       <c r="E116" s="2" t="n">
-        <v>168.5</v>
+        <v>51.7</v>
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
@@ -6594,16 +6594,16 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>51.07901750427845</v>
+        <v>38.82622993258804</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>20.27325832830773</v>
+        <v>19.87951539967662</v>
       </c>
       <c r="J116" s="2" t="n">
-        <v>0.2509217443451846</v>
+        <v>0.4480145761155067</v>
       </c>
       <c r="K116" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L116" s="2" t="n">
         <v>0</v>
@@ -6612,51 +6612,51 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>-1.551407385573853</v>
+        <v>-0.2831956551838774</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="n">
-        <v>5471</v>
+        <v>5371</v>
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>松翰</t>
+          <t>中光電</t>
         </is>
       </c>
       <c r="C117" s="2" t="n">
         <v/>
       </c>
       <c r="D117" s="2" t="n">
-        <v>377.2937479712092</v>
+        <v>376.878000930349</v>
       </c>
       <c r="E117" s="2" t="n">
-        <v>51.7</v>
+        <v>83.5</v>
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="G117" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>38.82622993258804</v>
+        <v>49.059970829028</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>19.87951539967662</v>
+        <v>19.84838971988606</v>
       </c>
       <c r="J117" s="2" t="n">
-        <v>0.4480145761155067</v>
+        <v>0.1790799411206339</v>
       </c>
       <c r="K117" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L117" s="2" t="n">
         <v>0</v>
@@ -6665,48 +6665,48 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>-0.2831956551838774</v>
+        <v>-0.1002586669852813</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="n">
-        <v>5371</v>
+        <v>4976</v>
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>中光電</t>
+          <t>佳凌</t>
         </is>
       </c>
       <c r="C118" s="2" t="n">
         <v/>
       </c>
       <c r="D118" s="2" t="n">
-        <v>376.878000930349</v>
+        <v>374.5695599834368</v>
       </c>
       <c r="E118" s="2" t="n">
-        <v>83.5</v>
+        <v>35.2</v>
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G118" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H118" s="2" t="n">
-        <v>49.059970829028</v>
+        <v>43.5024843199455</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>19.84838971988606</v>
+        <v>27.7417370232545</v>
       </c>
       <c r="J118" s="2" t="n">
-        <v>0.1790799411206339</v>
+        <v>0.200119664830243</v>
       </c>
       <c r="K118" s="2" t="n">
         <v>0</v>
@@ -6718,31 +6718,31 @@
         <v>-1</v>
       </c>
       <c r="N118" s="2" t="n">
-        <v>-0.1002586669852813</v>
+        <v>-0.2091529011495917</v>
       </c>
       <c r="O118" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="n">
-        <v>4976</v>
+        <v>5450</v>
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>佳凌</t>
+          <t>寶聯通</t>
         </is>
       </c>
       <c r="C119" s="2" t="n">
         <v/>
       </c>
       <c r="D119" s="2" t="n">
-        <v>374.5695599834368</v>
+        <v>374.2417141332528</v>
       </c>
       <c r="E119" s="2" t="n">
-        <v>35.2</v>
+        <v>14.85</v>
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
@@ -6753,16 +6753,16 @@
         <v>0</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>43.5024843199455</v>
+        <v>52.69302409881968</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>27.7417370232545</v>
+        <v>14.35700262227653</v>
       </c>
       <c r="J119" s="2" t="n">
-        <v>0.200119664830243</v>
+        <v>0.6713134887657505</v>
       </c>
       <c r="K119" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L119" s="2" t="n">
         <v>0</v>
@@ -6771,31 +6771,31 @@
         <v>-1</v>
       </c>
       <c r="N119" s="2" t="n">
-        <v>-0.2091529011495917</v>
+        <v>0.0394930893110192</v>
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, kd_golden_cross, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="n">
-        <v>5450</v>
+        <v>5328</v>
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>寶聯通</t>
+          <t>華容</t>
         </is>
       </c>
       <c r="C120" s="2" t="n">
         <v/>
       </c>
       <c r="D120" s="2" t="n">
-        <v>374.2417141332528</v>
+        <v>373.7479175246148</v>
       </c>
       <c r="E120" s="2" t="n">
-        <v>14.85</v>
+        <v>52.5</v>
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
@@ -6806,16 +6806,16 @@
         <v>0</v>
       </c>
       <c r="H120" s="2" t="n">
-        <v>52.69302409881968</v>
+        <v>35.48908699208265</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>14.35700262227653</v>
+        <v>17.16284906316569</v>
       </c>
       <c r="J120" s="2" t="n">
-        <v>0.6713134887657505</v>
+        <v>0.6216553896099903</v>
       </c>
       <c r="K120" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L120" s="2" t="n">
         <v>0</v>
@@ -6824,31 +6824,31 @@
         <v>-1</v>
       </c>
       <c r="N120" s="2" t="n">
-        <v>0.0394930893110192</v>
+        <v>-0.325325642679676</v>
       </c>
       <c r="O120" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, kd_golden_cross, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="n">
-        <v>5328</v>
+        <v>4736</v>
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>華容</t>
+          <t>泰博</t>
         </is>
       </c>
       <c r="C121" s="2" t="n">
         <v/>
       </c>
       <c r="D121" s="2" t="n">
-        <v>373.7479175246148</v>
+        <v>369.6217727484305</v>
       </c>
       <c r="E121" s="2" t="n">
-        <v>52.5</v>
+        <v>129.5</v>
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
@@ -6859,16 +6859,16 @@
         <v>0</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>35.48908699208265</v>
+        <v>47.23850738202734</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>17.16284906316569</v>
+        <v>18.72845506973326</v>
       </c>
       <c r="J121" s="2" t="n">
-        <v>0.6216553896099903</v>
+        <v>0.6903758132354407</v>
       </c>
       <c r="K121" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L121" s="2" t="n">
         <v>0</v>
@@ -6877,11 +6877,11 @@
         <v>-1</v>
       </c>
       <c r="N121" s="2" t="n">
-        <v>-0.325325642679676</v>
+        <v>0.4435926937202776</v>
       </c>
       <c r="O121" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
@@ -7428,7 +7428,7 @@
         <v/>
       </c>
       <c r="D132" s="2" t="n">
-        <v>340.0532727323804</v>
+        <v>340.0532727323797</v>
       </c>
       <c r="E132" s="2" t="n">
         <v>46.1</v>
@@ -7442,10 +7442,10 @@
         <v>0</v>
       </c>
       <c r="H132" s="2" t="n">
-        <v>43.60107828933761</v>
+        <v>43.60107828614754</v>
       </c>
       <c r="I132" s="2" t="n">
-        <v>15.01210521360166</v>
+        <v>15.01210524815607</v>
       </c>
       <c r="J132" s="2" t="n">
         <v>0.7708092727017104</v>
@@ -7460,7 +7460,7 @@
         <v>-1</v>
       </c>
       <c r="N132" s="2" t="n">
-        <v>-0.2255998323984899</v>
+        <v>-0.2255998326656032</v>
       </c>
       <c r="O132" s="2" t="inlineStr">
         <is>
@@ -7682,21 +7682,21 @@
     </row>
     <row r="137">
       <c r="A137" s="2" t="n">
-        <v>4746</v>
+        <v>4933</v>
       </c>
       <c r="B137" s="2" t="inlineStr">
         <is>
-          <t>台耀</t>
+          <t>友輝</t>
         </is>
       </c>
       <c r="C137" s="2" t="n">
         <v/>
       </c>
       <c r="D137" s="2" t="n">
-        <v>332.8108976928877</v>
+        <v>331.8525769142522</v>
       </c>
       <c r="E137" s="2" t="n">
-        <v>48.05</v>
+        <v>53.3</v>
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
@@ -7707,13 +7707,13 @@
         <v>0</v>
       </c>
       <c r="H137" s="2" t="n">
-        <v>48.9882245202915</v>
+        <v>49.11342259927697</v>
       </c>
       <c r="I137" s="2" t="n">
-        <v>19.64662258022237</v>
+        <v>19.29095252491589</v>
       </c>
       <c r="J137" s="2" t="n">
-        <v>0.9098321204909148</v>
+        <v>0.4986831378942747</v>
       </c>
       <c r="K137" s="2" t="n">
         <v>0</v>
@@ -7725,31 +7725,31 @@
         <v>-1</v>
       </c>
       <c r="N137" s="2" t="n">
-        <v>0.4509772723348415</v>
+        <v>0.2972900972454663</v>
       </c>
       <c r="O137" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="n">
-        <v>4933</v>
+        <v>5533</v>
       </c>
       <c r="B138" s="2" t="inlineStr">
         <is>
-          <t>友輝</t>
+          <t>皇鼎</t>
         </is>
       </c>
       <c r="C138" s="2" t="n">
         <v/>
       </c>
       <c r="D138" s="2" t="n">
-        <v>331.8525769142522</v>
+        <v>329.4071298218722</v>
       </c>
       <c r="E138" s="2" t="n">
-        <v>53.3</v>
+        <v>13.9</v>
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
@@ -7760,13 +7760,13 @@
         <v>0</v>
       </c>
       <c r="H138" s="2" t="n">
-        <v>49.11342259927697</v>
+        <v>45.96245656113359</v>
       </c>
       <c r="I138" s="2" t="n">
-        <v>19.29095252491589</v>
+        <v>22.22967874732579</v>
       </c>
       <c r="J138" s="2" t="n">
-        <v>0.4986831378942747</v>
+        <v>1.020011786286407</v>
       </c>
       <c r="K138" s="2" t="n">
         <v>0</v>
@@ -7778,31 +7778,31 @@
         <v>-1</v>
       </c>
       <c r="N138" s="2" t="n">
-        <v>0.2972900972454663</v>
+        <v>0.0136237558775179</v>
       </c>
       <c r="O138" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="n">
-        <v>5533</v>
+        <v>4554</v>
       </c>
       <c r="B139" s="2" t="inlineStr">
         <is>
-          <t>皇鼎</t>
+          <t>橙的</t>
         </is>
       </c>
       <c r="C139" s="2" t="n">
         <v/>
       </c>
       <c r="D139" s="2" t="n">
-        <v>329.4071298218722</v>
+        <v>328.7963069294382</v>
       </c>
       <c r="E139" s="2" t="n">
-        <v>13.9</v>
+        <v>28.25</v>
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
@@ -7813,13 +7813,13 @@
         <v>0</v>
       </c>
       <c r="H139" s="2" t="n">
-        <v>45.96245656113359</v>
+        <v>38.96062455407867</v>
       </c>
       <c r="I139" s="2" t="n">
-        <v>22.2296786745175</v>
+        <v>14.56126855376331</v>
       </c>
       <c r="J139" s="2" t="n">
-        <v>1.020011786286407</v>
+        <v>0.3050216295249408</v>
       </c>
       <c r="K139" s="2" t="n">
         <v>0</v>
@@ -7831,31 +7831,31 @@
         <v>-1</v>
       </c>
       <c r="N139" s="2" t="n">
-        <v>0.0136237558679783</v>
+        <v>0.0160174296318085</v>
       </c>
       <c r="O139" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
+          <t>macd_golden_cross, market_above_ma60, avoid_chase, hist_turn_positive, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="n">
-        <v>4554</v>
+        <v>5525</v>
       </c>
       <c r="B140" s="2" t="inlineStr">
         <is>
-          <t>橙的</t>
+          <t>順天</t>
         </is>
       </c>
       <c r="C140" s="2" t="n">
         <v/>
       </c>
       <c r="D140" s="2" t="n">
-        <v>328.7963069294382</v>
+        <v>325.6527003724277</v>
       </c>
       <c r="E140" s="2" t="n">
-        <v>28.25</v>
+        <v>22</v>
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
@@ -7866,13 +7866,13 @@
         <v>0</v>
       </c>
       <c r="H140" s="2" t="n">
-        <v>38.96062455407867</v>
+        <v>46.95076014018072</v>
       </c>
       <c r="I140" s="2" t="n">
-        <v>14.56126855376331</v>
+        <v>14.81113798317256</v>
       </c>
       <c r="J140" s="2" t="n">
-        <v>0.3050216295249408</v>
+        <v>1.445877026728663</v>
       </c>
       <c r="K140" s="2" t="n">
         <v>0</v>
@@ -7884,31 +7884,31 @@
         <v>-1</v>
       </c>
       <c r="N140" s="2" t="n">
-        <v>0.0160174296318085</v>
+        <v>0.0309726826107651</v>
       </c>
       <c r="O140" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, market_above_ma60, avoid_chase, hist_turn_positive, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="n">
-        <v>5525</v>
+        <v>4746</v>
       </c>
       <c r="B141" s="2" t="inlineStr">
         <is>
-          <t>順天</t>
+          <t>台耀</t>
         </is>
       </c>
       <c r="C141" s="2" t="n">
         <v/>
       </c>
       <c r="D141" s="2" t="n">
-        <v>325.6527003724277</v>
+        <v>322.8108976928878</v>
       </c>
       <c r="E141" s="2" t="n">
-        <v>22</v>
+        <v>48.05</v>
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
@@ -7919,13 +7919,13 @@
         <v>0</v>
       </c>
       <c r="H141" s="2" t="n">
-        <v>46.95076002583721</v>
+        <v>48.98822470495254</v>
       </c>
       <c r="I141" s="2" t="n">
-        <v>14.81113804703434</v>
+        <v>19.6466225514238</v>
       </c>
       <c r="J141" s="2" t="n">
-        <v>1.445877026728663</v>
+        <v>0.9098321204909148</v>
       </c>
       <c r="K141" s="2" t="n">
         <v>0</v>
@@ -7937,7 +7937,7 @@
         <v>-1</v>
       </c>
       <c r="N141" s="2" t="n">
-        <v>0.0309726826584648</v>
+        <v>0.4509772721822083</v>
       </c>
       <c r="O141" s="2" t="inlineStr">
         <is>
@@ -7972,10 +7972,10 @@
         <v>0</v>
       </c>
       <c r="H142" s="2" t="n">
-        <v>54.52397637915874</v>
+        <v>54.52397640275105</v>
       </c>
       <c r="I142" s="2" t="n">
-        <v>25.78690816602566</v>
+        <v>25.78690803195751</v>
       </c>
       <c r="J142" s="2" t="n">
         <v>0.5544223985408935</v>
@@ -7990,7 +7990,7 @@
         <v>-1</v>
       </c>
       <c r="N142" s="2" t="n">
-        <v>0.2224088638542499</v>
+        <v>0.2224088641812379</v>
       </c>
       <c r="O142" s="2" t="inlineStr">
         <is>
@@ -8064,7 +8064,7 @@
         <v/>
       </c>
       <c r="D144" s="2" t="n">
-        <v>313.2880976723586</v>
+        <v>313.2880976723588</v>
       </c>
       <c r="E144" s="2" t="n">
         <v>47.75</v>
@@ -8078,10 +8078,10 @@
         <v>0</v>
       </c>
       <c r="H144" s="2" t="n">
-        <v>51.4249725755913</v>
+        <v>51.42497257286751</v>
       </c>
       <c r="I144" s="2" t="n">
-        <v>9.150813281090976</v>
+        <v>9.150813316481772</v>
       </c>
       <c r="J144" s="2" t="n">
         <v>0.1764119572024591</v>
@@ -8096,7 +8096,7 @@
         <v>-1</v>
       </c>
       <c r="N144" s="2" t="n">
-        <v>0.9007175980841257</v>
+        <v>0.900717598198603</v>
       </c>
       <c r="O144" s="2" t="inlineStr">
         <is>
@@ -8131,10 +8131,10 @@
         <v>0</v>
       </c>
       <c r="H145" s="2" t="n">
-        <v>48.84779221907187</v>
+        <v>48.84779228111741</v>
       </c>
       <c r="I145" s="2" t="n">
-        <v>11.90645281349868</v>
+        <v>11.9064529118204</v>
       </c>
       <c r="J145" s="2" t="n">
         <v>0.9797262151725996</v>
@@ -8149,7 +8149,7 @@
         <v>-1</v>
       </c>
       <c r="N145" s="2" t="n">
-        <v>0.4121621668052841</v>
+        <v>0.4121621665572621</v>
       </c>
       <c r="O145" s="2" t="inlineStr">
         <is>
@@ -8488,7 +8488,7 @@
         <v/>
       </c>
       <c r="D152" s="2" t="n">
-        <v>305.9693742650846</v>
+        <v>305.9693742650847</v>
       </c>
       <c r="E152" s="2" t="n">
         <v>57</v>
@@ -8502,10 +8502,10 @@
         <v>0</v>
       </c>
       <c r="H152" s="2" t="n">
-        <v>42.44876130199821</v>
+        <v>42.44876136033536</v>
       </c>
       <c r="I152" s="2" t="n">
-        <v>22.7252763008583</v>
+        <v>22.72527630608824</v>
       </c>
       <c r="J152" s="2" t="n">
         <v>0.486597216991344</v>
@@ -8520,7 +8520,7 @@
         <v>-1</v>
       </c>
       <c r="N152" s="2" t="n">
-        <v>0.0105711743132836</v>
+        <v>0.0105711744277642</v>
       </c>
       <c r="O152" s="2" t="inlineStr">
         <is>
@@ -8555,10 +8555,10 @@
         <v>0</v>
       </c>
       <c r="H153" s="2" t="n">
-        <v>47.25069507169406</v>
+        <v>47.25069519294235</v>
       </c>
       <c r="I153" s="2" t="n">
-        <v>23.50623502243936</v>
+        <v>23.5062348453432</v>
       </c>
       <c r="J153" s="2" t="n">
         <v>0.9534628746549014</v>
@@ -8573,7 +8573,7 @@
         <v>-1</v>
       </c>
       <c r="N153" s="2" t="n">
-        <v>-0.0285971592483949</v>
+        <v>-0.0285971593437927</v>
       </c>
       <c r="O153" s="2" t="inlineStr">
         <is>
@@ -8661,10 +8661,10 @@
         <v>0</v>
       </c>
       <c r="H155" s="2" t="n">
-        <v>48.93469077698752</v>
+        <v>48.93469070577177</v>
       </c>
       <c r="I155" s="2" t="n">
-        <v>16.58839381840231</v>
+        <v>16.58839380905311</v>
       </c>
       <c r="J155" s="2" t="n">
         <v>0.514887230475541</v>
@@ -8679,7 +8679,7 @@
         <v>-1</v>
       </c>
       <c r="N155" s="2" t="n">
-        <v>1.381254261748911</v>
+        <v>1.381254263084448</v>
       </c>
       <c r="O155" s="2" t="inlineStr">
         <is>
@@ -8714,10 +8714,10 @@
         <v>0</v>
       </c>
       <c r="H156" s="2" t="n">
-        <v>43.60734476591416</v>
+        <v>43.60734499475668</v>
       </c>
       <c r="I156" s="2" t="n">
-        <v>20.37808577351033</v>
+        <v>20.37808563245102</v>
       </c>
       <c r="J156" s="2" t="n">
         <v>0.9822066545829666</v>
@@ -8732,7 +8732,7 @@
         <v>-1</v>
       </c>
       <c r="N156" s="2" t="n">
-        <v>-0.1709636220275723</v>
+        <v>-0.170963622285146</v>
       </c>
       <c r="O156" s="2" t="inlineStr">
         <is>
@@ -8753,7 +8753,7 @@
         <v/>
       </c>
       <c r="D157" s="2" t="n">
-        <v>297.4895334113256</v>
+        <v>297.4895334113253</v>
       </c>
       <c r="E157" s="2" t="n">
         <v>0</v>
@@ -8767,10 +8767,10 @@
         <v>0</v>
       </c>
       <c r="H157" s="2" t="n">
-        <v>43.259128592771</v>
+        <v>43.25912830508739</v>
       </c>
       <c r="I157" s="2" t="n">
-        <v>6.037876940130434</v>
+        <v>6.037876707501242</v>
       </c>
       <c r="J157" s="2" t="n">
         <v>0</v>
@@ -8785,7 +8785,7 @@
         <v>-1</v>
       </c>
       <c r="N157" s="2" t="n">
-        <v>-1.142128418987152</v>
+        <v>-1.142128409476045</v>
       </c>
       <c r="O157" s="2" t="inlineStr">
         <is>
@@ -8873,10 +8873,10 @@
         <v>0</v>
       </c>
       <c r="H159" s="2" t="n">
-        <v>54.12482346787461</v>
+        <v>54.12482351152418</v>
       </c>
       <c r="I159" s="2" t="n">
-        <v>15.48237277545052</v>
+        <v>15.48237274097931</v>
       </c>
       <c r="J159" s="2" t="n">
         <v>0.332006493111763</v>
@@ -8891,7 +8891,7 @@
         <v>-1</v>
       </c>
       <c r="N159" s="2" t="n">
-        <v>0.0403530022075236</v>
+        <v>0.0403530021979836</v>
       </c>
       <c r="O159" s="2" t="inlineStr">
         <is>
@@ -9032,10 +9032,10 @@
         <v>0</v>
       </c>
       <c r="H162" s="2" t="n">
-        <v>43.93351419499527</v>
+        <v>43.93351408240427</v>
       </c>
       <c r="I162" s="2" t="n">
-        <v>28.64462415761154</v>
+        <v>28.64462406918584</v>
       </c>
       <c r="J162" s="2" t="n">
         <v>0.4449259531982389</v>
@@ -9050,7 +9050,7 @@
         <v>-1</v>
       </c>
       <c r="N162" s="2" t="n">
-        <v>-0.0178037738321649</v>
+        <v>-0.0178037739084835</v>
       </c>
       <c r="O162" s="2" t="inlineStr">
         <is>
@@ -9085,10 +9085,10 @@
         <v>0</v>
       </c>
       <c r="H163" s="2" t="n">
-        <v>39.14733456831217</v>
+        <v>39.14733451439775</v>
       </c>
       <c r="I163" s="2" t="n">
-        <v>26.49209965893084</v>
+        <v>26.49209977612338</v>
       </c>
       <c r="J163" s="2" t="n">
         <v>0.2611405474991881</v>
@@ -9103,7 +9103,7 @@
         <v>-1</v>
       </c>
       <c r="N163" s="2" t="n">
-        <v>-0.3070688828413579</v>
+        <v>-0.3070688827650355</v>
       </c>
       <c r="O163" s="2" t="inlineStr">
         <is>
@@ -9247,7 +9247,7 @@
         <v>44.50176963169979</v>
       </c>
       <c r="I166" s="2" t="n">
-        <v>20.47116174710427</v>
+        <v>20.47116174225848</v>
       </c>
       <c r="J166" s="2" t="n">
         <v>1.530669433392466</v>
@@ -9403,10 +9403,10 @@
         <v>0</v>
       </c>
       <c r="H169" s="2" t="n">
-        <v>46.11593595909361</v>
+        <v>46.11593601681371</v>
       </c>
       <c r="I169" s="2" t="n">
-        <v>9.667543800332478</v>
+        <v>9.667543882387269</v>
       </c>
       <c r="J169" s="2" t="n">
         <v>0.4200221580799085</v>
@@ -9421,7 +9421,7 @@
         <v>-1</v>
       </c>
       <c r="N169" s="2" t="n">
-        <v>0.0593060403761354</v>
+        <v>0.0593060404524538</v>
       </c>
       <c r="O169" s="2" t="inlineStr">
         <is>
@@ -9615,10 +9615,10 @@
         <v>0</v>
       </c>
       <c r="H173" s="2" t="n">
-        <v>50.80143099141368</v>
+        <v>50.80143100325621</v>
       </c>
       <c r="I173" s="2" t="n">
-        <v>11.80607290582198</v>
+        <v>11.80607292896948</v>
       </c>
       <c r="J173" s="2" t="n">
         <v>1.111264795319508</v>
@@ -9633,7 +9633,7 @@
         <v>-1</v>
       </c>
       <c r="N173" s="2" t="n">
-        <v>0.9201757979893416</v>
+        <v>0.9201758001834928</v>
       </c>
       <c r="O173" s="2" t="inlineStr">
         <is>
@@ -9707,7 +9707,7 @@
         <v/>
       </c>
       <c r="D175" s="2" t="n">
-        <v>265.0492341646307</v>
+        <v>265.0492341646301</v>
       </c>
       <c r="E175" s="2" t="n">
         <v>49.8</v>
@@ -9721,10 +9721,10 @@
         <v>0</v>
       </c>
       <c r="H175" s="2" t="n">
-        <v>46.08649265746403</v>
+        <v>46.08649259479036</v>
       </c>
       <c r="I175" s="2" t="n">
-        <v>8.185717356126617</v>
+        <v>8.185717383722899</v>
       </c>
       <c r="J175" s="2" t="n">
         <v>0.5676462278746677</v>
@@ -9739,7 +9739,7 @@
         <v>-1</v>
       </c>
       <c r="N175" s="2" t="n">
-        <v>-0.0474868445833366</v>
+        <v>-0.0474868445642639</v>
       </c>
       <c r="O175" s="2" t="inlineStr">
         <is>
@@ -9827,10 +9827,10 @@
         <v>0</v>
       </c>
       <c r="H177" s="2" t="n">
-        <v>45.29301858717042</v>
+        <v>45.29301865733093</v>
       </c>
       <c r="I177" s="2" t="n">
-        <v>11.57049094855748</v>
+        <v>11.57049094369907</v>
       </c>
       <c r="J177" s="2" t="n">
         <v>0.5304997248117724</v>
@@ -10039,10 +10039,10 @@
         <v>0</v>
       </c>
       <c r="H181" s="2" t="n">
-        <v>36.6353901891469</v>
+        <v>36.63539027384758</v>
       </c>
       <c r="I181" s="2" t="n">
-        <v>28.64600020324098</v>
+        <v>28.64600017273147</v>
       </c>
       <c r="J181" s="2" t="n">
         <v>0.2566308928603555</v>
@@ -10057,7 +10057,7 @@
         <v>-1</v>
       </c>
       <c r="N181" s="2" t="n">
-        <v>1.690716617128061</v>
+        <v>1.690716613884558</v>
       </c>
       <c r="O181" s="2" t="inlineStr">
         <is>
@@ -10145,10 +10145,10 @@
         <v>0</v>
       </c>
       <c r="H183" s="2" t="n">
-        <v>43.3586856844763</v>
+        <v>43.35868592854909</v>
       </c>
       <c r="I183" s="2" t="n">
-        <v>16.11188418261095</v>
+        <v>16.11188419517899</v>
       </c>
       <c r="J183" s="2" t="n">
         <v>0.6735789684510514</v>
@@ -10290,7 +10290,7 @@
         <v/>
       </c>
       <c r="D186" s="2" t="n">
-        <v>240.4598281405351</v>
+        <v>240.4598281405352</v>
       </c>
       <c r="E186" s="2" t="n">
         <v>171</v>
@@ -10304,10 +10304,10 @@
         <v>0</v>
       </c>
       <c r="H186" s="2" t="n">
-        <v>39.72707185919232</v>
+        <v>39.72707153363234</v>
       </c>
       <c r="I186" s="2" t="n">
-        <v>22.35801553880813</v>
+        <v>22.35801579933901</v>
       </c>
       <c r="J186" s="2" t="n">
         <v>1.147983389838965</v>
@@ -10322,7 +10322,7 @@
         <v>-1</v>
       </c>
       <c r="N186" s="2" t="n">
-        <v>0.2374407730662109</v>
+        <v>0.2374407747833551</v>
       </c>
       <c r="O186" s="2" t="inlineStr">
         <is>
@@ -10357,10 +10357,10 @@
         <v>0</v>
       </c>
       <c r="H187" s="2" t="n">
-        <v>50.83245383142919</v>
+        <v>50.83245379515086</v>
       </c>
       <c r="I187" s="2" t="n">
-        <v>13.89687189842728</v>
+        <v>13.89687189943094</v>
       </c>
       <c r="J187" s="2" t="n">
         <v>0.4517965427289422</v>
@@ -10375,7 +10375,7 @@
         <v>-1</v>
       </c>
       <c r="N187" s="2" t="n">
-        <v>0.1323834426544801</v>
+        <v>0.1323834427021717</v>
       </c>
       <c r="O187" s="2" t="inlineStr">
         <is>
@@ -10396,7 +10396,7 @@
         <v/>
       </c>
       <c r="D188" s="2" t="n">
-        <v>240.1043172616621</v>
+        <v>240.1043172616622</v>
       </c>
       <c r="E188" s="2" t="n">
         <v>8.210000000000001</v>
@@ -10410,10 +10410,10 @@
         <v>0</v>
       </c>
       <c r="H188" s="2" t="n">
-        <v>45.39714223484096</v>
+        <v>45.39714226878964</v>
       </c>
       <c r="I188" s="2" t="n">
-        <v>10.3027364142341</v>
+        <v>10.30273647584461</v>
       </c>
       <c r="J188" s="2" t="n">
         <v>1.069619291800466</v>
@@ -10428,7 +10428,7 @@
         <v>-1</v>
       </c>
       <c r="N188" s="2" t="n">
-        <v>0.0177806431038886</v>
+        <v>0.017780643094348</v>
       </c>
       <c r="O188" s="2" t="inlineStr">
         <is>
@@ -10516,10 +10516,10 @@
         <v>0</v>
       </c>
       <c r="H190" s="2" t="n">
-        <v>43.67335942894762</v>
+        <v>43.67335931707998</v>
       </c>
       <c r="I190" s="2" t="n">
-        <v>11.82524764407072</v>
+        <v>11.82524768873736</v>
       </c>
       <c r="J190" s="2" t="n">
         <v>0.863673806706432</v>
@@ -10534,7 +10534,7 @@
         <v>-1</v>
       </c>
       <c r="N190" s="2" t="n">
-        <v>-0.2118147459046854</v>
+        <v>-0.2118147453323039</v>
       </c>
       <c r="O190" s="2" t="inlineStr">
         <is>
@@ -10675,10 +10675,10 @@
         <v>0</v>
       </c>
       <c r="H193" s="2" t="n">
-        <v>41.03211735407216</v>
+        <v>41.03211662333602</v>
       </c>
       <c r="I193" s="2" t="n">
-        <v>14.2909614641744</v>
+        <v>14.29096193881061</v>
       </c>
       <c r="J193" s="2" t="n">
         <v>0.4540399902863182</v>
@@ -10693,7 +10693,7 @@
         <v>-1</v>
       </c>
       <c r="N193" s="2" t="n">
-        <v>0.0248822417842151</v>
+        <v>0.0248822422230402</v>
       </c>
       <c r="O193" s="2" t="inlineStr">
         <is>
@@ -10714,7 +10714,7 @@
         <v/>
       </c>
       <c r="D194" s="2" t="n">
-        <v>225.6138940032888</v>
+        <v>225.6138940032889</v>
       </c>
       <c r="E194" s="2" t="n">
         <v>181</v>
@@ -10728,10 +10728,10 @@
         <v>0</v>
       </c>
       <c r="H194" s="2" t="n">
-        <v>42.98982478399673</v>
+        <v>42.98982491358635</v>
       </c>
       <c r="I194" s="2" t="n">
-        <v>25.41062739879325</v>
+        <v>25.4106273721635</v>
       </c>
       <c r="J194" s="2" t="n">
         <v>0.6742580983440967</v>
@@ -10746,7 +10746,7 @@
         <v>-1</v>
       </c>
       <c r="N194" s="2" t="n">
-        <v>0.3722414712251791</v>
+        <v>0.3722414713205726</v>
       </c>
       <c r="O194" s="2" t="inlineStr">
         <is>
@@ -10781,10 +10781,10 @@
         <v>0</v>
       </c>
       <c r="H195" s="2" t="n">
-        <v>44.58153139188328</v>
+        <v>44.58153137089904</v>
       </c>
       <c r="I195" s="2" t="n">
-        <v>13.59802077090101</v>
+        <v>13.59802084246598</v>
       </c>
       <c r="J195" s="2" t="n">
         <v>0.4776954869481463</v>
@@ -10799,7 +10799,7 @@
         <v>-1</v>
       </c>
       <c r="N195" s="2" t="n">
-        <v>0.2388942382693044</v>
+        <v>0.238894238364709</v>
       </c>
       <c r="O195" s="2" t="inlineStr">
         <is>
@@ -10834,10 +10834,10 @@
         <v>0</v>
       </c>
       <c r="H196" s="2" t="n">
-        <v>29.08697283132749</v>
+        <v>29.08697285597884</v>
       </c>
       <c r="I196" s="2" t="n">
-        <v>37.11217694972702</v>
+        <v>37.11217697473745</v>
       </c>
       <c r="J196" s="2" t="n">
         <v>1.365250432029785</v>
@@ -10852,7 +10852,7 @@
         <v>-1</v>
       </c>
       <c r="N196" s="2" t="n">
-        <v>-0.0132792431893705</v>
+        <v>-0.0132792431416709</v>
       </c>
       <c r="O196" s="2" t="inlineStr">
         <is>
@@ -10873,7 +10873,7 @@
         <v/>
       </c>
       <c r="D197" s="2" t="n">
-        <v>224.5130530660275</v>
+        <v>224.5130530660273</v>
       </c>
       <c r="E197" s="2" t="n">
         <v>115.5</v>
@@ -10887,10 +10887,10 @@
         <v>0</v>
       </c>
       <c r="H197" s="2" t="n">
-        <v>49.71025692028446</v>
+        <v>49.71025699316934</v>
       </c>
       <c r="I197" s="2" t="n">
-        <v>8.58947210663427</v>
+        <v>8.589472084514128</v>
       </c>
       <c r="J197" s="2" t="n">
         <v>0.4613105738754158</v>
@@ -10926,7 +10926,7 @@
         <v/>
       </c>
       <c r="D198" s="2" t="n">
-        <v>221.8750174789388</v>
+        <v>221.8750174789392</v>
       </c>
       <c r="E198" s="2" t="n">
         <v>41.65</v>
@@ -10940,10 +10940,10 @@
         <v>0</v>
       </c>
       <c r="H198" s="2" t="n">
-        <v>38.00506852453842</v>
+        <v>38.00506881005613</v>
       </c>
       <c r="I198" s="2" t="n">
-        <v>16.33185954024674</v>
+        <v>16.33185955715097</v>
       </c>
       <c r="J198" s="2" t="n">
         <v>0.8426139970972919</v>
@@ -10958,7 +10958,7 @@
         <v>-1</v>
       </c>
       <c r="N198" s="2" t="n">
-        <v>-0.07794737532970281</v>
+        <v>-0.07794737531062031</v>
       </c>
       <c r="O198" s="2" t="inlineStr">
         <is>
@@ -11021,21 +11021,21 @@
     </row>
     <row r="200">
       <c r="A200" s="2" t="n">
-        <v>4739</v>
+        <v>6125</v>
       </c>
       <c r="B200" s="2" t="inlineStr">
         <is>
-          <t>康普</t>
+          <t>廣運</t>
         </is>
       </c>
       <c r="C200" s="2" t="n">
         <v/>
       </c>
       <c r="D200" s="2" t="n">
-        <v>215.8760756526308</v>
+        <v>214.2199200800408</v>
       </c>
       <c r="E200" s="2" t="n">
-        <v>79.5</v>
+        <v>48.6</v>
       </c>
       <c r="F200" s="2" t="inlineStr">
         <is>
@@ -11046,16 +11046,16 @@
         <v>0</v>
       </c>
       <c r="H200" s="2" t="n">
-        <v>43.9425685125929</v>
+        <v>42.98035354207439</v>
       </c>
       <c r="I200" s="2" t="n">
-        <v>13.58983677710765</v>
+        <v>11.52490659082862</v>
       </c>
       <c r="J200" s="2" t="n">
-        <v>0.3586773918952333</v>
+        <v>0.3959101714644029</v>
       </c>
       <c r="K200" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L200" s="2" t="n">
         <v>0</v>
@@ -11064,31 +11064,31 @@
         <v>-1</v>
       </c>
       <c r="N200" s="2" t="n">
-        <v>0.3026009450450995</v>
+        <v>-0.0295914079375516</v>
       </c>
       <c r="O200" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="2" t="n">
-        <v>6125</v>
+        <v>5344</v>
       </c>
       <c r="B201" s="2" t="inlineStr">
         <is>
-          <t>廣運</t>
+          <t>立衛</t>
         </is>
       </c>
       <c r="C201" s="2" t="n">
         <v/>
       </c>
       <c r="D201" s="2" t="n">
-        <v>214.2199200800405</v>
+        <v>213.3802798857282</v>
       </c>
       <c r="E201" s="2" t="n">
-        <v>48.6</v>
+        <v>13.6</v>
       </c>
       <c r="F201" s="2" t="inlineStr">
         <is>
@@ -11099,16 +11099,16 @@
         <v>0</v>
       </c>
       <c r="H201" s="2" t="n">
-        <v>42.98035372881272</v>
+        <v>51.30382951280489</v>
       </c>
       <c r="I201" s="2" t="n">
-        <v>11.52490661724138</v>
+        <v>13.39901384771431</v>
       </c>
       <c r="J201" s="2" t="n">
-        <v>0.3959101714644029</v>
+        <v>2.408414771351022</v>
       </c>
       <c r="K201" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L201" s="2" t="n">
         <v>0</v>
@@ -11117,31 +11117,31 @@
         <v>-1</v>
       </c>
       <c r="N201" s="2" t="n">
-        <v>-0.0295914083191436</v>
+        <v>0.0743053857892178</v>
       </c>
       <c r="O201" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d</t>
+          <t>volume_break, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="2" t="n">
-        <v>5344</v>
+        <v>5484</v>
       </c>
       <c r="B202" s="2" t="inlineStr">
         <is>
-          <t>立衛</t>
+          <t>慧友</t>
         </is>
       </c>
       <c r="C202" s="2" t="n">
         <v/>
       </c>
       <c r="D202" s="2" t="n">
-        <v>213.3802798857282</v>
+        <v>212.027389601334</v>
       </c>
       <c r="E202" s="2" t="n">
-        <v>13.6</v>
+        <v>39.45</v>
       </c>
       <c r="F202" s="2" t="inlineStr">
         <is>
@@ -11152,13 +11152,13 @@
         <v>0</v>
       </c>
       <c r="H202" s="2" t="n">
-        <v>51.30382951280489</v>
+        <v>46.02314864527166</v>
       </c>
       <c r="I202" s="2" t="n">
-        <v>13.39901384771431</v>
+        <v>8.148483668587355</v>
       </c>
       <c r="J202" s="2" t="n">
-        <v>2.408414771351022</v>
+        <v>0.3683164154452263</v>
       </c>
       <c r="K202" s="2" t="n">
         <v>0</v>
@@ -11170,31 +11170,31 @@
         <v>-1</v>
       </c>
       <c r="N202" s="2" t="n">
-        <v>0.0743053857892178</v>
+        <v>0.0202360681737636</v>
       </c>
       <c r="O202" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="2" t="n">
-        <v>5484</v>
+        <v>5498</v>
       </c>
       <c r="B203" s="2" t="inlineStr">
         <is>
-          <t>慧友</t>
+          <t>凱崴</t>
         </is>
       </c>
       <c r="C203" s="2" t="n">
         <v/>
       </c>
       <c r="D203" s="2" t="n">
-        <v>212.027389601334</v>
+        <v>209.673416321169</v>
       </c>
       <c r="E203" s="2" t="n">
-        <v>39.45</v>
+        <v>50.1</v>
       </c>
       <c r="F203" s="2" t="inlineStr">
         <is>
@@ -11205,13 +11205,13 @@
         <v>0</v>
       </c>
       <c r="H203" s="2" t="n">
-        <v>46.02314864527166</v>
+        <v>44.49347795764776</v>
       </c>
       <c r="I203" s="2" t="n">
-        <v>8.148483668587355</v>
+        <v>13.27297460164622</v>
       </c>
       <c r="J203" s="2" t="n">
-        <v>0.3683164154452263</v>
+        <v>0.3235307004148744</v>
       </c>
       <c r="K203" s="2" t="n">
         <v>0</v>
@@ -11223,31 +11223,31 @@
         <v>-1</v>
       </c>
       <c r="N203" s="2" t="n">
-        <v>0.0202360681737636</v>
+        <v>-0.2630507003054484</v>
       </c>
       <c r="O203" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="2" t="n">
-        <v>5498</v>
+        <v>4306</v>
       </c>
       <c r="B204" s="2" t="inlineStr">
         <is>
-          <t>凱崴</t>
+          <t>炎洲</t>
         </is>
       </c>
       <c r="C204" s="2" t="n">
         <v/>
       </c>
       <c r="D204" s="2" t="n">
-        <v>209.673416321169</v>
+        <v>209.3153550017613</v>
       </c>
       <c r="E204" s="2" t="n">
-        <v>50.1</v>
+        <v>14.5</v>
       </c>
       <c r="F204" s="2" t="inlineStr">
         <is>
@@ -11258,13 +11258,13 @@
         <v>0</v>
       </c>
       <c r="H204" s="2" t="n">
-        <v>44.49347795764776</v>
+        <v>40.70635652953064</v>
       </c>
       <c r="I204" s="2" t="n">
-        <v>13.27297460164622</v>
+        <v>17.56143443508607</v>
       </c>
       <c r="J204" s="2" t="n">
-        <v>0.3235307004148744</v>
+        <v>0.8147368775389454</v>
       </c>
       <c r="K204" s="2" t="n">
         <v>0</v>
@@ -11276,31 +11276,31 @@
         <v>-1</v>
       </c>
       <c r="N204" s="2" t="n">
-        <v>-0.2630507003054484</v>
+        <v>-0.0382910523016062</v>
       </c>
       <c r="O204" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="2" t="n">
-        <v>4306</v>
+        <v>6151</v>
       </c>
       <c r="B205" s="2" t="inlineStr">
         <is>
-          <t>炎洲</t>
+          <t>晉倫</t>
         </is>
       </c>
       <c r="C205" s="2" t="n">
         <v/>
       </c>
       <c r="D205" s="2" t="n">
-        <v>209.3153550017615</v>
+        <v>208.3553204669721</v>
       </c>
       <c r="E205" s="2" t="n">
-        <v>14.5</v>
+        <v>35</v>
       </c>
       <c r="F205" s="2" t="inlineStr">
         <is>
@@ -11311,13 +11311,13 @@
         <v>0</v>
       </c>
       <c r="H205" s="2" t="n">
-        <v>40.70635648125419</v>
+        <v>46.936056668112</v>
       </c>
       <c r="I205" s="2" t="n">
-        <v>17.56143436058027</v>
+        <v>18.42540105037886</v>
       </c>
       <c r="J205" s="2" t="n">
-        <v>0.8147368775389454</v>
+        <v>0.7463693518935122</v>
       </c>
       <c r="K205" s="2" t="n">
         <v>0</v>
@@ -11329,7 +11329,7 @@
         <v>-1</v>
       </c>
       <c r="N205" s="2" t="n">
-        <v>-0.0382910522729885</v>
+        <v>0.09668930537474379</v>
       </c>
       <c r="O205" s="2" t="inlineStr">
         <is>
@@ -11339,21 +11339,21 @@
     </row>
     <row r="206">
       <c r="A206" s="2" t="n">
-        <v>6151</v>
+        <v>4739</v>
       </c>
       <c r="B206" s="2" t="inlineStr">
         <is>
-          <t>晉倫</t>
+          <t>康普</t>
         </is>
       </c>
       <c r="C206" s="2" t="n">
         <v/>
       </c>
       <c r="D206" s="2" t="n">
-        <v>208.3553204669719</v>
+        <v>205.8760756526308</v>
       </c>
       <c r="E206" s="2" t="n">
-        <v>35</v>
+        <v>79.5</v>
       </c>
       <c r="F206" s="2" t="inlineStr">
         <is>
@@ -11364,13 +11364,13 @@
         <v>0</v>
       </c>
       <c r="H206" s="2" t="n">
-        <v>46.93605660704999</v>
+        <v>43.94256847417937</v>
       </c>
       <c r="I206" s="2" t="n">
-        <v>18.42540108441149</v>
+        <v>13.58983687880244</v>
       </c>
       <c r="J206" s="2" t="n">
-        <v>0.7463693518935122</v>
+        <v>0.3586773918952333</v>
       </c>
       <c r="K206" s="2" t="n">
         <v>0</v>
@@ -11382,11 +11382,11 @@
         <v>-1</v>
       </c>
       <c r="N206" s="2" t="n">
-        <v>0.09668930536520549</v>
+        <v>0.3026009452168217</v>
       </c>
       <c r="O206" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
@@ -11417,10 +11417,10 @@
         <v>0</v>
       </c>
       <c r="H207" s="2" t="n">
-        <v>49.90384234064884</v>
+        <v>49.9038423290845</v>
       </c>
       <c r="I207" s="2" t="n">
-        <v>5.316723259777028</v>
+        <v>5.316723294879075</v>
       </c>
       <c r="J207" s="2" t="n">
         <v>1.280267166791001</v>
@@ -11509,7 +11509,7 @@
         <v/>
       </c>
       <c r="D209" s="2" t="n">
-        <v>198.2444567603909</v>
+        <v>198.244456760391</v>
       </c>
       <c r="E209" s="2" t="n">
         <v>295.5</v>
@@ -11526,7 +11526,7 @@
         <v>43.20183262250087</v>
       </c>
       <c r="I209" s="2" t="n">
-        <v>10.16147325876898</v>
+        <v>10.16147321757393</v>
       </c>
       <c r="J209" s="2" t="n">
         <v>0.912548454331184</v>
@@ -11541,7 +11541,7 @@
         <v>-1</v>
       </c>
       <c r="N209" s="2" t="n">
-        <v>-1.21534709890467</v>
+        <v>-1.215347097569116</v>
       </c>
       <c r="O209" s="2" t="inlineStr">
         <is>
@@ -11562,7 +11562,7 @@
         <v/>
       </c>
       <c r="D210" s="2" t="n">
-        <v>197.1723617639047</v>
+        <v>197.1723617639048</v>
       </c>
       <c r="E210" s="2" t="n">
         <v>155</v>
@@ -11579,7 +11579,7 @@
         <v>43.25751413791728</v>
       </c>
       <c r="I210" s="2" t="n">
-        <v>17.01080717634719</v>
+        <v>17.0108071892418</v>
       </c>
       <c r="J210" s="2" t="n">
         <v>0.2182509847570002</v>
@@ -11594,7 +11594,7 @@
         <v>-1</v>
       </c>
       <c r="N210" s="2" t="n">
-        <v>-0.8727172971763641</v>
+        <v>-0.8727172968901957</v>
       </c>
       <c r="O210" s="2" t="inlineStr">
         <is>
@@ -11629,10 +11629,10 @@
         <v>0</v>
       </c>
       <c r="H211" s="2" t="n">
-        <v>34.89787026931086</v>
+        <v>34.89787033965214</v>
       </c>
       <c r="I211" s="2" t="n">
-        <v>26.27540656790316</v>
+        <v>26.27540651129111</v>
       </c>
       <c r="J211" s="2" t="n">
         <v>0.4659778949367941</v>
@@ -11647,7 +11647,7 @@
         <v>-1</v>
       </c>
       <c r="N211" s="2" t="n">
-        <v>0.0474543884883225</v>
+        <v>0.0474543885837217</v>
       </c>
       <c r="O211" s="2" t="inlineStr">
         <is>
@@ -11788,10 +11788,10 @@
         <v>0</v>
       </c>
       <c r="H214" s="2" t="n">
-        <v>33.25420057456016</v>
+        <v>33.25420062616261</v>
       </c>
       <c r="I214" s="2" t="n">
-        <v>41.53569081838821</v>
+        <v>41.53569094490986</v>
       </c>
       <c r="J214" s="2" t="n">
         <v>0.3742701373005618</v>
@@ -11806,7 +11806,7 @@
         <v>-1</v>
       </c>
       <c r="N214" s="2" t="n">
-        <v>0.0505418803500555</v>
+        <v>0.0505418803977557</v>
       </c>
       <c r="O214" s="2" t="inlineStr">
         <is>
@@ -11841,10 +11841,10 @@
         <v>0</v>
       </c>
       <c r="H215" s="2" t="n">
-        <v>35.16156082767444</v>
+        <v>35.16156123042909</v>
       </c>
       <c r="I215" s="2" t="n">
-        <v>18.64751823172422</v>
+        <v>18.64751824143272</v>
       </c>
       <c r="J215" s="2" t="n">
         <v>1.248454553258586</v>
@@ -11859,7 +11859,7 @@
         <v>-1</v>
       </c>
       <c r="N215" s="2" t="n">
-        <v>-0.0567659600229502</v>
+        <v>-0.0567659600420298</v>
       </c>
       <c r="O215" s="2" t="inlineStr">
         <is>
@@ -11894,10 +11894,10 @@
         <v>0</v>
       </c>
       <c r="H216" s="2" t="n">
-        <v>44.25183874848275</v>
+        <v>44.25183873673489</v>
       </c>
       <c r="I216" s="2" t="n">
-        <v>12.18525462675094</v>
+        <v>12.18525471269858</v>
       </c>
       <c r="J216" s="2" t="n">
         <v>0.3668515811392365</v>
@@ -11912,7 +11912,7 @@
         <v>-1</v>
       </c>
       <c r="N216" s="2" t="n">
-        <v>-0.06373081484978051</v>
+        <v>-0.0637308148116183</v>
       </c>
       <c r="O216" s="2" t="inlineStr">
         <is>
@@ -12162,7 +12162,7 @@
         <v>47.48833833579987</v>
       </c>
       <c r="I221" s="2" t="n">
-        <v>13.25497070180886</v>
+        <v>13.25497075728752</v>
       </c>
       <c r="J221" s="2" t="n">
         <v>0.5519699318203939</v>
@@ -12198,7 +12198,7 @@
         <v/>
       </c>
       <c r="D222" s="2" t="n">
-        <v>153.1430886046355</v>
+        <v>153.1430886046356</v>
       </c>
       <c r="E222" s="2" t="n">
         <v>73.90000000000001</v>
@@ -12212,10 +12212,10 @@
         <v>0</v>
       </c>
       <c r="H222" s="2" t="n">
-        <v>41.0335635801373</v>
+        <v>41.03356368285541</v>
       </c>
       <c r="I222" s="2" t="n">
-        <v>17.14633575884762</v>
+        <v>17.14633581660162</v>
       </c>
       <c r="J222" s="2" t="n">
         <v>0.4349277615441214</v>
@@ -12230,7 +12230,7 @@
         <v>-1</v>
       </c>
       <c r="N222" s="2" t="n">
-        <v>0.0635818059874691</v>
+        <v>0.06358180602561141</v>
       </c>
       <c r="O222" s="2" t="inlineStr">
         <is>
@@ -12265,10 +12265,10 @@
         <v>0</v>
       </c>
       <c r="H223" s="2" t="n">
-        <v>44.44787840234896</v>
+        <v>44.44787842621128</v>
       </c>
       <c r="I223" s="2" t="n">
-        <v>16.35050515501829</v>
+        <v>16.35050535929451</v>
       </c>
       <c r="J223" s="2" t="n">
         <v>0.7105541588731364</v>
@@ -12283,7 +12283,7 @@
         <v>-1</v>
       </c>
       <c r="N223" s="2" t="n">
-        <v>-0.0319985910404985</v>
+        <v>-0.0319985907924613</v>
       </c>
       <c r="O223" s="2" t="inlineStr">
         <is>
@@ -12371,10 +12371,10 @@
         <v>0</v>
       </c>
       <c r="H225" s="2" t="n">
-        <v>45.6938801536231</v>
+        <v>45.6938801751085</v>
       </c>
       <c r="I225" s="2" t="n">
-        <v>8.052207164298357</v>
+        <v>8.052207063779052</v>
       </c>
       <c r="J225" s="2" t="n">
         <v>0.6764847080133984</v>
@@ -12389,7 +12389,7 @@
         <v>-1</v>
       </c>
       <c r="N225" s="2" t="n">
-        <v>1.382483324670436</v>
+        <v>1.382483326082328</v>
       </c>
       <c r="O225" s="2" t="inlineStr">
         <is>
@@ -12583,10 +12583,10 @@
         <v>0</v>
       </c>
       <c r="H229" s="2" t="n">
-        <v>38.17546831270572</v>
+        <v>38.17546847164717</v>
       </c>
       <c r="I229" s="2" t="n">
-        <v>18.69704826967136</v>
+        <v>18.6970482301331</v>
       </c>
       <c r="J229" s="2" t="n">
         <v>0.8073268913844186</v>
@@ -12728,7 +12728,7 @@
         <v/>
       </c>
       <c r="D232" s="2" t="n">
-        <v>100.2683716666646</v>
+        <v>100.2683716666647</v>
       </c>
       <c r="E232" s="2" t="n">
         <v>60.7</v>
@@ -12742,10 +12742,10 @@
         <v>0</v>
       </c>
       <c r="H232" s="2" t="n">
-        <v>39.82664323863034</v>
+        <v>39.82664318533468</v>
       </c>
       <c r="I232" s="2" t="n">
-        <v>12.79464949531454</v>
+        <v>12.79464961637038</v>
       </c>
       <c r="J232" s="2" t="n">
         <v>1.132880432255485</v>
@@ -12760,7 +12760,7 @@
         <v>-1</v>
       </c>
       <c r="N232" s="2" t="n">
-        <v>-0.0362612642454093</v>
+        <v>-0.0362612639782975</v>
       </c>
       <c r="O232" s="2" t="inlineStr">
         <is>
@@ -12795,10 +12795,10 @@
         <v>0</v>
       </c>
       <c r="H233" s="2" t="n">
-        <v>45.65549526928771</v>
+        <v>45.65549525937406</v>
       </c>
       <c r="I233" s="2" t="n">
-        <v>10.92818863624725</v>
+        <v>10.92818860019256</v>
       </c>
       <c r="J233" s="2" t="n">
         <v>0.3174744785326019</v>
@@ -12887,7 +12887,7 @@
         <v/>
       </c>
       <c r="D235" s="2" t="n">
-        <v>85.50787873335828</v>
+        <v>85.50787873335817</v>
       </c>
       <c r="E235" s="2" t="n">
         <v>152.5</v>
@@ -12901,10 +12901,10 @@
         <v>0</v>
       </c>
       <c r="H235" s="2" t="n">
-        <v>46.27645053095302</v>
+        <v>46.27645059366352</v>
       </c>
       <c r="I235" s="2" t="n">
-        <v>14.70029415869746</v>
+        <v>14.70029421995235</v>
       </c>
       <c r="J235" s="2" t="n">
         <v>0.5316619293856815</v>
@@ -12940,7 +12940,7 @@
         <v/>
       </c>
       <c r="D236" s="2" t="n">
-        <v>78.16668779222115</v>
+        <v>78.16668779222113</v>
       </c>
       <c r="E236" s="2" t="n">
         <v>6.98</v>
@@ -12954,10 +12954,10 @@
         <v>0</v>
       </c>
       <c r="H236" s="2" t="n">
-        <v>39.04631399389796</v>
+        <v>39.04631386231552</v>
       </c>
       <c r="I236" s="2" t="n">
-        <v>17.64359121928257</v>
+        <v>17.64359153731353</v>
       </c>
       <c r="J236" s="2" t="n">
         <v>0.4797449472608868</v>
@@ -12972,7 +12972,7 @@
         <v>-1</v>
       </c>
       <c r="N236" s="2" t="n">
-        <v>-0.003041863932628</v>
+        <v>-0.0030418638467705</v>
       </c>
       <c r="O236" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
scan: seg4 2026-09-28 15:55 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq5_2026-09-24.xlsx
+++ b/output/full_scan/batch_seq5_2026-09-24.xlsx
@@ -538,7 +538,7 @@
         <v/>
       </c>
       <c r="D2" s="2" t="n">
-        <v>1227.724121358847</v>
+        <v>1227.724121358848</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>167.5</v>
@@ -552,10 +552,10 @@
         <v>0</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>63.44963998223238</v>
+        <v>63.44963995835961</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>29.08177591647655</v>
+        <v>29.08177590217821</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>1.953804200323101</v>
@@ -570,7 +570,7 @@
         <v>-1</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>0.5735494622183817</v>
+        <v>0.5735494628365414</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
@@ -605,10 +605,10 @@
         <v>0</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>63.11557621559333</v>
+        <v>63.11557629510772</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>21.85065912430507</v>
+        <v>21.85065916508132</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>1.884566291001656</v>
@@ -623,7 +623,7 @@
         <v>-1</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>2.921862004864884</v>
+        <v>2.921862003999448</v>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
@@ -711,10 +711,10 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>58.14715927732101</v>
+        <v>58.14715924177326</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>7.428292181474113</v>
+        <v>7.42829218147411</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>2.984149960768015</v>
@@ -729,7 +729,7 @@
         <v>-1</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>0.419576754741398</v>
+        <v>0.4195767547620064</v>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
@@ -764,10 +764,10 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>71.87012517358598</v>
+        <v>71.87012486546516</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>41.21417960770197</v>
+        <v>41.21417952142738</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>2.221160022566784</v>
@@ -782,7 +782,7 @@
         <v>-1</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>0.9009467567006172</v>
+        <v>0.900946758019384</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
@@ -870,10 +870,10 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>82.3309830031868</v>
+        <v>82.33098303731487</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>34.1694528884513</v>
+        <v>34.16945289366775</v>
       </c>
       <c r="J8" s="2" t="n">
         <v>2.85452166384325</v>
@@ -888,7 +888,7 @@
         <v>-1</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>0.4972411724044994</v>
+        <v>0.4972411723838936</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
@@ -923,10 +923,10 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>60.02278600536215</v>
+        <v>60.02278602924059</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>20.81748097868815</v>
+        <v>20.81748097868814</v>
       </c>
       <c r="J9" s="2" t="n">
         <v>0.421897474397201</v>
@@ -941,7 +941,7 @@
         <v>-1</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>0.3933607759377659</v>
+        <v>0.3933607760407844</v>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
@@ -979,7 +979,7 @@
         <v>64.63268312631922</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>29.74017476859016</v>
+        <v>29.74017471876602</v>
       </c>
       <c r="J10" s="2" t="n">
         <v>3.074153476838017</v>
@@ -1029,10 +1029,10 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>59.79614933623459</v>
+        <v>59.79614940089044</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>13.48091117589519</v>
+        <v>13.48091120238967</v>
       </c>
       <c r="J11" s="2" t="n">
         <v>1.543262372369996</v>
@@ -1047,7 +1047,7 @@
         <v>-1</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>1.057951388550225</v>
+        <v>1.057951388282368</v>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
@@ -1082,10 +1082,10 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>61.92329036856442</v>
+        <v>61.92329039098972</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>24.35083567888885</v>
+        <v>24.35083573154417</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>0.5727392674672481</v>
@@ -1100,7 +1100,7 @@
         <v>-1</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>163.1536680328363</v>
+        <v>163.1536680163508</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>91.8344432393682</v>
+        <v>91.83444323761884</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>34.62572886182473</v>
+        <v>34.62572895809286</v>
       </c>
       <c r="J13" s="2" t="n">
         <v>3.270031234056824</v>
@@ -1153,7 +1153,7 @@
         <v>-1</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>1.008407352128402</v>
+        <v>1.008407352221131</v>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
@@ -1188,10 +1188,10 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>56.06317325998033</v>
+        <v>56.06317320654698</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>21.46421893329095</v>
+        <v>21.46421892338949</v>
       </c>
       <c r="J14" s="2" t="n">
         <v>0.4020898799005478</v>
@@ -1206,7 +1206,7 @@
         <v>-1</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>0.0494418617672866</v>
+        <v>0.049441861932133</v>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
@@ -1280,7 +1280,7 @@
         <v/>
       </c>
       <c r="D16" s="2" t="n">
-        <v>818.2264790585301</v>
+        <v>818.22647905853</v>
       </c>
       <c r="E16" s="2" t="n">
         <v>43.7</v>
@@ -1312,7 +1312,7 @@
         <v>-1</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>-0.0003830730131451</v>
+        <v>-0.000383072982238</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
@@ -1347,10 +1347,10 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>64.43335122487682</v>
+        <v>64.43335122965928</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>31.54345348825405</v>
+        <v>31.5434534908422</v>
       </c>
       <c r="J17" s="2" t="n">
         <v>2.59843557217022</v>
@@ -1365,7 +1365,7 @@
         <v>-1</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>0.99573277063622</v>
+        <v>0.99573277067743</v>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
@@ -1400,10 +1400,10 @@
         <v>0</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>68.98074728502132</v>
+        <v>68.98074731936074</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>18.77256793749486</v>
+        <v>18.77256796617817</v>
       </c>
       <c r="J18" s="2" t="n">
         <v>1.900051506336561</v>
@@ -1418,7 +1418,7 @@
         <v>-1</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>0.9426655583475668</v>
+        <v>0.9426655583063552</v>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
@@ -1453,10 +1453,10 @@
         <v>0</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>56.85456583217909</v>
+        <v>56.85456584897523</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>28.88064089336965</v>
+        <v>28.88064089336964</v>
       </c>
       <c r="J19" s="2" t="n">
         <v>0.5574263773374458</v>
@@ -1471,7 +1471,7 @@
         <v>-1</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>-0.5241005447123657</v>
+        <v>-0.5241005448463012</v>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
@@ -1612,10 +1612,10 @@
         <v>0</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>59.25548276602573</v>
+        <v>59.25548273227194</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>43.21471257502027</v>
+        <v>43.21471263336584</v>
       </c>
       <c r="J22" s="2" t="n">
         <v>0.3757633786134317</v>
@@ -1665,10 +1665,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>60.24061247101406</v>
+        <v>60.24061233449722</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>32.46129824339109</v>
+        <v>32.46129816305995</v>
       </c>
       <c r="J23" s="2" t="n">
         <v>0.4227213686110475</v>
@@ -1683,7 +1683,7 @@
         <v>-1</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>-0.0235976913651807</v>
+        <v>-0.0235976910767011</v>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
@@ -1718,7 +1718,7 @@
         <v>0</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>55.71869865310951</v>
+        <v>55.71869879383271</v>
       </c>
       <c r="I24" s="2" t="n">
         <v>34.43036432738403</v>
@@ -1736,7 +1736,7 @@
         <v>-1</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>0.3004232252137185</v>
+        <v>0.3004232251106888</v>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
@@ -1757,7 +1757,7 @@
         <v/>
       </c>
       <c r="D25" s="2" t="n">
-        <v>721.301953935002</v>
+        <v>721.3019539350013</v>
       </c>
       <c r="E25" s="2" t="n">
         <v>17.1</v>
@@ -1771,10 +1771,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>58.23727334979599</v>
+        <v>58.23727361844024</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>20.84949486189215</v>
+        <v>20.84949482275463</v>
       </c>
       <c r="J25" s="2" t="n">
         <v>0.7712497302890978</v>
@@ -1789,7 +1789,7 @@
         <v>-1</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>0.073358835770576</v>
+        <v>0.0733588355748223</v>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
@@ -1824,10 +1824,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>56.1802951230984</v>
+        <v>56.18029511990134</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>23.9828809924816</v>
+        <v>23.98288102773376</v>
       </c>
       <c r="J26" s="2" t="n">
         <v>0.7751675947090118</v>
@@ -1842,7 +1842,7 @@
         <v>-1</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>0.5530557937483991</v>
+        <v>0.5530557937689955</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
@@ -1863,7 +1863,7 @@
         <v/>
       </c>
       <c r="D27" s="2" t="n">
-        <v>697.0780762559249</v>
+        <v>697.0780762559248</v>
       </c>
       <c r="E27" s="2" t="n">
         <v>902</v>
@@ -1877,10 +1877,10 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>53.0484662994878</v>
+        <v>53.04846634345378</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>25.66360365024904</v>
+        <v>25.66360366329238</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>0.924484638416354</v>
@@ -1895,7 +1895,7 @@
         <v>-1</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>13.43349447356027</v>
+        <v>13.43349447108747</v>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
@@ -1983,10 +1983,10 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>57.1990037271645</v>
+        <v>57.19900437529167</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>7.55405858681615</v>
+        <v>7.554058761184928</v>
       </c>
       <c r="J29" s="2" t="n">
         <v>1.175352918501701</v>
@@ -2001,7 +2001,7 @@
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>0.0029533313620175</v>
+        <v>0.0029533226251539</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
@@ -2089,10 +2089,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>59.12638190250296</v>
+        <v>59.12638182791803</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>32.32609198842916</v>
+        <v>32.32609204662564</v>
       </c>
       <c r="J31" s="2" t="n">
         <v>0.633038859469333</v>
@@ -2107,7 +2107,7 @@
         <v>-1</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>0.2464063844203584</v>
+        <v>0.2464063847294466</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
@@ -2195,10 +2195,10 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>57.41459268925412</v>
+        <v>57.41459267749483</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>24.07478254840484</v>
+        <v>24.07478256314707</v>
       </c>
       <c r="J33" s="2" t="n">
         <v>1.688986979001533</v>
@@ -2213,7 +2213,7 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>0.515568243546727</v>
+        <v>0.5155682437527851</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
@@ -2354,10 +2354,10 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>54.71729516061193</v>
+        <v>54.71729541841169</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>28.86186428107606</v>
+        <v>28.86186423395426</v>
       </c>
       <c r="J36" s="2" t="n">
         <v>1.724578533030149</v>
@@ -2372,7 +2372,7 @@
         <v>-1</v>
       </c>
       <c r="N36" s="2" t="n">
-        <v>0.0566602568849521</v>
+        <v>0.0566602568746477</v>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
@@ -2407,10 +2407,10 @@
         <v>0</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>51.33578612005935</v>
+        <v>51.33578611008162</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>12.98734165509332</v>
+        <v>12.98734172244253</v>
       </c>
       <c r="J37" s="2" t="n">
         <v>2.343203902139264</v>
@@ -2425,7 +2425,7 @@
         <v>-1</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>0.07816491532261161</v>
+        <v>0.0781649154771555</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
@@ -2460,10 +2460,10 @@
         <v>0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>55.64752011282086</v>
+        <v>55.6475201331373</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>26.13648394540312</v>
+        <v>26.13648419642332</v>
       </c>
       <c r="J38" s="2" t="n">
         <v>1.008053368396489</v>
@@ -2478,7 +2478,7 @@
         <v>-1</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>0.1157617499200733</v>
+        <v>0.1157617499138938</v>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
@@ -2513,10 +2513,10 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>55.52770198338013</v>
+        <v>55.52770199042561</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>28.65730532381441</v>
+        <v>28.65730530298572</v>
       </c>
       <c r="J39" s="2" t="n">
         <v>0.3603977157635685</v>
@@ -2531,7 +2531,7 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>0.015157723079723</v>
+        <v>0.0151577232631128</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
@@ -2552,7 +2552,7 @@
         <v/>
       </c>
       <c r="D40" s="2" t="n">
-        <v>620.5436412419903</v>
+        <v>620.5436412419904</v>
       </c>
       <c r="E40" s="2" t="n">
         <v>1480</v>
@@ -2566,10 +2566,10 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>57.33412991657036</v>
+        <v>57.33413021235069</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>15.14866875395824</v>
+        <v>15.14866876138059</v>
       </c>
       <c r="J40" s="2" t="n">
         <v>0.5594201268994868</v>
@@ -2584,7 +2584,7 @@
         <v>-1</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>8.852339556913236</v>
+        <v>8.852339541458914</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
@@ -2619,7 +2619,7 @@
         <v>0</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>55.26940225081938</v>
+        <v>55.26940228631561</v>
       </c>
       <c r="I41" s="2" t="n">
         <v>13.64693905281207</v>
@@ -2637,7 +2637,7 @@
         <v>-1</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>0.225539889210089</v>
+        <v>0.2255398891482647</v>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
@@ -2831,10 +2831,10 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>52.49191152966954</v>
+        <v>52.49191153636426</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>21.01765888184759</v>
+        <v>21.01765887416846</v>
       </c>
       <c r="J45" s="2" t="n">
         <v>1.427502995560037</v>
@@ -2849,7 +2849,7 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>4.283296317078346</v>
+        <v>4.283296316460298</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
@@ -2870,7 +2870,7 @@
         <v/>
       </c>
       <c r="D46" s="2" t="n">
-        <v>589.2614349122488</v>
+        <v>589.2614349122492</v>
       </c>
       <c r="E46" s="2" t="n">
         <v>210</v>
@@ -2884,10 +2884,10 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>49.58953795492244</v>
+        <v>49.58953793864409</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>29.57965461105429</v>
+        <v>29.57965459744048</v>
       </c>
       <c r="J46" s="2" t="n">
         <v>0.4170884081219589</v>
@@ -2902,7 +2902,7 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>-4.661260069645284</v>
+        <v>-4.661260069480432</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
@@ -2937,10 +2937,10 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>60.07097329145326</v>
+        <v>60.07097331856691</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>20.34503097116776</v>
+        <v>20.34503094256065</v>
       </c>
       <c r="J47" s="2" t="n">
         <v>0.7550994623976465</v>
@@ -2955,7 +2955,7 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>2.049381678915836</v>
+        <v>2.049381678936451</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
@@ -2990,10 +2990,10 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>55.06256603479149</v>
+        <v>55.06280084247292</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>23.90759839088992</v>
+        <v>23.9076268618504</v>
       </c>
       <c r="J48" s="2" t="n">
         <v>0.750864911342356</v>
@@ -3008,7 +3008,7 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>-0.0408812519339094</v>
+        <v>-0.0408813491355607</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
@@ -3029,7 +3029,7 @@
         <v/>
       </c>
       <c r="D49" s="2" t="n">
-        <v>584.1966092945155</v>
+        <v>584.1966092945154</v>
       </c>
       <c r="E49" s="2" t="n">
         <v>463.5</v>
@@ -3043,10 +3043,10 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>48.61308083225934</v>
+        <v>48.61308083468805</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>11.59221439043382</v>
+        <v>11.59221451969522</v>
       </c>
       <c r="J49" s="2" t="n">
         <v>0.6497432162926046</v>
@@ -3061,7 +3061,7 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>-1.748505495594372</v>
+        <v>-1.748505497242898</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
@@ -3096,10 +3096,10 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>50.73592954388249</v>
+        <v>50.73592956563075</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>11.79802131706726</v>
+        <v>11.79802123688644</v>
       </c>
       <c r="J50" s="2" t="n">
         <v>0.341584082054018</v>
@@ -3114,7 +3114,7 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>-1.291579766227941</v>
+        <v>-1.291579766372162</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
@@ -3149,10 +3149,10 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>55.13875102721872</v>
+        <v>55.13875107210337</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>15.30581997705723</v>
+        <v>15.30582006085913</v>
       </c>
       <c r="J51" s="2" t="n">
         <v>0.4078870463424215</v>
@@ -3167,7 +3167,7 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>0.3612574150233349</v>
+        <v>0.3612574144050566</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
@@ -3202,10 +3202,10 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>54.47809578309266</v>
+        <v>54.47809592828287</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>12.46267680254679</v>
+        <v>12.46267683841879</v>
       </c>
       <c r="J52" s="2" t="n">
         <v>0.762192779135218</v>
@@ -3220,7 +3220,7 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>0.5096997680840337</v>
+        <v>0.5096997669507117</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
@@ -3258,7 +3258,7 @@
         <v>45.13442208869636</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>24.06717990361534</v>
+        <v>24.06717991221974</v>
       </c>
       <c r="J53" s="2" t="n">
         <v>0.3463453637564813</v>
@@ -3273,7 +3273,7 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>-2.038392700994547</v>
+        <v>-2.038392700984244</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
@@ -3294,7 +3294,7 @@
         <v/>
       </c>
       <c r="D54" s="2" t="n">
-        <v>556.2168763771105</v>
+        <v>556.2168763771126</v>
       </c>
       <c r="E54" s="2" t="n">
         <v>102.5</v>
@@ -3308,10 +3308,10 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>54.57857268202815</v>
+        <v>54.57857272155708</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>16.07075122321314</v>
+        <v>16.07075121060834</v>
       </c>
       <c r="J54" s="2" t="n">
         <v>1.15369639066315</v>
@@ -3326,7 +3326,7 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>1.055889345398644</v>
+        <v>1.055889345192573</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
@@ -3347,7 +3347,7 @@
         <v/>
       </c>
       <c r="D55" s="2" t="n">
-        <v>550.3503279119444</v>
+        <v>550.3503279119417</v>
       </c>
       <c r="E55" s="2" t="n">
         <v>6.8</v>
@@ -3361,10 +3361,10 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>64.83836030792037</v>
+        <v>64.8383600781322</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>26.21684416848806</v>
+        <v>26.21684433472234</v>
       </c>
       <c r="J55" s="2" t="n">
         <v>0.3673747869994226</v>
@@ -3379,7 +3379,7 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>0.07455675238018469</v>
+        <v>0.0745567524626083</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
@@ -3520,10 +3520,10 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>51.59429855760303</v>
+        <v>51.59429828885338</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>21.10364876105432</v>
+        <v>21.10364887817052</v>
       </c>
       <c r="J58" s="2" t="n">
         <v>0.7355786857594313</v>
@@ -3538,7 +3538,7 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>0.6615066183231602</v>
+        <v>0.6615066193534476</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
@@ -3559,7 +3559,7 @@
         <v/>
       </c>
       <c r="D59" s="2" t="n">
-        <v>541.6340817463193</v>
+        <v>541.6340817463197</v>
       </c>
       <c r="E59" s="2" t="n">
         <v>30.55</v>
@@ -3573,10 +3573,10 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>67.00871058632652</v>
+        <v>67.00871057113899</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>36.64823071891905</v>
+        <v>36.6482307325699</v>
       </c>
       <c r="J59" s="2" t="n">
         <v>0.6654071906683129</v>
@@ -3591,7 +3591,7 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>0.4353146937764984</v>
+        <v>0.4353146938589225</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
@@ -3626,10 +3626,10 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>63.45404211340973</v>
+        <v>63.45404211561035</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>18.3549154130111</v>
+        <v>18.35491539898681</v>
       </c>
       <c r="J60" s="2" t="n">
         <v>2.435090728538716</v>
@@ -3644,7 +3644,7 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>8.140550645885103</v>
+        <v>8.140550645843872</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
@@ -3665,7 +3665,7 @@
         <v/>
       </c>
       <c r="D61" s="2" t="n">
-        <v>533.8456678496028</v>
+        <v>533.8456678496029</v>
       </c>
       <c r="E61" s="2" t="n">
         <v>47.7</v>
@@ -3679,10 +3679,10 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>52.65024456085442</v>
+        <v>52.6502445649905</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>37.98861698439374</v>
+        <v>37.98861699141846</v>
       </c>
       <c r="J61" s="2" t="n">
         <v>0.6363499694301362</v>
@@ -3697,7 +3697,7 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>0.0253317368514731</v>
+        <v>0.0253317371605628</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
@@ -3718,7 +3718,7 @@
         <v/>
       </c>
       <c r="D62" s="2" t="n">
-        <v>530.2710476647961</v>
+        <v>530.2710476647962</v>
       </c>
       <c r="E62" s="2" t="n">
         <v>81.3</v>
@@ -3732,10 +3732,10 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>49.85590000712904</v>
+        <v>49.85590003709532</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>22.34724885163773</v>
+        <v>22.34724899464389</v>
       </c>
       <c r="J62" s="2" t="n">
         <v>0.2074546541020147</v>
@@ -3750,7 +3750,7 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>-0.4276252855318279</v>
+        <v>-0.4276252859542495</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
@@ -3824,7 +3824,7 @@
         <v/>
       </c>
       <c r="D64" s="2" t="n">
-        <v>526.2852605939221</v>
+        <v>526.2852605939219</v>
       </c>
       <c r="E64" s="2" t="n">
         <v>35.75</v>
@@ -3838,10 +3838,10 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>57.3983669588407</v>
+        <v>57.39836707844272</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>15.37385439237246</v>
+        <v>15.37385442342875</v>
       </c>
       <c r="J64" s="2" t="n">
         <v>0.4348291059323704</v>
@@ -3856,7 +3856,7 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>0.0933798414099254</v>
+        <v>0.0933798411935563</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
@@ -3891,7 +3891,7 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>64.54768696378756</v>
+        <v>64.54768698578494</v>
       </c>
       <c r="I65" s="2" t="n">
         <v>46.63107663782352</v>
@@ -3909,7 +3909,7 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>0.4241454768185426</v>
+        <v>0.4241454767979362</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
@@ -3983,7 +3983,7 @@
         <v/>
       </c>
       <c r="D67" s="2" t="n">
-        <v>514.9166908642846</v>
+        <v>514.9166908642867</v>
       </c>
       <c r="E67" s="2" t="n">
         <v>53.8</v>
@@ -3997,10 +3997,10 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>58.06174289798737</v>
+        <v>58.06174280922479</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>17.91995889632582</v>
+        <v>17.91995892139922</v>
       </c>
       <c r="J67" s="2" t="n">
         <v>1.922717119556777</v>
@@ -4015,7 +4015,7 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>0.4210570696020772</v>
+        <v>0.4210570697772331</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
@@ -4036,7 +4036,7 @@
         <v/>
       </c>
       <c r="D68" s="2" t="n">
-        <v>510.4372580088996</v>
+        <v>510.4372580088977</v>
       </c>
       <c r="E68" s="2" t="n">
         <v>33.1</v>
@@ -4050,10 +4050,10 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>52.71967607593986</v>
+        <v>52.71967601759888</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>23.1746240732888</v>
+        <v>23.17462412508665</v>
       </c>
       <c r="J68" s="2" t="n">
         <v>0.8214927973946836</v>
@@ -4068,7 +4068,7 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>0.1729641310155732</v>
+        <v>0.1729641312010237</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
@@ -4156,10 +4156,10 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>49.30065410695722</v>
+        <v>49.30065411006407</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>16.96709112784468</v>
+        <v>16.96709123618953</v>
       </c>
       <c r="J70" s="2" t="n">
         <v>1.224237450039564</v>
@@ -4174,7 +4174,7 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>-3.061603166502733</v>
+        <v>-3.061603167223822</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
@@ -4195,7 +4195,7 @@
         <v/>
       </c>
       <c r="D71" s="2" t="n">
-        <v>497.6371209997965</v>
+        <v>497.637120999797</v>
       </c>
       <c r="E71" s="2" t="n">
         <v>161</v>
@@ -4209,10 +4209,10 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>57.06483636362429</v>
+        <v>57.06483641132107</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>16.70906595090583</v>
+        <v>16.70906594739693</v>
       </c>
       <c r="J71" s="2" t="n">
         <v>0.6461843287725012</v>
@@ -4227,7 +4227,7 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>1.416010566680472</v>
+        <v>1.416010567092575</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
@@ -4301,7 +4301,7 @@
         <v/>
       </c>
       <c r="D73" s="2" t="n">
-        <v>494.8347184156829</v>
+        <v>494.8347184156828</v>
       </c>
       <c r="E73" s="2" t="n">
         <v>241.5</v>
@@ -4315,10 +4315,10 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>50.03733805391082</v>
+        <v>50.03733812933626</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>10.49060096230486</v>
+        <v>10.49060099929592</v>
       </c>
       <c r="J73" s="2" t="n">
         <v>0.2961244768753559</v>
@@ -4333,7 +4333,7 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>-0.703048432814261</v>
+        <v>-0.7030484341536392</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
@@ -4368,10 +4368,10 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>51.42485766484158</v>
+        <v>51.42485767734271</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>14.70725414522032</v>
+        <v>14.70725415692002</v>
       </c>
       <c r="J74" s="2" t="n">
         <v>0.4607548756613981</v>
@@ -4386,7 +4386,7 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>-1.228537451383385</v>
+        <v>-1.228537451671821</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
@@ -4580,10 +4580,10 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>48.87066503859311</v>
+        <v>48.87066510864693</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>12.82904556315741</v>
+        <v>12.82904562824002</v>
       </c>
       <c r="J78" s="2" t="n">
         <v>0.4844811293213995</v>
@@ -4598,7 +4598,7 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>0.1231530834204697</v>
+        <v>0.1231530833174412</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
@@ -4633,10 +4633,10 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>53.48501870095393</v>
+        <v>53.48501873500918</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>19.14013541368204</v>
+        <v>19.14013540553784</v>
       </c>
       <c r="J79" s="2" t="n">
         <v>0.5610376053204557</v>
@@ -4651,7 +4651,7 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>0.0240572879040506</v>
+        <v>0.0240572879246563</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
@@ -4672,7 +4672,7 @@
         <v/>
       </c>
       <c r="D80" s="2" t="n">
-        <v>475.5808675097707</v>
+        <v>475.5808675097709</v>
       </c>
       <c r="E80" s="2" t="n">
         <v>28.15</v>
@@ -4686,10 +4686,10 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>55.8996993676279</v>
+        <v>55.8996994434099</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>17.22470341649186</v>
+        <v>17.22470341385504</v>
       </c>
       <c r="J80" s="2" t="n">
         <v>0.3912776788159589</v>
@@ -4704,7 +4704,7 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>0.0685502767562544</v>
+        <v>0.0685502767768592</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
@@ -4951,10 +4951,10 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>54.42779453405551</v>
+        <v>54.42779459324473</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>15.55350517739935</v>
+        <v>15.55350517739934</v>
       </c>
       <c r="J85" s="2" t="n">
         <v>0.5419367886459436</v>
@@ -4969,7 +4969,7 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>0.1010957028045307</v>
+        <v>0.1010957025160541</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
@@ -5043,7 +5043,7 @@
         <v/>
       </c>
       <c r="D87" s="2" t="n">
-        <v>450.5197753210263</v>
+        <v>450.5197753210264</v>
       </c>
       <c r="E87" s="2" t="n">
         <v>54.8</v>
@@ -5057,10 +5057,10 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>56.6362049937689</v>
+        <v>56.63620498156541</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>22.69777143884325</v>
+        <v>22.69777143551548</v>
       </c>
       <c r="J87" s="2" t="n">
         <v>0.3681377020742047</v>
@@ -5075,7 +5075,7 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>0.2889941161775033</v>
+        <v>0.2889941163217426</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
@@ -5110,7 +5110,7 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>55.7086475778691</v>
+        <v>55.70864762472478</v>
       </c>
       <c r="I88" s="2" t="n">
         <v>35.21177968310418</v>
@@ -5128,7 +5128,7 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>1.307159016757416</v>
+        <v>1.307159016571963</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
@@ -5216,10 +5216,10 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>51.82367314476449</v>
+        <v>51.82367315202875</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>14.42359348939137</v>
+        <v>14.42359350109984</v>
       </c>
       <c r="J90" s="2" t="n">
         <v>0.2528404416509401</v>
@@ -5234,7 +5234,7 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>0.7352893226111732</v>
+        <v>0.7352893225288173</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
@@ -5269,10 +5269,10 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>42.35987115400469</v>
+        <v>42.35987114673463</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>14.73369941117633</v>
+        <v>14.73369941878737</v>
       </c>
       <c r="J91" s="2" t="n">
         <v>0.3103877663808355</v>
@@ -5287,7 +5287,7 @@
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>-0.8507525362436718</v>
+        <v>-0.8507525362745824</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
@@ -5308,7 +5308,7 @@
         <v/>
       </c>
       <c r="D92" s="2" t="n">
-        <v>441.7987579325161</v>
+        <v>441.7987579325157</v>
       </c>
       <c r="E92" s="2" t="n">
         <v>134</v>
@@ -5322,10 +5322,10 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>35.37067918903936</v>
+        <v>35.37067918106091</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>21.41567499410607</v>
+        <v>21.41567497769285</v>
       </c>
       <c r="J92" s="2" t="n">
         <v>0.6691616474275163</v>
@@ -5340,7 +5340,7 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>-0.8061002036184841</v>
+        <v>-0.806100203484529</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
@@ -5375,10 +5375,10 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>48.31167140625287</v>
+        <v>48.31167145927478</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>12.07117849064237</v>
+        <v>12.07117852681991</v>
       </c>
       <c r="J93" s="2" t="n">
         <v>0.311668630730234</v>
@@ -5393,7 +5393,7 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>-0.183306254904827</v>
+        <v>-0.183306254873925</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
@@ -5414,7 +5414,7 @@
         <v/>
       </c>
       <c r="D94" s="2" t="n">
-        <v>439.1632845985746</v>
+        <v>438.8165305790616</v>
       </c>
       <c r="E94" s="2" t="n">
         <v>76.09999999999999</v>
@@ -5428,7 +5428,7 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>67.50014790802021</v>
+        <v>63.57393396612694</v>
       </c>
       <c r="I94" s="2" t="n">
         <v/>
@@ -5446,7 +5446,7 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>0.5444018905409821</v>
+        <v>0.5985881897404215</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
@@ -5481,10 +5481,10 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>54.49649336954818</v>
+        <v>54.49649333085536</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>28.07253018447487</v>
+        <v>28.07253021830984</v>
       </c>
       <c r="J95" s="2" t="n">
         <v>0.1578218670790724</v>
@@ -5499,7 +5499,7 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>-1.326975405632483</v>
+        <v>-1.326975405014299</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
@@ -5626,7 +5626,7 @@
         <v/>
       </c>
       <c r="D98" s="2" t="n">
-        <v>426.0976663928128</v>
+        <v>426.097666392813</v>
       </c>
       <c r="E98" s="2" t="n">
         <v>107</v>
@@ -5640,10 +5640,10 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>49.91272109790702</v>
+        <v>49.91272105201376</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>19.13552210720557</v>
+        <v>19.13552208124386</v>
       </c>
       <c r="J98" s="2" t="n">
         <v>0.3493912695618686</v>
@@ -5658,7 +5658,7 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>-0.4985609657160809</v>
+        <v>-0.4985609652627495</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
@@ -5679,7 +5679,7 @@
         <v/>
       </c>
       <c r="D99" s="2" t="n">
-        <v>421.7600911239397</v>
+        <v>421.7600911239399</v>
       </c>
       <c r="E99" s="2" t="n">
         <v>552</v>
@@ -5693,10 +5693,10 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>48.65159826088248</v>
+        <v>48.65159827403787</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>14.70089382823801</v>
+        <v>14.70089391121134</v>
       </c>
       <c r="J99" s="2" t="n">
         <v>0.2614699995193363</v>
@@ -5711,7 +5711,7 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>-8.114497111069078</v>
+        <v>-8.11449711261448</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
@@ -5749,7 +5749,7 @@
         <v>54.70315064810057</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>16.13958151498428</v>
+        <v>16.13958149639615</v>
       </c>
       <c r="J100" s="2" t="n">
         <v>0.7716183243851067</v>
@@ -5764,7 +5764,7 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>0.4669909804725524</v>
+        <v>0.4669909805755881</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
@@ -5799,10 +5799,10 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>42.43346557016634</v>
+        <v>42.43346557667848</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>19.3488053411203</v>
+        <v>19.34880537729646</v>
       </c>
       <c r="J101" s="2" t="n">
         <v>0.6877835569447788</v>
@@ -5817,7 +5817,7 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>0.8485790673117464</v>
+        <v>0.8485790674147111</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
@@ -5852,10 +5852,10 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>47.09807985935856</v>
+        <v>47.09807987359476</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>24.99625970981491</v>
+        <v>24.99625974063477</v>
       </c>
       <c r="J102" s="2" t="n">
         <v>0.2146765541512863</v>
@@ -5870,7 +5870,7 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>-1.361256171004777</v>
+        <v>-1.361256171015074</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
@@ -5944,7 +5944,7 @@
         <v/>
       </c>
       <c r="D104" s="2" t="n">
-        <v>409.8033331801762</v>
+        <v>409.8033331801764</v>
       </c>
       <c r="E104" s="2" t="n">
         <v>14.15</v>
@@ -5958,10 +5958,10 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>50.89518454991226</v>
+        <v>50.89518450574337</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>26.79888456975429</v>
+        <v>26.79888456957421</v>
       </c>
       <c r="J104" s="2" t="n">
         <v>0.7905800466810933</v>
@@ -5976,7 +5976,7 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>0.1284416565856791</v>
+        <v>0.1284416566062848</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
@@ -6011,10 +6011,10 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>53.90066085573824</v>
+        <v>53.90066090156466</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>13.30469704959544</v>
+        <v>13.30469706478908</v>
       </c>
       <c r="J105" s="2" t="n">
         <v>0.8749879158732514</v>
@@ -6029,7 +6029,7 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>-0.1132983552922267</v>
+        <v>-0.1132983551685959</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
@@ -6064,10 +6064,10 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>50.84064981595174</v>
+        <v>50.84064985175647</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>13.40001720772202</v>
+        <v>13.40001722125442</v>
       </c>
       <c r="J106" s="2" t="n">
         <v>0.3726067530590306</v>
@@ -6082,7 +6082,7 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>0.0742691953579499</v>
+        <v>0.0742691939155555</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
@@ -6117,10 +6117,10 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>52.63667443676913</v>
+        <v>52.63667446777631</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>38.08941630466538</v>
+        <v>38.08941630040196</v>
       </c>
       <c r="J107" s="2" t="n">
         <v>0.3110684350557122</v>
@@ -6170,10 +6170,10 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>42.24809651097526</v>
+        <v>42.24809660376557</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>20.86450076914899</v>
+        <v>20.8645008136155</v>
       </c>
       <c r="J108" s="2" t="n">
         <v>0.6842898113909404</v>
@@ -6188,7 +6188,7 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>-0.1794007328506701</v>
+        <v>-0.1794007369717665</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
@@ -6226,7 +6226,7 @@
         <v>36.54270952727176</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>41.5202544053362</v>
+        <v>41.52025445807829</v>
       </c>
       <c r="J109" s="2" t="n">
         <v>0.1747383264792246</v>
@@ -6276,10 +6276,10 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>40.9458114396516</v>
+        <v>40.94581150039469</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>30.6150876867214</v>
+        <v>30.61508773061949</v>
       </c>
       <c r="J110" s="2" t="n">
         <v>0.4815845842733804</v>
@@ -6329,10 +6329,10 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>49.35164432755892</v>
+        <v>49.35164433419458</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>28.07364200242681</v>
+        <v>28.07364195575056</v>
       </c>
       <c r="J111" s="2" t="n">
         <v>0.1788642376827209</v>
@@ -6347,7 +6347,7 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>-0.4989466098230368</v>
+        <v>-0.4989466093594099</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
@@ -6435,10 +6435,10 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>47.21445772747118</v>
+        <v>47.21445761103659</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>13.56801720093325</v>
+        <v>13.56801736096864</v>
       </c>
       <c r="J113" s="2" t="n">
         <v>0.2810921294203762</v>
@@ -6453,7 +6453,7 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>-0.0560631453216839</v>
+        <v>-0.056063145115623</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
@@ -6488,10 +6488,10 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>44.93646308223838</v>
+        <v>44.9364619141345</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>11.40975289410236</v>
+        <v>11.40975239412487</v>
       </c>
       <c r="J114" s="2" t="n">
         <v>0.3498173980722026</v>
@@ -6506,7 +6506,7 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>0.1067815035370479</v>
+        <v>0.106781507163673</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
@@ -6527,7 +6527,7 @@
         <v/>
       </c>
       <c r="D115" s="2" t="n">
-        <v>377.4037210051063</v>
+        <v>377.4037210051055</v>
       </c>
       <c r="E115" s="2" t="n">
         <v>168.5</v>
@@ -6541,7 +6541,7 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>51.07901750427845</v>
+        <v>51.07901753159067</v>
       </c>
       <c r="I115" s="2" t="n">
         <v>20.27325832830773</v>
@@ -6559,7 +6559,7 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>-1.551407385573853</v>
+        <v>-1.551407385697517</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
@@ -6594,10 +6594,10 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>38.82622993258804</v>
+        <v>38.82622998673164</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>19.87951539967662</v>
+        <v>19.87951544963975</v>
       </c>
       <c r="J116" s="2" t="n">
         <v>0.4480145761155067</v>
@@ -6647,10 +6647,10 @@
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>49.059970829028</v>
+        <v>49.05997137979319</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>19.84838971988606</v>
+        <v>19.84838980169912</v>
       </c>
       <c r="J117" s="2" t="n">
         <v>0.1790799411206339</v>
@@ -6665,7 +6665,7 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>-0.1002586669852813</v>
+        <v>-0.1002586673772798</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
@@ -6686,7 +6686,7 @@
         <v/>
       </c>
       <c r="D118" s="2" t="n">
-        <v>374.5695599834368</v>
+        <v>374.5695599834369</v>
       </c>
       <c r="E118" s="2" t="n">
         <v>35.2</v>
@@ -6700,10 +6700,10 @@
         <v>0</v>
       </c>
       <c r="H118" s="2" t="n">
-        <v>43.5024843199455</v>
+        <v>43.50248428887807</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>27.7417370232545</v>
+        <v>27.74173703966152</v>
       </c>
       <c r="J118" s="2" t="n">
         <v>0.200119664830243</v>
@@ -6718,7 +6718,7 @@
         <v>-1</v>
       </c>
       <c r="N118" s="2" t="n">
-        <v>-0.2091529011495917</v>
+        <v>-0.2091529009229275</v>
       </c>
       <c r="O118" s="2" t="inlineStr">
         <is>
@@ -6753,10 +6753,10 @@
         <v>0</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>52.69302409881968</v>
+        <v>52.69302413070555</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>14.35700262227653</v>
+        <v>14.35700264821923</v>
       </c>
       <c r="J119" s="2" t="n">
         <v>0.6713134887657505</v>
@@ -6771,7 +6771,7 @@
         <v>-1</v>
       </c>
       <c r="N119" s="2" t="n">
-        <v>0.0394930893110192</v>
+        <v>0.0394930892904135</v>
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
@@ -6806,10 +6806,10 @@
         <v>0</v>
       </c>
       <c r="H120" s="2" t="n">
-        <v>35.48908699208265</v>
+        <v>35.48908700056226</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>17.16284906316569</v>
+        <v>17.16284904848618</v>
       </c>
       <c r="J120" s="2" t="n">
         <v>0.6216553896099903</v>
@@ -6824,7 +6824,7 @@
         <v>-1</v>
       </c>
       <c r="N120" s="2" t="n">
-        <v>-0.325325642679676</v>
+        <v>-0.3253256426590702</v>
       </c>
       <c r="O120" s="2" t="inlineStr">
         <is>
@@ -6898,7 +6898,7 @@
         <v/>
       </c>
       <c r="D122" s="2" t="n">
-        <v>366.7380509514761</v>
+        <v>366.7380509514766</v>
       </c>
       <c r="E122" s="2" t="n">
         <v>12.75</v>
@@ -6912,10 +6912,10 @@
         <v>0</v>
       </c>
       <c r="H122" s="2" t="n">
-        <v>54.08166252646294</v>
+        <v>54.0816625059113</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>21.66531700664019</v>
+        <v>21.66531706308997</v>
       </c>
       <c r="J122" s="2" t="n">
         <v>0.7465067496436718</v>
@@ -6930,7 +6930,7 @@
         <v>-1</v>
       </c>
       <c r="N122" s="2" t="n">
-        <v>0.1146389211591637</v>
+        <v>0.1146389212121365</v>
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
@@ -6965,10 +6965,10 @@
         <v>0</v>
       </c>
       <c r="H123" s="2" t="n">
-        <v>44.65261079935557</v>
+        <v>44.65261067112694</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>8.824914191020772</v>
+        <v>8.824914331750067</v>
       </c>
       <c r="J123" s="2" t="n">
         <v>0.4309676316319739</v>
@@ -6983,7 +6983,7 @@
         <v>-1</v>
       </c>
       <c r="N123" s="2" t="n">
-        <v>-0.0376735089648747</v>
+        <v>-0.0376735087073021</v>
       </c>
       <c r="O123" s="2" t="inlineStr">
         <is>
@@ -7004,7 +7004,7 @@
         <v/>
       </c>
       <c r="D124" s="2" t="n">
-        <v>362.3006010653235</v>
+        <v>362.3006010653233</v>
       </c>
       <c r="E124" s="2" t="n">
         <v>73</v>
@@ -7018,10 +7018,10 @@
         <v>0</v>
       </c>
       <c r="H124" s="2" t="n">
-        <v>50.66027037542064</v>
+        <v>50.66027050813302</v>
       </c>
       <c r="I124" s="2" t="n">
-        <v>12.40789829633828</v>
+        <v>12.40789837150023</v>
       </c>
       <c r="J124" s="2" t="n">
         <v>0.4593774800495414</v>
@@ -7036,7 +7036,7 @@
         <v>-1</v>
       </c>
       <c r="N124" s="2" t="n">
-        <v>0.1148062033537681</v>
+        <v>0.1148062030446774</v>
       </c>
       <c r="O124" s="2" t="inlineStr">
         <is>
@@ -7057,7 +7057,7 @@
         <v/>
       </c>
       <c r="D125" s="2" t="n">
-        <v>359.928946019946</v>
+        <v>359.9289460199461</v>
       </c>
       <c r="E125" s="2" t="n">
         <v>89.09999999999999</v>
@@ -7071,10 +7071,10 @@
         <v>0</v>
       </c>
       <c r="H125" s="2" t="n">
-        <v>49.16766023121527</v>
+        <v>49.16766022517653</v>
       </c>
       <c r="I125" s="2" t="n">
-        <v>8.887865250236686</v>
+        <v>8.887865261556751</v>
       </c>
       <c r="J125" s="2" t="n">
         <v>0.5836001186386491</v>
@@ -7089,7 +7089,7 @@
         <v>-1</v>
       </c>
       <c r="N125" s="2" t="n">
-        <v>-0.1216337554923439</v>
+        <v>-0.1216337553068931</v>
       </c>
       <c r="O125" s="2" t="inlineStr">
         <is>
@@ -7110,7 +7110,7 @@
         <v/>
       </c>
       <c r="D126" s="2" t="n">
-        <v>355.1004099863981</v>
+        <v>355.1004099863991</v>
       </c>
       <c r="E126" s="2" t="n">
         <v>22.45</v>
@@ -7124,10 +7124,10 @@
         <v>0</v>
       </c>
       <c r="H126" s="2" t="n">
-        <v>56.2566616253173</v>
+        <v>56.25666164329371</v>
       </c>
       <c r="I126" s="2" t="n">
-        <v>19.69539302594258</v>
+        <v>19.69539300564676</v>
       </c>
       <c r="J126" s="2" t="n">
         <v>0.7431898094856607</v>
@@ -7142,7 +7142,7 @@
         <v>-1</v>
       </c>
       <c r="N126" s="2" t="n">
-        <v>0.3002929920333149</v>
+        <v>0.3002929920436163</v>
       </c>
       <c r="O126" s="2" t="inlineStr">
         <is>
@@ -7177,10 +7177,10 @@
         <v>0</v>
       </c>
       <c r="H127" s="2" t="n">
-        <v>50.38079189977495</v>
+        <v>50.3807919105456</v>
       </c>
       <c r="I127" s="2" t="n">
-        <v>15.05223290992262</v>
+        <v>15.05223293271061</v>
       </c>
       <c r="J127" s="2" t="n">
         <v>0.2757648843765496</v>
@@ -7195,7 +7195,7 @@
         <v>-1</v>
       </c>
       <c r="N127" s="2" t="n">
-        <v>-0.273983819135411</v>
+        <v>-0.2739838191251047</v>
       </c>
       <c r="O127" s="2" t="inlineStr">
         <is>
@@ -7216,7 +7216,7 @@
         <v/>
       </c>
       <c r="D128" s="2" t="n">
-        <v>342.3844781090697</v>
+        <v>342.3844781090693</v>
       </c>
       <c r="E128" s="2" t="n">
         <v>18.8</v>
@@ -7230,7 +7230,7 @@
         <v>0</v>
       </c>
       <c r="H128" s="2" t="n">
-        <v>48.36076234688368</v>
+        <v>48.36076267934536</v>
       </c>
       <c r="I128" s="2" t="n">
         <v>15.64894933771602</v>
@@ -7248,7 +7248,7 @@
         <v>-1</v>
       </c>
       <c r="N128" s="2" t="n">
-        <v>0.07721418634574639</v>
+        <v>0.0772141860881724</v>
       </c>
       <c r="O128" s="2" t="inlineStr">
         <is>
@@ -7283,10 +7283,10 @@
         <v>0</v>
       </c>
       <c r="H129" s="2" t="n">
-        <v>54.02314296321296</v>
+        <v>54.02314297851248</v>
       </c>
       <c r="I129" s="2" t="n">
-        <v>15.68052880164562</v>
+        <v>15.68052882251902</v>
       </c>
       <c r="J129" s="2" t="n">
         <v>1.249709820880819</v>
@@ -7336,10 +7336,10 @@
         <v>0</v>
       </c>
       <c r="H130" s="2" t="n">
-        <v>45.01857687006528</v>
+        <v>45.01857701141954</v>
       </c>
       <c r="I130" s="2" t="n">
-        <v>11.87660470155189</v>
+        <v>11.87660472977026</v>
       </c>
       <c r="J130" s="2" t="n">
         <v>0.2804059971007694</v>
@@ -7354,7 +7354,7 @@
         <v>-1</v>
       </c>
       <c r="N130" s="2" t="n">
-        <v>0.1586922184149628</v>
+        <v>0.1586922173846652</v>
       </c>
       <c r="O130" s="2" t="inlineStr">
         <is>
@@ -7548,10 +7548,10 @@
         <v>0</v>
       </c>
       <c r="H134" s="2" t="n">
-        <v>47.64242968364371</v>
+        <v>47.64242969575523</v>
       </c>
       <c r="I134" s="2" t="n">
-        <v>12.91445381979274</v>
+        <v>12.91445383966534</v>
       </c>
       <c r="J134" s="2" t="n">
         <v>0.6201343432672642</v>
@@ -7566,7 +7566,7 @@
         <v>-1</v>
       </c>
       <c r="N134" s="2" t="n">
-        <v>-0.9080151786185456</v>
+        <v>-0.9080151785876424</v>
       </c>
       <c r="O134" s="2" t="inlineStr">
         <is>
@@ -7601,10 +7601,10 @@
         <v>0</v>
       </c>
       <c r="H135" s="2" t="n">
-        <v>52.31799469726688</v>
+        <v>52.31799467041767</v>
       </c>
       <c r="I135" s="2" t="n">
-        <v>16.89519620174653</v>
+        <v>16.89519652908161</v>
       </c>
       <c r="J135" s="2" t="n">
         <v>0.7724967168761327</v>
@@ -7619,7 +7619,7 @@
         <v>-1</v>
       </c>
       <c r="N135" s="2" t="n">
-        <v>4.615995424531931</v>
+        <v>4.615995431537876</v>
       </c>
       <c r="O135" s="2" t="inlineStr">
         <is>
@@ -7654,7 +7654,7 @@
         <v>0</v>
       </c>
       <c r="H136" s="2" t="n">
-        <v>49.8707528919547</v>
+        <v>49.8707529117172</v>
       </c>
       <c r="I136" s="2" t="n">
         <v>11.14911214174636</v>
@@ -7672,7 +7672,7 @@
         <v>-1</v>
       </c>
       <c r="N136" s="2" t="n">
-        <v>-0.0316748751475708</v>
+        <v>-0.0316748751990852</v>
       </c>
       <c r="O136" s="2" t="inlineStr">
         <is>
@@ -7693,7 +7693,7 @@
         <v/>
       </c>
       <c r="D137" s="2" t="n">
-        <v>331.8525769142522</v>
+        <v>331.8525769142521</v>
       </c>
       <c r="E137" s="2" t="n">
         <v>53.3</v>
@@ -7707,10 +7707,10 @@
         <v>0</v>
       </c>
       <c r="H137" s="2" t="n">
-        <v>49.11342259927697</v>
+        <v>49.11342267105825</v>
       </c>
       <c r="I137" s="2" t="n">
-        <v>19.29095252491589</v>
+        <v>19.29095251795042</v>
       </c>
       <c r="J137" s="2" t="n">
         <v>0.4986831378942747</v>
@@ -7725,7 +7725,7 @@
         <v>-1</v>
       </c>
       <c r="N137" s="2" t="n">
-        <v>0.2972900972454663</v>
+        <v>0.2972900971630422</v>
       </c>
       <c r="O137" s="2" t="inlineStr">
         <is>
@@ -7799,7 +7799,7 @@
         <v/>
       </c>
       <c r="D139" s="2" t="n">
-        <v>328.7963069294382</v>
+        <v>328.7963069294381</v>
       </c>
       <c r="E139" s="2" t="n">
         <v>28.25</v>
@@ -7813,10 +7813,10 @@
         <v>0</v>
       </c>
       <c r="H139" s="2" t="n">
-        <v>38.96062455407867</v>
+        <v>38.96062482781012</v>
       </c>
       <c r="I139" s="2" t="n">
-        <v>14.56126855376331</v>
+        <v>14.56126857127882</v>
       </c>
       <c r="J139" s="2" t="n">
         <v>0.3050216295249408</v>
@@ -7831,7 +7831,7 @@
         <v>-1</v>
       </c>
       <c r="N139" s="2" t="n">
-        <v>0.0160174296318085</v>
+        <v>0.0160174296524124</v>
       </c>
       <c r="O139" s="2" t="inlineStr">
         <is>
@@ -8025,10 +8025,10 @@
         <v>0</v>
       </c>
       <c r="H143" s="2" t="n">
-        <v>32.78298276564745</v>
+        <v>32.78298279450875</v>
       </c>
       <c r="I143" s="2" t="n">
-        <v>40.92715194414077</v>
+        <v>40.92715197733646</v>
       </c>
       <c r="J143" s="2" t="n">
         <v>0.2928281927313216</v>
@@ -8043,7 +8043,7 @@
         <v>-1</v>
       </c>
       <c r="N143" s="2" t="n">
-        <v>0.0287051293574839</v>
+        <v>0.028705129347176</v>
       </c>
       <c r="O143" s="2" t="inlineStr">
         <is>
@@ -8184,10 +8184,10 @@
         <v>0</v>
       </c>
       <c r="H146" s="2" t="n">
-        <v>48.17770302250919</v>
+        <v>48.17770309841374</v>
       </c>
       <c r="I146" s="2" t="n">
-        <v>20.68501278496717</v>
+        <v>20.68501280779751</v>
       </c>
       <c r="J146" s="2" t="n">
         <v>0.6050939752277208</v>
@@ -8202,7 +8202,7 @@
         <v>-1</v>
       </c>
       <c r="N146" s="2" t="n">
-        <v>0.7896431988363362</v>
+        <v>0.7896431989393569</v>
       </c>
       <c r="O146" s="2" t="inlineStr">
         <is>
@@ -8223,7 +8223,7 @@
         <v/>
       </c>
       <c r="D147" s="2" t="n">
-        <v>311.2387436631762</v>
+        <v>311.2387436631761</v>
       </c>
       <c r="E147" s="2" t="n">
         <v>70.5</v>
@@ -8237,10 +8237,10 @@
         <v>0</v>
       </c>
       <c r="H147" s="2" t="n">
-        <v>49.61773714520052</v>
+        <v>49.61773696468212</v>
       </c>
       <c r="I147" s="2" t="n">
-        <v>21.30566605802777</v>
+        <v>21.30566636649676</v>
       </c>
       <c r="J147" s="2" t="n">
         <v>0.3281214053564047</v>
@@ -8255,7 +8255,7 @@
         <v>-1</v>
       </c>
       <c r="N147" s="2" t="n">
-        <v>-0.1513563445537133</v>
+        <v>-0.1513563438531188</v>
       </c>
       <c r="O147" s="2" t="inlineStr">
         <is>
@@ -8290,7 +8290,7 @@
         <v>0</v>
       </c>
       <c r="H148" s="2" t="n">
-        <v>35.1818458222961</v>
+        <v>35.18184587003479</v>
       </c>
       <c r="I148" s="2" t="n">
         <v>21.13206810474157</v>
@@ -8308,7 +8308,7 @@
         <v>-1</v>
       </c>
       <c r="N148" s="2" t="n">
-        <v>0.1057536531351583</v>
+        <v>0.1057536530939443</v>
       </c>
       <c r="O148" s="2" t="inlineStr">
         <is>
@@ -8343,10 +8343,10 @@
         <v>0</v>
       </c>
       <c r="H149" s="2" t="n">
-        <v>40.13266332095092</v>
+        <v>40.13266335534574</v>
       </c>
       <c r="I149" s="2" t="n">
-        <v>27.89340669835518</v>
+        <v>27.89340673215142</v>
       </c>
       <c r="J149" s="2" t="n">
         <v>0.4548197657062259</v>
@@ -8361,7 +8361,7 @@
         <v>-1</v>
       </c>
       <c r="N149" s="2" t="n">
-        <v>0.6159358295930382</v>
+        <v>0.6159358295724284</v>
       </c>
       <c r="O149" s="2" t="inlineStr">
         <is>
@@ -8382,7 +8382,7 @@
         <v/>
       </c>
       <c r="D150" s="2" t="n">
-        <v>308.6245679653881</v>
+        <v>308.624567965388</v>
       </c>
       <c r="E150" s="2" t="n">
         <v>73.40000000000001</v>
@@ -8396,10 +8396,10 @@
         <v>0</v>
       </c>
       <c r="H150" s="2" t="n">
-        <v>41.90036533673492</v>
+        <v>41.90036571390005</v>
       </c>
       <c r="I150" s="2" t="n">
-        <v>26.85054707362442</v>
+        <v>26.85054725490464</v>
       </c>
       <c r="J150" s="2" t="n">
         <v>0.6290230468080952</v>
@@ -8414,7 +8414,7 @@
         <v>-1</v>
       </c>
       <c r="N150" s="2" t="n">
-        <v>0.3803465288514673</v>
+        <v>0.3803465274090709</v>
       </c>
       <c r="O150" s="2" t="inlineStr">
         <is>
@@ -8435,7 +8435,7 @@
         <v/>
       </c>
       <c r="D151" s="2" t="n">
-        <v>306.2165522716384</v>
+        <v>306.2165522716376</v>
       </c>
       <c r="E151" s="2" t="n">
         <v>17.2</v>
@@ -8449,10 +8449,10 @@
         <v>0</v>
       </c>
       <c r="H151" s="2" t="n">
-        <v>50.81022645033688</v>
+        <v>50.81022648628935</v>
       </c>
       <c r="I151" s="2" t="n">
-        <v>15.271038492247</v>
+        <v>15.27103849565707</v>
       </c>
       <c r="J151" s="2" t="n">
         <v>0.5334259334336893</v>
@@ -8467,7 +8467,7 @@
         <v>-1</v>
       </c>
       <c r="N151" s="2" t="n">
-        <v>0.1090729572407929</v>
+        <v>0.1090729572304917</v>
       </c>
       <c r="O151" s="2" t="inlineStr">
         <is>
@@ -8608,10 +8608,10 @@
         <v>0</v>
       </c>
       <c r="H154" s="2" t="n">
-        <v>54.13840279201916</v>
+        <v>54.13840280505708</v>
       </c>
       <c r="I154" s="2" t="n">
-        <v>17.62324588280387</v>
+        <v>17.62324586682953</v>
       </c>
       <c r="J154" s="2" t="n">
         <v>0.7526873444599393</v>
@@ -8626,7 +8626,7 @@
         <v>-1</v>
       </c>
       <c r="N154" s="2" t="n">
-        <v>0.0710784230261941</v>
+        <v>0.07107842304267969</v>
       </c>
       <c r="O154" s="2" t="inlineStr">
         <is>
@@ -8820,10 +8820,10 @@
         <v>0</v>
       </c>
       <c r="H158" s="2" t="n">
-        <v>53.51838362572512</v>
+        <v>53.51838365770299</v>
       </c>
       <c r="I158" s="2" t="n">
-        <v>15.28346117684702</v>
+        <v>15.2834611855122</v>
       </c>
       <c r="J158" s="2" t="n">
         <v>0.6074349846612459</v>
@@ -8838,7 +8838,7 @@
         <v>-1</v>
       </c>
       <c r="N158" s="2" t="n">
-        <v>0.1775913544251872</v>
+        <v>0.1775913544045831</v>
       </c>
       <c r="O158" s="2" t="inlineStr">
         <is>
@@ -8926,10 +8926,10 @@
         <v>0</v>
       </c>
       <c r="H160" s="2" t="n">
-        <v>41.91523509741097</v>
+        <v>41.91523511002013</v>
       </c>
       <c r="I160" s="2" t="n">
-        <v>8.978740852174358</v>
+        <v>8.978740847096313</v>
       </c>
       <c r="J160" s="2" t="n">
         <v>0.5556673360774486</v>
@@ -8944,7 +8944,7 @@
         <v>-1</v>
       </c>
       <c r="N160" s="2" t="n">
-        <v>0.1971938656331595</v>
+        <v>0.1971938656228598</v>
       </c>
       <c r="O160" s="2" t="inlineStr">
         <is>
@@ -8979,10 +8979,10 @@
         <v>0</v>
       </c>
       <c r="H161" s="2" t="n">
-        <v>44.49172067611673</v>
+        <v>44.49172081302632</v>
       </c>
       <c r="I161" s="2" t="n">
-        <v>24.84009638825352</v>
+        <v>24.84009642778226</v>
       </c>
       <c r="J161" s="2" t="n">
         <v>0.4681225797999144</v>
@@ -8997,7 +8997,7 @@
         <v>-1</v>
       </c>
       <c r="N161" s="2" t="n">
-        <v>2.170828989597755</v>
+        <v>2.170828988258444</v>
       </c>
       <c r="O161" s="2" t="inlineStr">
         <is>
@@ -9191,10 +9191,10 @@
         <v>0</v>
       </c>
       <c r="H165" s="2" t="n">
-        <v>43.20564695749677</v>
+        <v>43.20564701922287</v>
       </c>
       <c r="I165" s="2" t="n">
-        <v>22.5453901806132</v>
+        <v>22.54539022370206</v>
       </c>
       <c r="J165" s="2" t="n">
         <v>0.1943630593282188</v>
@@ -9209,7 +9209,7 @@
         <v>-1</v>
       </c>
       <c r="N165" s="2" t="n">
-        <v>0.0204334616576649</v>
+        <v>0.0204334616267549</v>
       </c>
       <c r="O165" s="2" t="inlineStr">
         <is>
@@ -9283,7 +9283,7 @@
         <v/>
       </c>
       <c r="D167" s="2" t="n">
-        <v>274.6376983986449</v>
+        <v>274.637698398645</v>
       </c>
       <c r="E167" s="2" t="n">
         <v>37.95</v>
@@ -9297,10 +9297,10 @@
         <v>0</v>
       </c>
       <c r="H167" s="2" t="n">
-        <v>43.23009622402483</v>
+        <v>43.23009625529529</v>
       </c>
       <c r="I167" s="2" t="n">
-        <v>15.76232076362064</v>
+        <v>15.76232088414027</v>
       </c>
       <c r="J167" s="2" t="n">
         <v>0.7109783951440176</v>
@@ -9315,7 +9315,7 @@
         <v>-1</v>
       </c>
       <c r="N167" s="2" t="n">
-        <v>0.018293542590536</v>
+        <v>0.0182935425699303</v>
       </c>
       <c r="O167" s="2" t="inlineStr">
         <is>
@@ -9350,10 +9350,10 @@
         <v>0</v>
       </c>
       <c r="H168" s="2" t="n">
-        <v>47.48501946645725</v>
+        <v>47.48501946061283</v>
       </c>
       <c r="I168" s="2" t="n">
-        <v>22.11711750314617</v>
+        <v>22.11711753953133</v>
       </c>
       <c r="J168" s="2" t="n">
         <v>0.4816641291088135</v>
@@ -9368,7 +9368,7 @@
         <v>-1</v>
       </c>
       <c r="N168" s="2" t="n">
-        <v>0.1722172713828971</v>
+        <v>0.1722172714241077</v>
       </c>
       <c r="O168" s="2" t="inlineStr">
         <is>
@@ -9442,7 +9442,7 @@
         <v/>
       </c>
       <c r="D170" s="2" t="n">
-        <v>268.6634765066525</v>
+        <v>268.6634765066526</v>
       </c>
       <c r="E170" s="2" t="n">
         <v>28.85</v>
@@ -9456,10 +9456,10 @@
         <v>0</v>
       </c>
       <c r="H170" s="2" t="n">
-        <v>46.15786799958428</v>
+        <v>46.15786796166086</v>
       </c>
       <c r="I170" s="2" t="n">
-        <v>14.41653921340601</v>
+        <v>14.41653899545132</v>
       </c>
       <c r="J170" s="2" t="n">
         <v>1.56409781885161</v>
@@ -9474,7 +9474,7 @@
         <v>-1</v>
       </c>
       <c r="N170" s="2" t="n">
-        <v>-0.0601819063162045</v>
+        <v>-0.0601819063986266</v>
       </c>
       <c r="O170" s="2" t="inlineStr">
         <is>
@@ -9512,7 +9512,7 @@
         <v>44.86463029433289</v>
       </c>
       <c r="I171" s="2" t="n">
-        <v>14.97519179425167</v>
+        <v>14.97519183239302</v>
       </c>
       <c r="J171" s="2" t="n">
         <v>0.6205225341530777</v>
@@ -9562,10 +9562,10 @@
         <v>0</v>
       </c>
       <c r="H172" s="2" t="n">
-        <v>44.85232543802774</v>
+        <v>44.85232544049845</v>
       </c>
       <c r="I172" s="2" t="n">
-        <v>9.017612817406247</v>
+        <v>9.017612618339223</v>
       </c>
       <c r="J172" s="2" t="n">
         <v>0.5066696452871983</v>
@@ -9580,7 +9580,7 @@
         <v>-1</v>
       </c>
       <c r="N172" s="2" t="n">
-        <v>-1.113140869668616</v>
+        <v>-1.113140869689222</v>
       </c>
       <c r="O172" s="2" t="inlineStr">
         <is>
@@ -9668,10 +9668,10 @@
         <v>0</v>
       </c>
       <c r="H174" s="2" t="n">
-        <v>35.3271284279768</v>
+        <v>35.32712851484118</v>
       </c>
       <c r="I174" s="2" t="n">
-        <v>26.43196683347772</v>
+        <v>26.43196683729027</v>
       </c>
       <c r="J174" s="2" t="n">
         <v>0.4590776792621344</v>
@@ -9686,7 +9686,7 @@
         <v>-1</v>
       </c>
       <c r="N174" s="2" t="n">
-        <v>-0.1480067099448716</v>
+        <v>-0.1480067099860851</v>
       </c>
       <c r="O174" s="2" t="inlineStr">
         <is>
@@ -9760,7 +9760,7 @@
         <v/>
       </c>
       <c r="D176" s="2" t="n">
-        <v>262.1921772983613</v>
+        <v>262.1921772983612</v>
       </c>
       <c r="E176" s="2" t="n">
         <v>18.85</v>
@@ -9774,10 +9774,10 @@
         <v>0</v>
       </c>
       <c r="H176" s="2" t="n">
-        <v>49.37260801041465</v>
+        <v>49.37260807910715</v>
       </c>
       <c r="I176" s="2" t="n">
-        <v>27.09237087477331</v>
+        <v>27.09237094026302</v>
       </c>
       <c r="J176" s="2" t="n">
         <v>0.2578301485020183</v>
@@ -9792,7 +9792,7 @@
         <v>-1</v>
       </c>
       <c r="N176" s="2" t="n">
-        <v>0.1077854099981878</v>
+        <v>0.1077854100084901</v>
       </c>
       <c r="O176" s="2" t="inlineStr">
         <is>
@@ -9880,10 +9880,10 @@
         <v>0</v>
       </c>
       <c r="H178" s="2" t="n">
-        <v>45.94636000989786</v>
+        <v>45.94635992343058</v>
       </c>
       <c r="I178" s="2" t="n">
-        <v>6.185344691750891</v>
+        <v>6.1853445096596</v>
       </c>
       <c r="J178" s="2" t="n">
         <v>2.259878935577577</v>
@@ -9898,7 +9898,7 @@
         <v>-1</v>
       </c>
       <c r="N178" s="2" t="n">
-        <v>-0.1107225683984555</v>
+        <v>-0.1107225684499647</v>
       </c>
       <c r="O178" s="2" t="inlineStr">
         <is>
@@ -9933,10 +9933,10 @@
         <v>0</v>
       </c>
       <c r="H179" s="2" t="n">
-        <v>48.88873733415579</v>
+        <v>48.88873728690079</v>
       </c>
       <c r="I179" s="2" t="n">
-        <v>22.09072760588004</v>
+        <v>22.09072751224576</v>
       </c>
       <c r="J179" s="2" t="n">
         <v>0.8764615542565138</v>
@@ -9951,7 +9951,7 @@
         <v>-1</v>
       </c>
       <c r="N179" s="2" t="n">
-        <v>-0.0295287097701717</v>
+        <v>-0.0295287097289581</v>
       </c>
       <c r="O179" s="2" t="inlineStr">
         <is>
@@ -9986,10 +9986,10 @@
         <v>0</v>
       </c>
       <c r="H180" s="2" t="n">
-        <v>45.31743808099211</v>
+        <v>45.31743799988511</v>
       </c>
       <c r="I180" s="2" t="n">
-        <v>23.07309444079258</v>
+        <v>23.07309443353122</v>
       </c>
       <c r="J180" s="2" t="n">
         <v>0.3764681828305214</v>
@@ -10004,7 +10004,7 @@
         <v>-1</v>
       </c>
       <c r="N180" s="2" t="n">
-        <v>0.0837241802564878</v>
+        <v>0.0837241803080075</v>
       </c>
       <c r="O180" s="2" t="inlineStr">
         <is>
@@ -10095,7 +10095,7 @@
         <v>47.92328170685263</v>
       </c>
       <c r="I182" s="2" t="n">
-        <v>8.366549493812458</v>
+        <v>8.366549532310094</v>
       </c>
       <c r="J182" s="2" t="n">
         <v>0.6556075649590389</v>
@@ -10110,7 +10110,7 @@
         <v>-1</v>
       </c>
       <c r="N182" s="2" t="n">
-        <v>-1.401566005266196</v>
+        <v>-1.401566005369199</v>
       </c>
       <c r="O182" s="2" t="inlineStr">
         <is>
@@ -10198,10 +10198,10 @@
         <v>0</v>
       </c>
       <c r="H184" s="2" t="n">
-        <v>32.83036119618393</v>
+        <v>32.83036102433954</v>
       </c>
       <c r="I184" s="2" t="n">
-        <v>27.16153917818483</v>
+        <v>27.16153934248857</v>
       </c>
       <c r="J184" s="2" t="n">
         <v>0.6616704717568114</v>
@@ -10216,7 +10216,7 @@
         <v>-1</v>
       </c>
       <c r="N184" s="2" t="n">
-        <v>-0.0323062109936387</v>
+        <v>-0.0323062105815257</v>
       </c>
       <c r="O184" s="2" t="inlineStr">
         <is>
@@ -10237,7 +10237,7 @@
         <v/>
       </c>
       <c r="D185" s="2" t="n">
-        <v>243.7701097166696</v>
+        <v>243.7701097166695</v>
       </c>
       <c r="E185" s="2" t="n">
         <v>23.5</v>
@@ -10251,10 +10251,10 @@
         <v>0</v>
       </c>
       <c r="H185" s="2" t="n">
-        <v>40.49576253253403</v>
+        <v>40.49576314616158</v>
       </c>
       <c r="I185" s="2" t="n">
-        <v>12.55738295124505</v>
+        <v>12.55738297376676</v>
       </c>
       <c r="J185" s="2" t="n">
         <v>0.9295942804790364</v>
@@ -10269,7 +10269,7 @@
         <v>-1</v>
       </c>
       <c r="N185" s="2" t="n">
-        <v>0.0010613441643649</v>
+        <v>0.0010613443498179</v>
       </c>
       <c r="O185" s="2" t="inlineStr">
         <is>
@@ -10463,10 +10463,10 @@
         <v>0</v>
       </c>
       <c r="H189" s="2" t="n">
-        <v>41.10051326212356</v>
+        <v>41.10051329336616</v>
       </c>
       <c r="I189" s="2" t="n">
-        <v>20.78257963403994</v>
+        <v>20.7825795512342</v>
       </c>
       <c r="J189" s="2" t="n">
         <v>0.166833289795846</v>
@@ -10481,7 +10481,7 @@
         <v>-1</v>
       </c>
       <c r="N189" s="2" t="n">
-        <v>0.0234764349605718</v>
+        <v>0.0234764351006903</v>
       </c>
       <c r="O189" s="2" t="inlineStr">
         <is>
@@ -10569,10 +10569,10 @@
         <v>0</v>
       </c>
       <c r="H191" s="2" t="n">
-        <v>45.99081792819845</v>
+        <v>45.99081749386461</v>
       </c>
       <c r="I191" s="2" t="n">
-        <v>12.81316959337054</v>
+        <v>12.81316966643857</v>
       </c>
       <c r="J191" s="2" t="n">
         <v>0.6983862696223849</v>
@@ -10587,7 +10587,7 @@
         <v>-1</v>
       </c>
       <c r="N191" s="2" t="n">
-        <v>0.7104996416205132</v>
+        <v>0.7104996440932041</v>
       </c>
       <c r="O191" s="2" t="inlineStr">
         <is>
@@ -10625,7 +10625,7 @@
         <v>51.57613043637703</v>
       </c>
       <c r="I192" s="2" t="n">
-        <v>5.403615127968136</v>
+        <v>5.403615100931309</v>
       </c>
       <c r="J192" s="2" t="n">
         <v>1.426256844495429</v>
@@ -10640,7 +10640,7 @@
         <v>-1</v>
       </c>
       <c r="N192" s="2" t="n">
-        <v>-0.09228495282742399</v>
+        <v>-0.09228495283772679</v>
       </c>
       <c r="O192" s="2" t="inlineStr">
         <is>
@@ -10993,10 +10993,10 @@
         <v>0</v>
       </c>
       <c r="H199" s="2" t="n">
-        <v>44.73568552066919</v>
+        <v>44.73568551699211</v>
       </c>
       <c r="I199" s="2" t="n">
-        <v>10.57163902391792</v>
+        <v>10.5716391139303</v>
       </c>
       <c r="J199" s="2" t="n">
         <v>0.6735475843633582</v>
@@ -11011,7 +11011,7 @@
         <v>-1</v>
       </c>
       <c r="N199" s="2" t="n">
-        <v>0.1403709463790188</v>
+        <v>0.1403709463893205</v>
       </c>
       <c r="O199" s="2" t="inlineStr">
         <is>
@@ -11099,10 +11099,10 @@
         <v>0</v>
       </c>
       <c r="H201" s="2" t="n">
-        <v>51.30382951280489</v>
+        <v>51.30382940906799</v>
       </c>
       <c r="I201" s="2" t="n">
-        <v>13.39901384771431</v>
+        <v>13.39901383099268</v>
       </c>
       <c r="J201" s="2" t="n">
         <v>2.408414771351022</v>
@@ -11117,7 +11117,7 @@
         <v>-1</v>
       </c>
       <c r="N201" s="2" t="n">
-        <v>0.0743053857892178</v>
+        <v>0.07430538585103449</v>
       </c>
       <c r="O201" s="2" t="inlineStr">
         <is>
@@ -11138,7 +11138,7 @@
         <v/>
       </c>
       <c r="D202" s="2" t="n">
-        <v>212.027389601334</v>
+        <v>212.0273896013339</v>
       </c>
       <c r="E202" s="2" t="n">
         <v>39.45</v>
@@ -11155,7 +11155,7 @@
         <v>46.02314864527166</v>
       </c>
       <c r="I202" s="2" t="n">
-        <v>8.148483668587355</v>
+        <v>8.148483680469683</v>
       </c>
       <c r="J202" s="2" t="n">
         <v>0.3683164154452263</v>
@@ -11170,7 +11170,7 @@
         <v>-1</v>
       </c>
       <c r="N202" s="2" t="n">
-        <v>0.0202360681737636</v>
+        <v>0.0202360682973981</v>
       </c>
       <c r="O202" s="2" t="inlineStr">
         <is>
@@ -11191,7 +11191,7 @@
         <v/>
       </c>
       <c r="D203" s="2" t="n">
-        <v>209.673416321169</v>
+        <v>209.6734163211624</v>
       </c>
       <c r="E203" s="2" t="n">
         <v>50.1</v>
@@ -11205,10 +11205,10 @@
         <v>0</v>
       </c>
       <c r="H203" s="2" t="n">
-        <v>44.49347795764776</v>
+        <v>44.49347792802456</v>
       </c>
       <c r="I203" s="2" t="n">
-        <v>13.27297460164622</v>
+        <v>13.27297459595983</v>
       </c>
       <c r="J203" s="2" t="n">
         <v>0.3235307004148744</v>
@@ -11223,7 +11223,7 @@
         <v>-1</v>
       </c>
       <c r="N203" s="2" t="n">
-        <v>-0.2630507003054484</v>
+        <v>-0.2630507003569595</v>
       </c>
       <c r="O203" s="2" t="inlineStr">
         <is>
@@ -11470,10 +11470,10 @@
         <v>0</v>
       </c>
       <c r="H208" s="2" t="n">
-        <v>33.81006031015482</v>
+        <v>33.81006028863537</v>
       </c>
       <c r="I208" s="2" t="n">
-        <v>28.7528731462949</v>
+        <v>28.75287316975542</v>
       </c>
       <c r="J208" s="2" t="n">
         <v>0.3483637896855789</v>
@@ -11488,7 +11488,7 @@
         <v>-1</v>
       </c>
       <c r="N208" s="2" t="n">
-        <v>0.1357178134291341</v>
+        <v>0.1357178134085277</v>
       </c>
       <c r="O208" s="2" t="inlineStr">
         <is>
@@ -11682,10 +11682,10 @@
         <v>0</v>
       </c>
       <c r="H212" s="2" t="n">
-        <v>44.33429217649953</v>
+        <v>44.3342919644781</v>
       </c>
       <c r="I212" s="2" t="n">
-        <v>13.37645202960286</v>
+        <v>13.37645196452319</v>
       </c>
       <c r="J212" s="2" t="n">
         <v>0.3533149221793441</v>
@@ -11700,7 +11700,7 @@
         <v>-1</v>
       </c>
       <c r="N212" s="2" t="n">
-        <v>0.0717462523650613</v>
+        <v>0.0717462524722107</v>
       </c>
       <c r="O212" s="2" t="inlineStr">
         <is>
@@ -11721,7 +11721,7 @@
         <v/>
       </c>
       <c r="D213" s="2" t="n">
-        <v>190.2696826443415</v>
+        <v>190.2696826443416</v>
       </c>
       <c r="E213" s="2" t="n">
         <v>23.85</v>
@@ -11735,10 +11735,10 @@
         <v>0</v>
       </c>
       <c r="H213" s="2" t="n">
-        <v>32.47341758663477</v>
+        <v>32.47341757123189</v>
       </c>
       <c r="I213" s="2" t="n">
-        <v>41.4144716319393</v>
+        <v>41.41447171499399</v>
       </c>
       <c r="J213" s="2" t="n">
         <v>0.5608709432649793</v>
@@ -11753,7 +11753,7 @@
         <v>-1</v>
       </c>
       <c r="N213" s="2" t="n">
-        <v>-0.1156564094377401</v>
+        <v>-0.1156564093553165</v>
       </c>
       <c r="O213" s="2" t="inlineStr">
         <is>
@@ -11947,10 +11947,10 @@
         <v>0</v>
       </c>
       <c r="H217" s="2" t="n">
-        <v>14.03263476699561</v>
+        <v>14.03263476767056</v>
       </c>
       <c r="I217" s="2" t="n">
-        <v>11.55213201120356</v>
+        <v>11.5521320352254</v>
       </c>
       <c r="J217" s="2" t="n">
         <v>0.0001033340738941</v>
@@ -11965,7 +11965,7 @@
         <v>-1</v>
       </c>
       <c r="N217" s="2" t="n">
-        <v>-1.331809858866918</v>
+        <v>-1.331809858887526</v>
       </c>
       <c r="O217" s="2" t="inlineStr">
         <is>
@@ -12000,10 +12000,10 @@
         <v>0</v>
       </c>
       <c r="H218" s="2" t="n">
-        <v>46.57945951746101</v>
+        <v>46.57945935525485</v>
       </c>
       <c r="I218" s="2" t="n">
-        <v>22.64096206598294</v>
+        <v>22.64096213143648</v>
       </c>
       <c r="J218" s="2" t="n">
         <v>0.6352566297552983</v>
@@ -12018,7 +12018,7 @@
         <v>-1</v>
       </c>
       <c r="N218" s="2" t="n">
-        <v>0.3988504549530156</v>
+        <v>0.398850455200282</v>
       </c>
       <c r="O218" s="2" t="inlineStr">
         <is>
@@ -12106,10 +12106,10 @@
         <v>0</v>
       </c>
       <c r="H220" s="2" t="n">
-        <v>36.28119457681836</v>
+        <v>36.28119488538385</v>
       </c>
       <c r="I220" s="2" t="n">
-        <v>26.73821218942108</v>
+        <v>26.73821221688288</v>
       </c>
       <c r="J220" s="2" t="n">
         <v>0.2728386372437038</v>
@@ -12124,7 +12124,7 @@
         <v>-1</v>
       </c>
       <c r="N220" s="2" t="n">
-        <v>0.012021443979556</v>
+        <v>0.0120214439486453</v>
       </c>
       <c r="O220" s="2" t="inlineStr">
         <is>
@@ -12318,10 +12318,10 @@
         <v>0</v>
       </c>
       <c r="H224" s="2" t="n">
-        <v>42.05975173924313</v>
+        <v>42.05975172705464</v>
       </c>
       <c r="I224" s="2" t="n">
-        <v>12.43183919145812</v>
+        <v>12.43183920830346</v>
       </c>
       <c r="J224" s="2" t="n">
         <v>0.2621223965725815</v>
@@ -12336,7 +12336,7 @@
         <v>-1</v>
       </c>
       <c r="N224" s="2" t="n">
-        <v>-0.0442062475999228</v>
+        <v>-0.0442062475587131</v>
       </c>
       <c r="O224" s="2" t="inlineStr">
         <is>
@@ -12424,10 +12424,10 @@
         <v>0</v>
       </c>
       <c r="H226" s="2" t="n">
-        <v>43.10064890702567</v>
+        <v>43.10064873514557</v>
       </c>
       <c r="I226" s="2" t="n">
-        <v>9.640384928557165</v>
+        <v>9.640384965874944</v>
       </c>
       <c r="J226" s="2" t="n">
         <v>0.27527310306977</v>
@@ -12442,7 +12442,7 @@
         <v>-1</v>
       </c>
       <c r="N226" s="2" t="n">
-        <v>0.0262598745202042</v>
+        <v>0.0262598746850515</v>
       </c>
       <c r="O226" s="2" t="inlineStr">
         <is>
@@ -12463,7 +12463,7 @@
         <v/>
       </c>
       <c r="D227" s="2" t="n">
-        <v>135.8884050881668</v>
+        <v>135.8884050881667</v>
       </c>
       <c r="E227" s="2" t="n">
         <v>90</v>
@@ -12477,7 +12477,7 @@
         <v>0</v>
       </c>
       <c r="H227" s="2" t="n">
-        <v>40.72529993588686</v>
+        <v>40.72529984493859</v>
       </c>
       <c r="I227" s="2" t="n">
         <v>19.54495682826579</v>
@@ -12495,7 +12495,7 @@
         <v>-1</v>
       </c>
       <c r="N227" s="2" t="n">
-        <v>-0.2713259276443998</v>
+        <v>-0.2713259274383348</v>
       </c>
       <c r="O227" s="2" t="inlineStr">
         <is>
@@ -12639,7 +12639,7 @@
         <v>36.02263457370197</v>
       </c>
       <c r="I230" s="2" t="n">
-        <v>14.89105107188655</v>
+        <v>14.89105108001897</v>
       </c>
       <c r="J230" s="2" t="n">
         <v>0.2094990021225618</v>
@@ -12654,7 +12654,7 @@
         <v>-1</v>
       </c>
       <c r="N230" s="2" t="n">
-        <v>0.0108507391456483</v>
+        <v>0.0108507391250421</v>
       </c>
       <c r="O230" s="2" t="inlineStr">
         <is>
@@ -12675,7 +12675,7 @@
         <v/>
       </c>
       <c r="D231" s="2" t="n">
-        <v>125.3321013761241</v>
+        <v>125.3321013761243</v>
       </c>
       <c r="E231" s="2" t="n">
         <v>61.7</v>
@@ -12689,10 +12689,10 @@
         <v>0</v>
       </c>
       <c r="H231" s="2" t="n">
-        <v>43.41890544046306</v>
+        <v>43.4189054175521</v>
       </c>
       <c r="I231" s="2" t="n">
-        <v>16.39227180720466</v>
+        <v>16.39227202841185</v>
       </c>
       <c r="J231" s="2" t="n">
         <v>0.3933832535536709</v>
@@ -12707,7 +12707,7 @@
         <v>-1</v>
       </c>
       <c r="N231" s="2" t="n">
-        <v>0.1629262728460297</v>
+        <v>0.1629262730314779</v>
       </c>
       <c r="O231" s="2" t="inlineStr">
         <is>
@@ -12834,7 +12834,7 @@
         <v/>
       </c>
       <c r="D234" s="2" t="n">
-        <v>90.60044220284048</v>
+        <v>90.60044220283956</v>
       </c>
       <c r="E234" s="2" t="n">
         <v>23.25</v>
@@ -12848,10 +12848,10 @@
         <v>0</v>
       </c>
       <c r="H234" s="2" t="n">
-        <v>42.38523066474614</v>
+        <v>42.38523108184168</v>
       </c>
       <c r="I234" s="2" t="n">
-        <v>14.81990147390572</v>
+        <v>14.81990168765324</v>
       </c>
       <c r="J234" s="2" t="n">
         <v>0.4465814656574527</v>
@@ -12866,7 +12866,7 @@
         <v>-1</v>
       </c>
       <c r="N234" s="2" t="n">
-        <v>-0.0246458246176702</v>
+        <v>-0.024645824928308</v>
       </c>
       <c r="O234" s="2" t="inlineStr">
         <is>
@@ -12993,7 +12993,7 @@
         <v/>
       </c>
       <c r="D237" s="2" t="n">
-        <v>78.11529850297265</v>
+        <v>78.11529850297259</v>
       </c>
       <c r="E237" s="2" t="n">
         <v>82.5</v>
@@ -13007,10 +13007,10 @@
         <v>0</v>
       </c>
       <c r="H237" s="2" t="n">
-        <v>46.74576163274421</v>
+        <v>46.74576170981788</v>
       </c>
       <c r="I237" s="2" t="n">
-        <v>11.26892833406143</v>
+        <v>11.2689283138482</v>
       </c>
       <c r="J237" s="2" t="n">
         <v>0.7810850283452343</v>
@@ -13025,7 +13025,7 @@
         <v>-1</v>
       </c>
       <c r="N237" s="2" t="n">
-        <v>0.2994196065256638</v>
+        <v>0.2994196063402188</v>
       </c>
       <c r="O237" s="2" t="inlineStr">
         <is>
@@ -13046,7 +13046,7 @@
         <v/>
       </c>
       <c r="D238" s="2" t="n">
-        <v>72.11443353152545</v>
+        <v>72.11443353152501</v>
       </c>
       <c r="E238" s="2" t="n">
         <v>34.35</v>
@@ -13060,10 +13060,10 @@
         <v>0</v>
       </c>
       <c r="H238" s="2" t="n">
-        <v>39.20207154762437</v>
+        <v>39.20207102550129</v>
       </c>
       <c r="I238" s="2" t="n">
-        <v>19.82230170135819</v>
+        <v>19.82230216112758</v>
       </c>
       <c r="J238" s="2" t="n">
         <v>0.2293162367733994</v>
@@ -13078,7 +13078,7 @@
         <v>-1</v>
       </c>
       <c r="N238" s="2" t="n">
-        <v>0.0485330031300224</v>
+        <v>0.0485330040572808</v>
       </c>
       <c r="O238" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
scan: seg4 2026-09-28 18:04 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq5_2026-09-24.xlsx
+++ b/output/full_scan/batch_seq5_2026-09-24.xlsx
@@ -658,10 +658,10 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>68.81035902333016</v>
+        <v>68.8103590193341</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>12.73687841764105</v>
+        <v>12.73687842839478</v>
       </c>
       <c r="J4" s="2" t="n">
         <v>6.479544065060112</v>
@@ -676,7 +676,7 @@
         <v>-1</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>0.9960066264025988</v>
+        <v>0.9960066267529016</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
@@ -792,21 +792,21 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>4770</v>
+        <v>5230</v>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>上品</t>
+          <t>雷笛克光學</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
         <v/>
       </c>
       <c r="D7" s="2" t="n">
-        <v>932.2605833459944</v>
+        <v>922.5452166384324</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>281.5</v>
+        <v>23.3</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
@@ -817,49 +817,49 @@
         <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>71.77572352993795</v>
+        <v>82.33098303731487</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>32.04757420387939</v>
+        <v>34.16945289366775</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>3.826058334599439</v>
+        <v>2.85452166384325</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L7" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M7" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>5.013370794555861</v>
+        <v>0.4972411723838936</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, breakout_volume_confirm, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, volume_break, rsi_strong, breakout_20d, market_above_ma60, adx_trending, stronger_than_market, obv_uptrend, breakout_volume_confirm, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>5230</v>
+        <v>4770</v>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>雷笛克光學</t>
+          <t>上品</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
         <v/>
       </c>
       <c r="D8" s="2" t="n">
-        <v>922.5452166384324</v>
+        <v>872.2605833459944</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>23.3</v>
+        <v>281.5</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
@@ -870,29 +870,29 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>82.33098303731487</v>
+        <v>71.77572336390294</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>34.16945289366775</v>
+        <v>32.04757419309107</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>2.85452166384325</v>
+        <v>3.826058334599439</v>
       </c>
       <c r="K8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="L8" s="2" t="n">
-        <v>0</v>
-      </c>
       <c r="M8" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>0.4972411723838936</v>
+        <v>5.013370799810367</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, rsi_strong, breakout_20d, market_above_ma60, adx_trending, stronger_than_market, obv_uptrend, breakout_volume_confirm, mfi_strong, above_ichimoku_cloud</t>
+          <t>volume_break, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, breakout_volume_confirm, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
@@ -1241,10 +1241,10 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>62.25575136218347</v>
+        <v>62.25575124382432</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>39.64747602894467</v>
+        <v>39.64747619749159</v>
       </c>
       <c r="J15" s="2" t="n">
         <v>0.3437488000058795</v>
@@ -1259,7 +1259,7 @@
         <v>-1</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>-0.0103754105487001</v>
+        <v>-0.0103754103838538</v>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
@@ -1492,7 +1492,7 @@
         <v/>
       </c>
       <c r="D20" s="2" t="n">
-        <v>762.9578359188235</v>
+        <v>762.9578359188234</v>
       </c>
       <c r="E20" s="2" t="n">
         <v>14.4</v>
@@ -1506,10 +1506,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>57.90946925768867</v>
+        <v>57.90946926686114</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>20.85976556234633</v>
+        <v>20.85976566882331</v>
       </c>
       <c r="J20" s="2" t="n">
         <v>2.618020138616451</v>
@@ -1524,7 +1524,7 @@
         <v>-1</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>0.0806836185966833</v>
+        <v>0.08068361862759239</v>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
@@ -1559,10 +1559,10 @@
         <v>0</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>61.02121080777088</v>
+        <v>61.02120237972896</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>29.84671089453922</v>
+        <v>29.84670461985296</v>
       </c>
       <c r="J21" s="2" t="n">
         <v>1.767059278639126</v>
@@ -1577,7 +1577,7 @@
         <v>-1</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>0.0113587181559157</v>
+        <v>0.0113587210922419</v>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
@@ -1930,10 +1930,10 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>54.6924297492144</v>
+        <v>54.69242967056417</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>29.11161250777786</v>
+        <v>29.11161255222388</v>
       </c>
       <c r="J28" s="2" t="n">
         <v>0.5849274908302399</v>
@@ -1948,7 +1948,7 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>0.0568726371169409</v>
+        <v>0.0568726374775424</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
@@ -2036,10 +2036,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>59.90121715096843</v>
+        <v>59.90121715626299</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>28.881675981026</v>
+        <v>28.88167600580463</v>
       </c>
       <c r="J30" s="2" t="n">
         <v>0.3278584951746066</v>
@@ -2054,7 +2054,7 @@
         <v>-1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>1.871470356788881</v>
+        <v>1.871470356644656</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
@@ -2128,7 +2128,7 @@
         <v/>
       </c>
       <c r="D32" s="2" t="n">
-        <v>674.858081363328</v>
+        <v>674.8580813633281</v>
       </c>
       <c r="E32" s="2" t="n">
         <v>225</v>
@@ -2142,10 +2142,10 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>48.71103069234053</v>
+        <v>48.71103067923735</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>20.00882355644496</v>
+        <v>20.00882354979169</v>
       </c>
       <c r="J32" s="2" t="n">
         <v>0.2560333412723786</v>
@@ -2160,7 +2160,7 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>-2.033759712485915</v>
+        <v>-2.033759711970776</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
@@ -2251,7 +2251,7 @@
         <v>62.16432837317918</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>19.62741977985568</v>
+        <v>19.62741980182255</v>
       </c>
       <c r="J34" s="2" t="n">
         <v>1.541918131860579</v>
@@ -2266,7 +2266,7 @@
         <v>-1</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>-0.1145444814164639</v>
+        <v>-0.1145444813752565</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
@@ -2301,7 +2301,7 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>55.60400285124288</v>
+        <v>55.60400286893166</v>
       </c>
       <c r="I35" s="2" t="n">
         <v>36.55019272855143</v>
@@ -2672,10 +2672,10 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>49.46790685615793</v>
+        <v>49.46790683397014</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>41.51741410640639</v>
+        <v>41.5174142345079</v>
       </c>
       <c r="J42" s="2" t="n">
         <v>0.6974006104383712</v>
@@ -2690,7 +2690,7 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>-0.0777381052861708</v>
+        <v>-0.0777381052346577</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
@@ -2764,7 +2764,7 @@
         <v/>
       </c>
       <c r="D44" s="2" t="n">
-        <v>598.2299759138505</v>
+        <v>598.2299759138506</v>
       </c>
       <c r="E44" s="2" t="n">
         <v>212</v>
@@ -2778,10 +2778,10 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>53.29595625236897</v>
+        <v>53.29595615924087</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>20.28415106042165</v>
+        <v>20.28415105549253</v>
       </c>
       <c r="J44" s="2" t="n">
         <v>0.5381882763402255</v>
@@ -2796,7 +2796,7 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>0.3206892979974283</v>
+        <v>0.3206892985125789</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
@@ -3414,10 +3414,10 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>52.09329616100742</v>
+        <v>52.09329597354725</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>31.353295028226</v>
+        <v>31.35329504572269</v>
       </c>
       <c r="J56" s="2" t="n">
         <v>0.6987920384932089</v>
@@ -3432,7 +3432,7 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>-0.1160734882695108</v>
+        <v>-0.1160734871980122</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
@@ -3453,7 +3453,7 @@
         <v/>
       </c>
       <c r="D57" s="2" t="n">
-        <v>549.2786236044436</v>
+        <v>549.2786236044437</v>
       </c>
       <c r="E57" s="2" t="n">
         <v>343.5</v>
@@ -3467,10 +3467,10 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>53.31637305601383</v>
+        <v>53.31637293137671</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>10.85050409600881</v>
+        <v>10.85050413189508</v>
       </c>
       <c r="J57" s="2" t="n">
         <v>0.5676270190493309</v>
@@ -3485,7 +3485,7 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>0.0610160808808112</v>
+        <v>0.0610160822201687</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
@@ -3785,10 +3785,10 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>45.69705808265042</v>
+        <v>45.69705813874491</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>22.0068992142726</v>
+        <v>22.00689920484161</v>
       </c>
       <c r="J63" s="2" t="n">
         <v>1.611857819242779</v>
@@ -3803,7 +3803,7 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>0.1081445649211649</v>
+        <v>0.1081445649314659</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
@@ -3944,10 +3944,10 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>46.26723549184492</v>
+        <v>46.26723554553796</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>17.36164429409034</v>
+        <v>17.36164432349543</v>
       </c>
       <c r="J66" s="2" t="n">
         <v>0.4550434989940676</v>
@@ -3962,7 +3962,7 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>-0.2974107543535805</v>
+        <v>-0.2974107544153953</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
@@ -4103,10 +4103,10 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>64.0391531291524</v>
+        <v>64.03915317304212</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>24.56988951403187</v>
+        <v>24.56988949834657</v>
       </c>
       <c r="J69" s="2" t="n">
         <v>0.8539018775809273</v>
@@ -4262,10 +4262,10 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>51.15748839583868</v>
+        <v>51.15748830007258</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>22.47658364165237</v>
+        <v>22.47658374657749</v>
       </c>
       <c r="J72" s="2" t="n">
         <v>0.322345670775057</v>
@@ -4280,7 +4280,7 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>-0.0294860576120866</v>
+        <v>-0.0294860571381571</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
@@ -4421,10 +4421,10 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>58.47076365709396</v>
+        <v>58.47076384662746</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>20.80775742474945</v>
+        <v>20.80775750843143</v>
       </c>
       <c r="J75" s="2" t="n">
         <v>0.5340344449746914</v>
@@ -4439,7 +4439,7 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>0.0488235968493397</v>
+        <v>0.0488235968390339</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
         <v/>
       </c>
       <c r="D76" s="2" t="n">
-        <v>484.4073872998474</v>
+        <v>484.4073872998455</v>
       </c>
       <c r="E76" s="2" t="n">
         <v>184</v>
@@ -4474,10 +4474,10 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>39.39066430309327</v>
+        <v>39.39066430015361</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>22.16140032556028</v>
+        <v>22.16140028808008</v>
       </c>
       <c r="J76" s="2" t="n">
         <v>0.9857091137268152</v>
@@ -4492,7 +4492,7 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>0.3570944329173606</v>
+        <v>0.3570944329585641</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
@@ -4527,10 +4527,10 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>33.58239287847695</v>
+        <v>33.58239341310666</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>20.69928986808966</v>
+        <v>20.69929204132883</v>
       </c>
       <c r="J77" s="2" t="n">
         <v>1.163180969647383</v>
@@ -4545,7 +4545,7 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>-1.917727767653598</v>
+        <v>-1.91772777600926</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
@@ -4739,10 +4739,10 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>56.38742636564721</v>
+        <v>56.38742608247564</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>16.66945247917815</v>
+        <v>16.66945241409192</v>
       </c>
       <c r="J81" s="2" t="n">
         <v>0.5628232816407717</v>
@@ -4757,7 +4757,7 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>0.0558172353993436</v>
+        <v>0.0558172358320655</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
@@ -4792,10 +4792,10 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>55.74857831255809</v>
+        <v>55.74857822940203</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>27.27099603144418</v>
+        <v>27.27099603194092</v>
       </c>
       <c r="J82" s="2" t="n">
         <v>0.5205154316030123</v>
@@ -4810,7 +4810,7 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>0.2567259754232558</v>
+        <v>0.2567259758044622</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
@@ -4845,7 +4845,7 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>49.10782016714725</v>
+        <v>49.10782020953558</v>
       </c>
       <c r="I83" s="2" t="n">
         <v>19.27507845469787</v>
@@ -4863,7 +4863,7 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>0.3093416667446095</v>
+        <v>0.3093416668476508</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
@@ -4898,10 +4898,10 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>48.43153034516915</v>
+        <v>48.43153022096617</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>11.14616932445286</v>
+        <v>11.14616957238591</v>
       </c>
       <c r="J84" s="2" t="n">
         <v>0.1621140391137049</v>
@@ -4916,7 +4916,7 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>0.004335008761779</v>
+        <v>0.0043350088338979</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
@@ -4990,7 +4990,7 @@
         <v/>
       </c>
       <c r="D86" s="2" t="n">
-        <v>456.4896247062656</v>
+        <v>456.4896247062657</v>
       </c>
       <c r="E86" s="2" t="n">
         <v>31.75</v>
@@ -5004,10 +5004,10 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>53.49049835994364</v>
+        <v>53.49049845865163</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>17.71646470836197</v>
+        <v>17.71646470836198</v>
       </c>
       <c r="J86" s="2" t="n">
         <v>0.2831828438973704</v>
@@ -5022,7 +5022,7 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>0.1230489110270717</v>
+        <v>0.1230489108931337</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
@@ -5163,10 +5163,10 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>46.25650474090093</v>
+        <v>46.25650475782972</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>24.21747499731798</v>
+        <v>24.21747501111855</v>
       </c>
       <c r="J89" s="2" t="n">
         <v>0.3851726453046433</v>
@@ -5520,7 +5520,7 @@
         <v/>
       </c>
       <c r="D96" s="2" t="n">
-        <v>434.9205764127134</v>
+        <v>434.920576412714</v>
       </c>
       <c r="E96" s="2" t="n">
         <v>32</v>
@@ -5534,10 +5534,10 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>50.13890692747822</v>
+        <v>50.13890691514087</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>13.72758210319665</v>
+        <v>13.72758207588924</v>
       </c>
       <c r="J96" s="2" t="n">
         <v>0.9215231654956528</v>
@@ -5552,7 +5552,7 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>0.1341400420394524</v>
+        <v>0.1341400420909687</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
@@ -5587,10 +5587,10 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>36.96293594032589</v>
+        <v>36.96293586602814</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>12.69260824695648</v>
+        <v>12.69260824695647</v>
       </c>
       <c r="J97" s="2" t="n">
         <v>0.688833328680561</v>
@@ -5605,7 +5605,7 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>-0.5553395643820627</v>
+        <v>-0.5553395641759957</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
@@ -5908,7 +5908,7 @@
         <v>49.94527225999974</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>10.94208471153626</v>
+        <v>10.94208472570935</v>
       </c>
       <c r="J103" s="2" t="n">
         <v>0.941309601978234</v>
@@ -5923,7 +5923,7 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>0.4404509179898528</v>
+        <v>0.440450918505002</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
@@ -6382,10 +6382,10 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>52.32291639244881</v>
+        <v>52.32291637534784</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>24.27558905999737</v>
+        <v>24.27558909387223</v>
       </c>
       <c r="J112" s="2" t="n">
         <v>0.343876719416974</v>
@@ -6400,7 +6400,7 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>0.1537580470644267</v>
+        <v>0.153758047095335</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
@@ -6859,10 +6859,10 @@
         <v>0</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>47.23850738202734</v>
+        <v>47.23850741795591</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>18.72845506973326</v>
+        <v>18.72845507205989</v>
       </c>
       <c r="J121" s="2" t="n">
         <v>0.6903758132354407</v>
@@ -6877,7 +6877,7 @@
         <v>-1</v>
       </c>
       <c r="N121" s="2" t="n">
-        <v>0.4435926937202776</v>
+        <v>0.4435926938232778</v>
       </c>
       <c r="O121" s="2" t="inlineStr">
         <is>
@@ -7389,10 +7389,10 @@
         <v>0</v>
       </c>
       <c r="H131" s="2" t="n">
-        <v>42.90911986313471</v>
+        <v>42.90912001657082</v>
       </c>
       <c r="I131" s="2" t="n">
-        <v>16.80064891298318</v>
+        <v>16.80064890355461</v>
       </c>
       <c r="J131" s="2" t="n">
         <v>0.3209158335419296</v>
@@ -7407,7 +7407,7 @@
         <v>-1</v>
       </c>
       <c r="N131" s="2" t="n">
-        <v>-0.6210357604224761</v>
+        <v>-0.6210357608345181</v>
       </c>
       <c r="O131" s="2" t="inlineStr">
         <is>
@@ -7428,7 +7428,7 @@
         <v/>
       </c>
       <c r="D132" s="2" t="n">
-        <v>340.0532727323797</v>
+        <v>340.0532727323796</v>
       </c>
       <c r="E132" s="2" t="n">
         <v>46.1</v>
@@ -7442,10 +7442,10 @@
         <v>0</v>
       </c>
       <c r="H132" s="2" t="n">
-        <v>43.60107828614754</v>
+        <v>43.60107833080873</v>
       </c>
       <c r="I132" s="2" t="n">
-        <v>15.01210524815607</v>
+        <v>15.01210528152589</v>
       </c>
       <c r="J132" s="2" t="n">
         <v>0.7708092727017104</v>
@@ -7460,7 +7460,7 @@
         <v>-1</v>
       </c>
       <c r="N132" s="2" t="n">
-        <v>-0.2255998326656032</v>
+        <v>-0.2255998329746933</v>
       </c>
       <c r="O132" s="2" t="inlineStr">
         <is>
@@ -7481,7 +7481,7 @@
         <v/>
       </c>
       <c r="D133" s="2" t="n">
-        <v>339.592970191393</v>
+        <v>339.5929701913932</v>
       </c>
       <c r="E133" s="2" t="n">
         <v>16</v>
@@ -7495,10 +7495,10 @@
         <v>0</v>
       </c>
       <c r="H133" s="2" t="n">
-        <v>58.0661766162033</v>
+        <v>58.06617656499727</v>
       </c>
       <c r="I133" s="2" t="n">
-        <v>16.7990329044096</v>
+        <v>16.79903290908473</v>
       </c>
       <c r="J133" s="2" t="n">
         <v>6.609273966177796</v>
@@ -7513,7 +7513,7 @@
         <v>-1</v>
       </c>
       <c r="N133" s="2" t="n">
-        <v>0.154787307537849</v>
+        <v>0.1547873076099683</v>
       </c>
       <c r="O133" s="2" t="inlineStr">
         <is>
@@ -7746,7 +7746,7 @@
         <v/>
       </c>
       <c r="D138" s="2" t="n">
-        <v>329.4071298218722</v>
+        <v>329.4071298218726</v>
       </c>
       <c r="E138" s="2" t="n">
         <v>13.9</v>
@@ -7760,10 +7760,10 @@
         <v>0</v>
       </c>
       <c r="H138" s="2" t="n">
-        <v>45.96245656113359</v>
+        <v>45.96245648437187</v>
       </c>
       <c r="I138" s="2" t="n">
-        <v>22.22967874732579</v>
+        <v>22.22967895731598</v>
       </c>
       <c r="J138" s="2" t="n">
         <v>1.020011786286407</v>
@@ -7778,7 +7778,7 @@
         <v>-1</v>
       </c>
       <c r="N138" s="2" t="n">
-        <v>0.0136237558775179</v>
+        <v>0.0136237558878201</v>
       </c>
       <c r="O138" s="2" t="inlineStr">
         <is>
@@ -7866,10 +7866,10 @@
         <v>0</v>
       </c>
       <c r="H140" s="2" t="n">
-        <v>46.95076014018072</v>
+        <v>46.95076007575143</v>
       </c>
       <c r="I140" s="2" t="n">
-        <v>14.81113798317256</v>
+        <v>14.81113782022021</v>
       </c>
       <c r="J140" s="2" t="n">
         <v>1.445877026728663</v>
@@ -7884,7 +7884,7 @@
         <v>-1</v>
       </c>
       <c r="N140" s="2" t="n">
-        <v>0.0309726826107651</v>
+        <v>0.0309726826416733</v>
       </c>
       <c r="O140" s="2" t="inlineStr">
         <is>
@@ -7905,7 +7905,7 @@
         <v/>
       </c>
       <c r="D141" s="2" t="n">
-        <v>322.8108976928878</v>
+        <v>322.8108976928877</v>
       </c>
       <c r="E141" s="2" t="n">
         <v>48.05</v>
@@ -7919,10 +7919,10 @@
         <v>0</v>
       </c>
       <c r="H141" s="2" t="n">
-        <v>48.98822470495254</v>
+        <v>48.98822482580609</v>
       </c>
       <c r="I141" s="2" t="n">
-        <v>19.6466225514238</v>
+        <v>19.64662270171388</v>
       </c>
       <c r="J141" s="2" t="n">
         <v>0.9098321204909148</v>
@@ -7937,7 +7937,7 @@
         <v>-1</v>
       </c>
       <c r="N141" s="2" t="n">
-        <v>0.4509772721822083</v>
+        <v>0.4509772725325056</v>
       </c>
       <c r="O141" s="2" t="inlineStr">
         <is>
@@ -7972,10 +7972,10 @@
         <v>0</v>
       </c>
       <c r="H142" s="2" t="n">
-        <v>54.52397640275105</v>
+        <v>54.52397642815816</v>
       </c>
       <c r="I142" s="2" t="n">
-        <v>25.78690803195751</v>
+        <v>25.78690796842927</v>
       </c>
       <c r="J142" s="2" t="n">
         <v>0.5544223985408935</v>
@@ -7990,7 +7990,7 @@
         <v>-1</v>
       </c>
       <c r="N142" s="2" t="n">
-        <v>0.2224088641812379</v>
+        <v>0.2224088645696987</v>
       </c>
       <c r="O142" s="2" t="inlineStr">
         <is>
@@ -8078,10 +8078,10 @@
         <v>0</v>
       </c>
       <c r="H144" s="2" t="n">
-        <v>51.42497257286751</v>
+        <v>51.42497256475853</v>
       </c>
       <c r="I144" s="2" t="n">
-        <v>9.150813316481772</v>
+        <v>9.150813209458414</v>
       </c>
       <c r="J144" s="2" t="n">
         <v>0.1764119572024591</v>
@@ -8096,7 +8096,7 @@
         <v>-1</v>
       </c>
       <c r="N144" s="2" t="n">
-        <v>0.900717598198603</v>
+        <v>0.9007175982604247</v>
       </c>
       <c r="O144" s="2" t="inlineStr">
         <is>
@@ -8131,10 +8131,10 @@
         <v>0</v>
       </c>
       <c r="H145" s="2" t="n">
-        <v>48.84779228111741</v>
+        <v>48.84779226299291</v>
       </c>
       <c r="I145" s="2" t="n">
-        <v>11.9064529118204</v>
+        <v>11.90645289884771</v>
       </c>
       <c r="J145" s="2" t="n">
         <v>0.9797262151725996</v>
@@ -8149,7 +8149,7 @@
         <v>-1</v>
       </c>
       <c r="N145" s="2" t="n">
-        <v>0.4121621665572621</v>
+        <v>0.4121621665984782</v>
       </c>
       <c r="O145" s="2" t="inlineStr">
         <is>
@@ -8488,7 +8488,7 @@
         <v/>
       </c>
       <c r="D152" s="2" t="n">
-        <v>305.9693742650847</v>
+        <v>305.9693742650848</v>
       </c>
       <c r="E152" s="2" t="n">
         <v>57</v>
@@ -8502,10 +8502,10 @@
         <v>0</v>
       </c>
       <c r="H152" s="2" t="n">
-        <v>42.44876136033536</v>
+        <v>42.44876134777043</v>
       </c>
       <c r="I152" s="2" t="n">
-        <v>22.72527630608824</v>
+        <v>22.72527637262008</v>
       </c>
       <c r="J152" s="2" t="n">
         <v>0.486597216991344</v>
@@ -8520,7 +8520,7 @@
         <v>-1</v>
       </c>
       <c r="N152" s="2" t="n">
-        <v>0.0105711744277642</v>
+        <v>0.0105711746544221</v>
       </c>
       <c r="O152" s="2" t="inlineStr">
         <is>
@@ -8555,10 +8555,10 @@
         <v>0</v>
       </c>
       <c r="H153" s="2" t="n">
-        <v>47.25069519294235</v>
+        <v>47.2506951276548</v>
       </c>
       <c r="I153" s="2" t="n">
-        <v>23.5062348453432</v>
+        <v>23.50623481752676</v>
       </c>
       <c r="J153" s="2" t="n">
         <v>0.9534628746549014</v>
@@ -8661,10 +8661,10 @@
         <v>0</v>
       </c>
       <c r="H155" s="2" t="n">
-        <v>48.93469070577177</v>
+        <v>48.93469071500669</v>
       </c>
       <c r="I155" s="2" t="n">
-        <v>16.58839380905311</v>
+        <v>16.5883938256746</v>
       </c>
       <c r="J155" s="2" t="n">
         <v>0.514887230475541</v>
@@ -8679,7 +8679,7 @@
         <v>-1</v>
       </c>
       <c r="N155" s="2" t="n">
-        <v>1.381254263084448</v>
+        <v>1.381254262878405</v>
       </c>
       <c r="O155" s="2" t="inlineStr">
         <is>
@@ -8714,7 +8714,7 @@
         <v>0</v>
       </c>
       <c r="H156" s="2" t="n">
-        <v>43.60734499475668</v>
+        <v>43.60734509613496</v>
       </c>
       <c r="I156" s="2" t="n">
         <v>20.37808563245102</v>
@@ -8732,7 +8732,7 @@
         <v>-1</v>
       </c>
       <c r="N156" s="2" t="n">
-        <v>-0.170963622285146</v>
+        <v>-0.1709636222748444</v>
       </c>
       <c r="O156" s="2" t="inlineStr">
         <is>
@@ -8767,10 +8767,10 @@
         <v>0</v>
       </c>
       <c r="H157" s="2" t="n">
-        <v>43.25912830508739</v>
+        <v>43.25912861190307</v>
       </c>
       <c r="I157" s="2" t="n">
-        <v>6.037876707501242</v>
+        <v>6.037877090897888</v>
       </c>
       <c r="J157" s="2" t="n">
         <v>0</v>
@@ -8785,7 +8785,7 @@
         <v>-1</v>
       </c>
       <c r="N157" s="2" t="n">
-        <v>-1.142128409476045</v>
+        <v>-1.142128419748036</v>
       </c>
       <c r="O157" s="2" t="inlineStr">
         <is>
@@ -8876,7 +8876,7 @@
         <v>54.12482351152418</v>
       </c>
       <c r="I159" s="2" t="n">
-        <v>15.48237274097931</v>
+        <v>15.48237278294358</v>
       </c>
       <c r="J159" s="2" t="n">
         <v>0.332006493111763</v>
@@ -9032,10 +9032,10 @@
         <v>0</v>
       </c>
       <c r="H162" s="2" t="n">
-        <v>43.93351408240427</v>
+        <v>43.93351467826615</v>
       </c>
       <c r="I162" s="2" t="n">
-        <v>28.64462406918584</v>
+        <v>28.64462439139245</v>
       </c>
       <c r="J162" s="2" t="n">
         <v>0.4449259531982389</v>
@@ -9050,7 +9050,7 @@
         <v>-1</v>
       </c>
       <c r="N162" s="2" t="n">
-        <v>-0.0178037739084835</v>
+        <v>-0.017803774032117</v>
       </c>
       <c r="O162" s="2" t="inlineStr">
         <is>
@@ -9085,10 +9085,10 @@
         <v>0</v>
       </c>
       <c r="H163" s="2" t="n">
-        <v>39.14733451439775</v>
+        <v>39.14733454291106</v>
       </c>
       <c r="I163" s="2" t="n">
-        <v>26.49209977612338</v>
+        <v>26.49209976947338</v>
       </c>
       <c r="J163" s="2" t="n">
         <v>0.2611405474991881</v>
@@ -9103,7 +9103,7 @@
         <v>-1</v>
       </c>
       <c r="N163" s="2" t="n">
-        <v>-0.3070688827650355</v>
+        <v>-0.3070688828886745</v>
       </c>
       <c r="O163" s="2" t="inlineStr">
         <is>
@@ -9124,7 +9124,7 @@
         <v/>
       </c>
       <c r="D164" s="2" t="n">
-        <v>282.2001529132012</v>
+        <v>282.2001529132016</v>
       </c>
       <c r="E164" s="2" t="n">
         <v>27.45</v>
@@ -9138,10 +9138,10 @@
         <v>0</v>
       </c>
       <c r="H164" s="2" t="n">
-        <v>53.08475069270737</v>
+        <v>53.08475074088366</v>
       </c>
       <c r="I164" s="2" t="n">
-        <v>5.18080770295569</v>
+        <v>5.180807737624968</v>
       </c>
       <c r="J164" s="2" t="n">
         <v>1.109966894948321</v>
@@ -9156,7 +9156,7 @@
         <v>-1</v>
       </c>
       <c r="N164" s="2" t="n">
-        <v>0.06956769010931151</v>
+        <v>0.0695676900474943</v>
       </c>
       <c r="O164" s="2" t="inlineStr">
         <is>
@@ -9247,7 +9247,7 @@
         <v>44.50176963169979</v>
       </c>
       <c r="I166" s="2" t="n">
-        <v>20.47116174225848</v>
+        <v>20.47116167441988</v>
       </c>
       <c r="J166" s="2" t="n">
         <v>1.530669433392466</v>
@@ -9403,10 +9403,10 @@
         <v>0</v>
       </c>
       <c r="H169" s="2" t="n">
-        <v>46.11593601681371</v>
+        <v>46.11593583033336</v>
       </c>
       <c r="I169" s="2" t="n">
-        <v>9.667543882387269</v>
+        <v>9.667543944253071</v>
       </c>
       <c r="J169" s="2" t="n">
         <v>0.4200221580799085</v>
@@ -9421,7 +9421,7 @@
         <v>-1</v>
       </c>
       <c r="N169" s="2" t="n">
-        <v>0.0593060404524538</v>
+        <v>0.0593060405760843</v>
       </c>
       <c r="O169" s="2" t="inlineStr">
         <is>
@@ -9615,10 +9615,10 @@
         <v>0</v>
       </c>
       <c r="H173" s="2" t="n">
-        <v>50.80143100325621</v>
+        <v>50.80143100963292</v>
       </c>
       <c r="I173" s="2" t="n">
-        <v>11.80607292896948</v>
+        <v>11.80607301807635</v>
       </c>
       <c r="J173" s="2" t="n">
         <v>1.111264795319508</v>
@@ -9633,7 +9633,7 @@
         <v>-1</v>
       </c>
       <c r="N173" s="2" t="n">
-        <v>0.9201758001834928</v>
+        <v>0.92017580275922</v>
       </c>
       <c r="O173" s="2" t="inlineStr">
         <is>
@@ -9707,7 +9707,7 @@
         <v/>
       </c>
       <c r="D175" s="2" t="n">
-        <v>265.0492341646301</v>
+        <v>265.0492341646307</v>
       </c>
       <c r="E175" s="2" t="n">
         <v>49.8</v>
@@ -9721,10 +9721,10 @@
         <v>0</v>
       </c>
       <c r="H175" s="2" t="n">
-        <v>46.08649259479036</v>
+        <v>46.08649273864883</v>
       </c>
       <c r="I175" s="2" t="n">
-        <v>8.185717383722899</v>
+        <v>8.185717296623725</v>
       </c>
       <c r="J175" s="2" t="n">
         <v>0.5676462278746677</v>
@@ -9739,7 +9739,7 @@
         <v>-1</v>
       </c>
       <c r="N175" s="2" t="n">
-        <v>-0.0474868445642639</v>
+        <v>-0.0474868446466825</v>
       </c>
       <c r="O175" s="2" t="inlineStr">
         <is>
@@ -9827,10 +9827,10 @@
         <v>0</v>
       </c>
       <c r="H177" s="2" t="n">
-        <v>45.29301865733093</v>
+        <v>45.29301863214511</v>
       </c>
       <c r="I177" s="2" t="n">
-        <v>11.57049094369907</v>
+        <v>11.57049105796166</v>
       </c>
       <c r="J177" s="2" t="n">
         <v>0.5304997248117724</v>
@@ -9845,7 +9845,7 @@
         <v>-1</v>
       </c>
       <c r="N177" s="2" t="n">
-        <v>0.1355798989250533</v>
+        <v>0.1355798990486855</v>
       </c>
       <c r="O177" s="2" t="inlineStr">
         <is>
@@ -10039,10 +10039,10 @@
         <v>0</v>
       </c>
       <c r="H181" s="2" t="n">
-        <v>36.63539027384758</v>
+        <v>36.6353903016889</v>
       </c>
       <c r="I181" s="2" t="n">
-        <v>28.64600017273147</v>
+        <v>28.64600020432608</v>
       </c>
       <c r="J181" s="2" t="n">
         <v>0.2566308928603555</v>
@@ -10145,10 +10145,10 @@
         <v>0</v>
       </c>
       <c r="H183" s="2" t="n">
-        <v>43.35868592854909</v>
+        <v>43.35868565166364</v>
       </c>
       <c r="I183" s="2" t="n">
-        <v>16.11188419517899</v>
+        <v>16.11188465489843</v>
       </c>
       <c r="J183" s="2" t="n">
         <v>0.6735789684510514</v>
@@ -10163,7 +10163,7 @@
         <v>-1</v>
       </c>
       <c r="N183" s="2" t="n">
-        <v>-0.1270231311073095</v>
+        <v>-0.1270231302212598</v>
       </c>
       <c r="O183" s="2" t="inlineStr">
         <is>
@@ -10304,10 +10304,10 @@
         <v>0</v>
       </c>
       <c r="H186" s="2" t="n">
-        <v>39.72707153363234</v>
+        <v>39.72707148227914</v>
       </c>
       <c r="I186" s="2" t="n">
-        <v>22.35801579933901</v>
+        <v>22.3580159205347</v>
       </c>
       <c r="J186" s="2" t="n">
         <v>1.147983389838965</v>
@@ -10357,10 +10357,10 @@
         <v>0</v>
       </c>
       <c r="H187" s="2" t="n">
-        <v>50.83245379515086</v>
+        <v>50.83245386352154</v>
       </c>
       <c r="I187" s="2" t="n">
-        <v>13.89687189943094</v>
+        <v>13.89687190009988</v>
       </c>
       <c r="J187" s="2" t="n">
         <v>0.4517965427289422</v>
@@ -10375,7 +10375,7 @@
         <v>-1</v>
       </c>
       <c r="N187" s="2" t="n">
-        <v>0.1323834427021717</v>
+        <v>0.1323834427124825</v>
       </c>
       <c r="O187" s="2" t="inlineStr">
         <is>
@@ -10396,7 +10396,7 @@
         <v/>
       </c>
       <c r="D188" s="2" t="n">
-        <v>240.1043172616622</v>
+        <v>240.1043172616621</v>
       </c>
       <c r="E188" s="2" t="n">
         <v>8.210000000000001</v>
@@ -10410,10 +10410,10 @@
         <v>0</v>
       </c>
       <c r="H188" s="2" t="n">
-        <v>45.39714226878964</v>
+        <v>45.39714215910929</v>
       </c>
       <c r="I188" s="2" t="n">
-        <v>10.30273647584461</v>
+        <v>10.30273646784695</v>
       </c>
       <c r="J188" s="2" t="n">
         <v>1.069619291800466</v>
@@ -10502,7 +10502,7 @@
         <v/>
       </c>
       <c r="D190" s="2" t="n">
-        <v>237.5808219382308</v>
+        <v>237.580821938231</v>
       </c>
       <c r="E190" s="2" t="n">
         <v>139.5</v>
@@ -10516,10 +10516,10 @@
         <v>0</v>
       </c>
       <c r="H190" s="2" t="n">
-        <v>43.67335931707998</v>
+        <v>43.67335934719818</v>
       </c>
       <c r="I190" s="2" t="n">
-        <v>11.82524768873736</v>
+        <v>11.82524778691246</v>
       </c>
       <c r="J190" s="2" t="n">
         <v>0.863673806706432</v>
@@ -10534,7 +10534,7 @@
         <v>-1</v>
       </c>
       <c r="N190" s="2" t="n">
-        <v>-0.2118147453323039</v>
+        <v>-0.2118147451262456</v>
       </c>
       <c r="O190" s="2" t="inlineStr">
         <is>
@@ -10661,7 +10661,7 @@
         <v/>
       </c>
       <c r="D193" s="2" t="n">
-        <v>227.2727906401962</v>
+        <v>227.2727906401961</v>
       </c>
       <c r="E193" s="2" t="n">
         <v>16.5</v>
@@ -10675,10 +10675,10 @@
         <v>0</v>
       </c>
       <c r="H193" s="2" t="n">
-        <v>41.03211662333602</v>
+        <v>41.0321172865267</v>
       </c>
       <c r="I193" s="2" t="n">
-        <v>14.29096193881061</v>
+        <v>14.29096195027476</v>
       </c>
       <c r="J193" s="2" t="n">
         <v>0.4540399902863182</v>
@@ -10693,7 +10693,7 @@
         <v>-1</v>
       </c>
       <c r="N193" s="2" t="n">
-        <v>0.0248822422230402</v>
+        <v>0.0248822421509212</v>
       </c>
       <c r="O193" s="2" t="inlineStr">
         <is>
@@ -10728,10 +10728,10 @@
         <v>0</v>
       </c>
       <c r="H194" s="2" t="n">
-        <v>42.98982491358635</v>
+        <v>42.98982495346007</v>
       </c>
       <c r="I194" s="2" t="n">
-        <v>25.4106273721635</v>
+        <v>25.41062740935982</v>
       </c>
       <c r="J194" s="2" t="n">
         <v>0.6742580983440967</v>
@@ -10746,7 +10746,7 @@
         <v>-1</v>
       </c>
       <c r="N194" s="2" t="n">
-        <v>0.3722414713205726</v>
+        <v>0.3722414721448239</v>
       </c>
       <c r="O194" s="2" t="inlineStr">
         <is>
@@ -10767,7 +10767,7 @@
         <v/>
       </c>
       <c r="D195" s="2" t="n">
-        <v>225.6053347572988</v>
+        <v>225.6053347572991</v>
       </c>
       <c r="E195" s="2" t="n">
         <v>47.8</v>
@@ -10781,10 +10781,10 @@
         <v>0</v>
       </c>
       <c r="H195" s="2" t="n">
-        <v>44.58153137089904</v>
+        <v>44.58153138596465</v>
       </c>
       <c r="I195" s="2" t="n">
-        <v>13.59802084246598</v>
+        <v>13.59802084492075</v>
       </c>
       <c r="J195" s="2" t="n">
         <v>0.4776954869481463</v>
@@ -10799,7 +10799,7 @@
         <v>-1</v>
       </c>
       <c r="N195" s="2" t="n">
-        <v>0.238894238364709</v>
+        <v>0.2388942383750041</v>
       </c>
       <c r="O195" s="2" t="inlineStr">
         <is>
@@ -10834,10 +10834,10 @@
         <v>0</v>
       </c>
       <c r="H196" s="2" t="n">
-        <v>29.08697285597884</v>
+        <v>29.08697273583902</v>
       </c>
       <c r="I196" s="2" t="n">
-        <v>37.11217697473745</v>
+        <v>37.11217705213708</v>
       </c>
       <c r="J196" s="2" t="n">
         <v>1.365250432029785</v>
@@ -10852,7 +10852,7 @@
         <v>-1</v>
       </c>
       <c r="N196" s="2" t="n">
-        <v>-0.0132792431416709</v>
+        <v>-0.0132792430695503</v>
       </c>
       <c r="O196" s="2" t="inlineStr">
         <is>
@@ -10887,10 +10887,10 @@
         <v>0</v>
       </c>
       <c r="H197" s="2" t="n">
-        <v>49.71025699316934</v>
+        <v>49.71025689528117</v>
       </c>
       <c r="I197" s="2" t="n">
-        <v>8.589472084514128</v>
+        <v>8.589472111646288</v>
       </c>
       <c r="J197" s="2" t="n">
         <v>0.4613105738754158</v>
@@ -10905,7 +10905,7 @@
         <v>-1</v>
       </c>
       <c r="N197" s="2" t="n">
-        <v>0.3814746973334473</v>
+        <v>0.3814746977455547</v>
       </c>
       <c r="O197" s="2" t="inlineStr">
         <is>
@@ -10926,7 +10926,7 @@
         <v/>
       </c>
       <c r="D198" s="2" t="n">
-        <v>221.8750174789392</v>
+        <v>221.8750174789388</v>
       </c>
       <c r="E198" s="2" t="n">
         <v>41.65</v>
@@ -10940,10 +10940,10 @@
         <v>0</v>
       </c>
       <c r="H198" s="2" t="n">
-        <v>38.00506881005613</v>
+        <v>38.00506853874971</v>
       </c>
       <c r="I198" s="2" t="n">
-        <v>16.33185955715097</v>
+        <v>16.33185966627813</v>
       </c>
       <c r="J198" s="2" t="n">
         <v>0.8426139970972919</v>
@@ -10958,7 +10958,7 @@
         <v>-1</v>
       </c>
       <c r="N198" s="2" t="n">
-        <v>-0.07794737531062031</v>
+        <v>-0.0779473745894185</v>
       </c>
       <c r="O198" s="2" t="inlineStr">
         <is>
@@ -11046,10 +11046,10 @@
         <v>0</v>
       </c>
       <c r="H200" s="2" t="n">
-        <v>42.98035354207439</v>
+        <v>42.98035354845194</v>
       </c>
       <c r="I200" s="2" t="n">
-        <v>11.52490659082862</v>
+        <v>11.52490665508769</v>
       </c>
       <c r="J200" s="2" t="n">
         <v>0.3959101714644029</v>
@@ -11064,7 +11064,7 @@
         <v>-1</v>
       </c>
       <c r="N200" s="2" t="n">
-        <v>-0.0295914079375516</v>
+        <v>-0.029591408040584</v>
       </c>
       <c r="O200" s="2" t="inlineStr">
         <is>
@@ -11244,7 +11244,7 @@
         <v/>
       </c>
       <c r="D204" s="2" t="n">
-        <v>209.3153550017613</v>
+        <v>209.3153550017614</v>
       </c>
       <c r="E204" s="2" t="n">
         <v>14.5</v>
@@ -11258,10 +11258,10 @@
         <v>0</v>
       </c>
       <c r="H204" s="2" t="n">
-        <v>40.70635652953064</v>
+        <v>40.70635663050353</v>
       </c>
       <c r="I204" s="2" t="n">
-        <v>17.56143443508607</v>
+        <v>17.56143439081395</v>
       </c>
       <c r="J204" s="2" t="n">
         <v>0.8147368775389454</v>
@@ -11297,7 +11297,7 @@
         <v/>
       </c>
       <c r="D205" s="2" t="n">
-        <v>208.3553204669721</v>
+        <v>208.355320466972</v>
       </c>
       <c r="E205" s="2" t="n">
         <v>35</v>
@@ -11311,10 +11311,10 @@
         <v>0</v>
       </c>
       <c r="H205" s="2" t="n">
-        <v>46.936056668112</v>
+        <v>46.93605660235291</v>
       </c>
       <c r="I205" s="2" t="n">
-        <v>18.42540105037886</v>
+        <v>18.42540105669678</v>
       </c>
       <c r="J205" s="2" t="n">
         <v>0.7463693518935122</v>
@@ -11329,7 +11329,7 @@
         <v>-1</v>
       </c>
       <c r="N205" s="2" t="n">
-        <v>0.09668930537474379</v>
+        <v>0.09668930545716541</v>
       </c>
       <c r="O205" s="2" t="inlineStr">
         <is>
@@ -11364,10 +11364,10 @@
         <v>0</v>
       </c>
       <c r="H206" s="2" t="n">
-        <v>43.94256847417937</v>
+        <v>43.94256852337695</v>
       </c>
       <c r="I206" s="2" t="n">
-        <v>13.58983687880244</v>
+        <v>13.58983687880243</v>
       </c>
       <c r="J206" s="2" t="n">
         <v>0.3586773918952333</v>
@@ -11382,7 +11382,7 @@
         <v>-1</v>
       </c>
       <c r="N206" s="2" t="n">
-        <v>0.3026009452168217</v>
+        <v>0.3026009451756049</v>
       </c>
       <c r="O206" s="2" t="inlineStr">
         <is>
@@ -11417,10 +11417,10 @@
         <v>0</v>
       </c>
       <c r="H207" s="2" t="n">
-        <v>49.9038423290845</v>
+        <v>49.90384234403876</v>
       </c>
       <c r="I207" s="2" t="n">
-        <v>5.316723294879075</v>
+        <v>5.316723274065076</v>
       </c>
       <c r="J207" s="2" t="n">
         <v>1.280267166791001</v>
@@ -11435,7 +11435,7 @@
         <v>-1</v>
       </c>
       <c r="N207" s="2" t="n">
-        <v>-0.1439664851255673</v>
+        <v>-0.1439664851770781</v>
       </c>
       <c r="O207" s="2" t="inlineStr">
         <is>
@@ -11509,7 +11509,7 @@
         <v/>
       </c>
       <c r="D209" s="2" t="n">
-        <v>198.244456760391</v>
+        <v>198.2444567603908</v>
       </c>
       <c r="E209" s="2" t="n">
         <v>295.5</v>
@@ -11523,10 +11523,10 @@
         <v>0</v>
       </c>
       <c r="H209" s="2" t="n">
-        <v>43.20183262250087</v>
+        <v>43.20183255608121</v>
       </c>
       <c r="I209" s="2" t="n">
-        <v>10.16147321757393</v>
+        <v>10.16147319595598</v>
       </c>
       <c r="J209" s="2" t="n">
         <v>0.912548454331184</v>
@@ -11541,7 +11541,7 @@
         <v>-1</v>
       </c>
       <c r="N209" s="2" t="n">
-        <v>-1.215347097569116</v>
+        <v>-1.215347096126666</v>
       </c>
       <c r="O209" s="2" t="inlineStr">
         <is>
@@ -11576,10 +11576,10 @@
         <v>0</v>
       </c>
       <c r="H210" s="2" t="n">
-        <v>43.25751413791728</v>
+        <v>43.25751416697918</v>
       </c>
       <c r="I210" s="2" t="n">
-        <v>17.0108071892418</v>
+        <v>17.01080720025966</v>
       </c>
       <c r="J210" s="2" t="n">
         <v>0.2182509847570002</v>
@@ -11594,7 +11594,7 @@
         <v>-1</v>
       </c>
       <c r="N210" s="2" t="n">
-        <v>-0.8727172968901957</v>
+        <v>-0.8727172965810697</v>
       </c>
       <c r="O210" s="2" t="inlineStr">
         <is>
@@ -11629,10 +11629,10 @@
         <v>0</v>
       </c>
       <c r="H211" s="2" t="n">
-        <v>34.89787033965214</v>
+        <v>34.89787041540427</v>
       </c>
       <c r="I211" s="2" t="n">
-        <v>26.27540651129111</v>
+        <v>26.27540661362959</v>
       </c>
       <c r="J211" s="2" t="n">
         <v>0.4659778949367941</v>
@@ -11647,7 +11647,7 @@
         <v>-1</v>
       </c>
       <c r="N211" s="2" t="n">
-        <v>0.0474543885837217</v>
+        <v>0.0474543888928016</v>
       </c>
       <c r="O211" s="2" t="inlineStr">
         <is>
@@ -11788,10 +11788,10 @@
         <v>0</v>
       </c>
       <c r="H214" s="2" t="n">
-        <v>33.25420062616261</v>
+        <v>33.25420060763865</v>
       </c>
       <c r="I214" s="2" t="n">
-        <v>41.53569094490986</v>
+        <v>41.53569116067565</v>
       </c>
       <c r="J214" s="2" t="n">
         <v>0.3742701373005618</v>
@@ -11806,7 +11806,7 @@
         <v>-1</v>
       </c>
       <c r="N214" s="2" t="n">
-        <v>0.0505418803977557</v>
+        <v>0.0505418804801787</v>
       </c>
       <c r="O214" s="2" t="inlineStr">
         <is>
@@ -11841,10 +11841,10 @@
         <v>0</v>
       </c>
       <c r="H215" s="2" t="n">
-        <v>35.16156123042909</v>
+        <v>35.16156092809275</v>
       </c>
       <c r="I215" s="2" t="n">
-        <v>18.64751824143272</v>
+        <v>18.64751837017852</v>
       </c>
       <c r="J215" s="2" t="n">
         <v>1.248454553258586</v>
@@ -11859,7 +11859,7 @@
         <v>-1</v>
       </c>
       <c r="N215" s="2" t="n">
-        <v>-0.0567659600420298</v>
+        <v>-0.056765959846274</v>
       </c>
       <c r="O215" s="2" t="inlineStr">
         <is>
@@ -11894,10 +11894,10 @@
         <v>0</v>
       </c>
       <c r="H216" s="2" t="n">
-        <v>44.25183873673489</v>
+        <v>44.25183874306067</v>
       </c>
       <c r="I216" s="2" t="n">
-        <v>12.18525471269858</v>
+        <v>12.18525471554482</v>
       </c>
       <c r="J216" s="2" t="n">
         <v>0.3668515811392365</v>
@@ -11912,7 +11912,7 @@
         <v>-1</v>
       </c>
       <c r="N216" s="2" t="n">
-        <v>-0.0637308148116183</v>
+        <v>-0.0637308147910107</v>
       </c>
       <c r="O216" s="2" t="inlineStr">
         <is>
@@ -12053,10 +12053,10 @@
         <v>0</v>
       </c>
       <c r="H219" s="2" t="n">
-        <v>35.86825336225456</v>
+        <v>35.86825331525951</v>
       </c>
       <c r="I219" s="2" t="n">
-        <v>15.11754320054294</v>
+        <v>15.11754323010767</v>
       </c>
       <c r="J219" s="2" t="n">
         <v>0.5450451063984345</v>
@@ -12071,7 +12071,7 @@
         <v>-1</v>
       </c>
       <c r="N219" s="2" t="n">
-        <v>0.0559012323667916</v>
+        <v>0.0559012324698215</v>
       </c>
       <c r="O219" s="2" t="inlineStr">
         <is>
@@ -12159,10 +12159,10 @@
         <v>0</v>
       </c>
       <c r="H221" s="2" t="n">
-        <v>47.48833833579987</v>
+        <v>47.48833836616231</v>
       </c>
       <c r="I221" s="2" t="n">
-        <v>13.25497075728752</v>
+        <v>13.25497076732725</v>
       </c>
       <c r="J221" s="2" t="n">
         <v>0.5519699318203939</v>
@@ -12212,10 +12212,10 @@
         <v>0</v>
       </c>
       <c r="H222" s="2" t="n">
-        <v>41.03356368285541</v>
+        <v>41.03356354929616</v>
       </c>
       <c r="I222" s="2" t="n">
-        <v>17.14633581660162</v>
+        <v>17.14633585377615</v>
       </c>
       <c r="J222" s="2" t="n">
         <v>0.4349277615441214</v>
@@ -12230,7 +12230,7 @@
         <v>-1</v>
       </c>
       <c r="N222" s="2" t="n">
-        <v>0.06358180602561141</v>
+        <v>0.0635818063347106</v>
       </c>
       <c r="O222" s="2" t="inlineStr">
         <is>
@@ -12265,10 +12265,10 @@
         <v>0</v>
       </c>
       <c r="H223" s="2" t="n">
-        <v>44.44787842621128</v>
+        <v>44.44787829129385</v>
       </c>
       <c r="I223" s="2" t="n">
-        <v>16.35050535929451</v>
+        <v>16.35050563783041</v>
       </c>
       <c r="J223" s="2" t="n">
         <v>0.7105541588731364</v>
@@ -12283,7 +12283,7 @@
         <v>-1</v>
       </c>
       <c r="N223" s="2" t="n">
-        <v>-0.0319985907924613</v>
+        <v>-0.0319985904421611</v>
       </c>
       <c r="O223" s="2" t="inlineStr">
         <is>
@@ -12371,10 +12371,10 @@
         <v>0</v>
       </c>
       <c r="H225" s="2" t="n">
-        <v>45.6938801751085</v>
+        <v>45.69388000959538</v>
       </c>
       <c r="I225" s="2" t="n">
-        <v>8.052207063779052</v>
+        <v>8.052206926004676</v>
       </c>
       <c r="J225" s="2" t="n">
         <v>0.6764847080133984</v>
@@ -12389,7 +12389,7 @@
         <v>-1</v>
       </c>
       <c r="N225" s="2" t="n">
-        <v>1.382483326082328</v>
+        <v>1.382483327998655</v>
       </c>
       <c r="O225" s="2" t="inlineStr">
         <is>
@@ -12530,10 +12530,10 @@
         <v>0</v>
       </c>
       <c r="H228" s="2" t="n">
-        <v>44.7613198805416</v>
+        <v>44.76132004602521</v>
       </c>
       <c r="I228" s="2" t="n">
-        <v>11.97885378818574</v>
+        <v>11.97885374124939</v>
       </c>
       <c r="J228" s="2" t="n">
         <v>1.075970684547014</v>
@@ -12548,7 +12548,7 @@
         <v>-1</v>
       </c>
       <c r="N228" s="2" t="n">
-        <v>-0.0327249696986962</v>
+        <v>-0.0327249697399</v>
       </c>
       <c r="O228" s="2" t="inlineStr">
         <is>
@@ -12583,10 +12583,10 @@
         <v>0</v>
       </c>
       <c r="H229" s="2" t="n">
-        <v>38.17546847164717</v>
+        <v>38.17546850017513</v>
       </c>
       <c r="I229" s="2" t="n">
-        <v>18.6970482301331</v>
+        <v>18.69704844641749</v>
       </c>
       <c r="J229" s="2" t="n">
         <v>0.8073268913844186</v>
@@ -12601,7 +12601,7 @@
         <v>-1</v>
       </c>
       <c r="N229" s="2" t="n">
-        <v>0.0283828822595879</v>
+        <v>0.028382882383226</v>
       </c>
       <c r="O229" s="2" t="inlineStr">
         <is>
@@ -12742,10 +12742,10 @@
         <v>0</v>
       </c>
       <c r="H232" s="2" t="n">
-        <v>39.82664318533468</v>
+        <v>39.82664312793936</v>
       </c>
       <c r="I232" s="2" t="n">
-        <v>12.79464961637038</v>
+        <v>12.7946497329102</v>
       </c>
       <c r="J232" s="2" t="n">
         <v>1.132880432255485</v>
@@ -12760,7 +12760,7 @@
         <v>-1</v>
       </c>
       <c r="N232" s="2" t="n">
-        <v>-0.0362612639782975</v>
+        <v>-0.036261263813454</v>
       </c>
       <c r="O232" s="2" t="inlineStr">
         <is>
@@ -12795,10 +12795,10 @@
         <v>0</v>
       </c>
       <c r="H233" s="2" t="n">
-        <v>45.65549525937406</v>
+        <v>45.65549524869781</v>
       </c>
       <c r="I233" s="2" t="n">
-        <v>10.92818860019256</v>
+        <v>10.92818860426249</v>
       </c>
       <c r="J233" s="2" t="n">
         <v>0.3174744785326019</v>
@@ -12813,7 +12813,7 @@
         <v>-1</v>
       </c>
       <c r="N233" s="2" t="n">
-        <v>-0.003064019692285</v>
+        <v>-0.0030640196943465</v>
       </c>
       <c r="O233" s="2" t="inlineStr">
         <is>
@@ -12887,7 +12887,7 @@
         <v/>
       </c>
       <c r="D235" s="2" t="n">
-        <v>85.50787873335817</v>
+        <v>85.50787873335838</v>
       </c>
       <c r="E235" s="2" t="n">
         <v>152.5</v>
@@ -12901,10 +12901,10 @@
         <v>0</v>
       </c>
       <c r="H235" s="2" t="n">
-        <v>46.27645059366352</v>
+        <v>46.27645058015664</v>
       </c>
       <c r="I235" s="2" t="n">
-        <v>14.70029421995235</v>
+        <v>14.70029423489958</v>
       </c>
       <c r="J235" s="2" t="n">
         <v>0.5316619293856815</v>
@@ -12919,7 +12919,7 @@
         <v>-1</v>
       </c>
       <c r="N235" s="2" t="n">
-        <v>0.3474653261700879</v>
+        <v>0.3474653266852572</v>
       </c>
       <c r="O235" s="2" t="inlineStr">
         <is>
@@ -12940,7 +12940,7 @@
         <v/>
       </c>
       <c r="D236" s="2" t="n">
-        <v>78.16668779222113</v>
+        <v>78.16668779222108</v>
       </c>
       <c r="E236" s="2" t="n">
         <v>6.98</v>
@@ -12954,10 +12954,10 @@
         <v>0</v>
       </c>
       <c r="H236" s="2" t="n">
-        <v>39.04631386231552</v>
+        <v>39.04631366840459</v>
       </c>
       <c r="I236" s="2" t="n">
-        <v>17.64359153731353</v>
+        <v>17.64359221301126</v>
       </c>
       <c r="J236" s="2" t="n">
         <v>0.4797449472608868</v>
@@ -12972,7 +12972,7 @@
         <v>-1</v>
       </c>
       <c r="N236" s="2" t="n">
-        <v>-0.0030418638467705</v>
+        <v>-0.0030418637931954</v>
       </c>
       <c r="O236" s="2" t="inlineStr">
         <is>

</xml_diff>